<commit_message>
Updated Design Parameters - to confirm with Sim
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4963132-573E-4A26-8042-99616575E8D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6A9838-3AA0-4CF2-BCC0-2FC60A914F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="162">
   <si>
     <t>Parameter</t>
   </si>
@@ -496,12 +496,6 @@
     <t>Rload-crit</t>
   </si>
   <si>
-    <t>µH (1-7)</t>
-  </si>
-  <si>
-    <t>Ω (1-6)</t>
-  </si>
-  <si>
     <t>Min L with 20% margin</t>
   </si>
   <si>
@@ -511,21 +505,37 @@
     <t>Min Co with 20% margin</t>
   </si>
   <si>
-    <t>A (1-8)</t>
-  </si>
-  <si>
-    <t>µF (1-9)</t>
+    <t>µF (1-7)</t>
+  </si>
+  <si>
+    <t>Ω</t>
+  </si>
+  <si>
+    <t>µH (1-6)</t>
+  </si>
+  <si>
+    <t>Iin(min) = IL(min)</t>
+  </si>
+  <si>
+    <t>Schottky Diode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSA34-E3/61T </t>
+  </si>
+  <si>
+    <t>0.46V (@3A)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000E+00"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.00000"/>
+    <numFmt numFmtId="168" formatCode="0.0000000"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -1453,7 +1463,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1565,6 +1575,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="58" xfId="2" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="57" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="57" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -1902,25 +1923,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:N108"/>
   <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="20.4375" customWidth="1"/>
     <col min="2" max="11" width="12.8125" customWidth="1"/>
+    <col min="12" max="12" width="17.4375" customWidth="1"/>
+    <col min="13" max="13" width="18.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21">
+    <row r="1" spans="1:3" ht="20.65">
       <c r="A1" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.5">
+    <row r="3" spans="1:3" ht="17.649999999999999">
       <c r="A3" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1"/>
-    <row r="5" spans="1:3" ht="15.5" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1931,7 +1954,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickTop="1">
+    <row r="6" spans="1:3" ht="13.9" thickTop="1">
       <c r="A6" s="38" t="s">
         <v>37</v>
       </c>
@@ -1942,7 +1965,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="14.55">
+    <row r="7" spans="1:3">
       <c r="A7" s="39" t="s">
         <v>38</v>
       </c>
@@ -1953,7 +1976,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="14.55">
+    <row r="8" spans="1:3">
       <c r="A8" s="39" t="s">
         <v>39</v>
       </c>
@@ -1964,7 +1987,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="14.55">
+    <row r="9" spans="1:3">
       <c r="A9" s="39" t="s">
         <v>57</v>
       </c>
@@ -1975,7 +1998,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="14.55">
+    <row r="10" spans="1:3">
       <c r="A10" s="39" t="s">
         <v>58</v>
       </c>
@@ -1986,7 +2009,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1">
+    <row r="11" spans="1:3" ht="13.9" thickBot="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -1997,16 +2020,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.5" thickTop="1">
+    <row r="12" spans="1:3" ht="15.4" thickTop="1">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18.5">
+    <row r="14" spans="1:3" ht="17.649999999999999">
       <c r="A14" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1"/>
-    <row r="16" spans="1:3" ht="15.5" thickTop="1" thickBot="1">
+    <row r="15" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -2017,7 +2040,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1">
+    <row r="17" spans="1:3" ht="13.9" thickTop="1">
       <c r="A17" s="46" t="s">
         <v>42</v>
       </c>
@@ -2029,7 +2052,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="14.55">
+    <row r="18" spans="1:3">
       <c r="A18" s="48" t="s">
         <v>41</v>
       </c>
@@ -2041,7 +2064,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="14.55">
+    <row r="19" spans="1:3">
       <c r="A19" s="57" t="s">
         <v>60</v>
       </c>
@@ -2086,7 +2109,7 @@
         <v>50</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -2098,12 +2121,12 @@
         <v>37.037037037037045</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="96" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B24" s="29">
         <f>B23*1.2</f>
@@ -2155,14 +2178,14 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="98" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B32" s="99">
         <f>B9/B8</f>
         <v>1</v>
       </c>
       <c r="C32" s="36" t="s">
-        <v>157</v>
+        <v>43</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -2174,12 +2197,12 @@
         <v>50</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" s="28" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B34" s="29">
         <f>B33*1.2</f>
@@ -2200,114 +2223,13 @@
         <v>110</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
-      <c r="D36" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="I36" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="K36" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="13.9" thickTop="1">
-      <c r="D37" s="5">
-        <v>5</v>
-      </c>
-      <c r="E37" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="F37" s="54">
-        <v>5</v>
-      </c>
-      <c r="G37" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="H37" s="5">
-        <v>5</v>
-      </c>
-      <c r="I37" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="J37" s="5">
-        <v>5</v>
-      </c>
-      <c r="K37" s="22" t="s">
-        <v>3</v>
-      </c>
-    </row>
+    <row r="36" spans="1:11" ht="13.9" thickTop="1"/>
     <row r="38" spans="1:11" ht="17.649999999999999">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D38" s="42">
-        <v>3.33</v>
-      </c>
-      <c r="E38" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="F38" s="55">
-        <v>3.5</v>
-      </c>
-      <c r="G38" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="H38" s="42">
-        <v>2.5</v>
-      </c>
-      <c r="I38" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="J38" s="42">
-        <v>3.5</v>
-      </c>
-      <c r="K38" s="44" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="13.9" thickBot="1">
-      <c r="D39" s="8">
-        <f>B10</f>
-        <v>0.5</v>
-      </c>
-      <c r="E39" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="F39" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="G39" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="H39" s="8">
-        <v>5</v>
-      </c>
-      <c r="I39" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="J39" s="8">
-        <v>5</v>
-      </c>
-      <c r="K39" s="24" t="s">
-        <v>4</v>
-      </c>
-    </row>
+    </row>
+    <row r="39" spans="1:11" ht="13.9" thickBot="1"/>
     <row r="40" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
       <c r="A40" s="3" t="s">
         <v>0</v>
@@ -2318,21 +2240,29 @@
       <c r="C40" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D40" s="25"/>
-      <c r="E40" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="F40" s="25"/>
-      <c r="G40" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="H40" s="25"/>
-      <c r="I40" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="J40" s="25"/>
-      <c r="K40" s="23" t="s">
-        <v>111</v>
+      <c r="D40" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="13.9" thickTop="1">
@@ -2345,21 +2275,29 @@
       <c r="C41" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="D41" s="25"/>
-      <c r="E41" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="F41" s="25"/>
-      <c r="G41" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="H41" s="25"/>
-      <c r="I41" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="J41" s="25"/>
-      <c r="K41" s="23" t="s">
-        <v>112</v>
+      <c r="D41" s="54">
+        <v>5</v>
+      </c>
+      <c r="E41" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="F41" s="5">
+        <v>5</v>
+      </c>
+      <c r="G41" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="H41" s="5">
+        <v>5</v>
+      </c>
+      <c r="I41" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="J41" s="5">
+        <v>5</v>
+      </c>
+      <c r="K41" s="22" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -2372,21 +2310,29 @@
       <c r="C42" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="D42" s="25"/>
-      <c r="E42" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="F42" s="25"/>
-      <c r="G42" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="H42" s="25"/>
-      <c r="I42" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="J42" s="25"/>
-      <c r="K42" s="23" t="s">
-        <v>113</v>
+      <c r="D42" s="55">
+        <v>3.5</v>
+      </c>
+      <c r="E42" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="F42" s="42">
+        <v>2.5</v>
+      </c>
+      <c r="G42" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="H42" s="42">
+        <v>3.5</v>
+      </c>
+      <c r="I42" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="J42" s="42">
+        <v>3</v>
+      </c>
+      <c r="K42" s="44" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2400,853 +2346,1137 @@
       <c r="C43" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="D43" s="25"/>
+      <c r="D43" s="56">
+        <v>0.5</v>
+      </c>
       <c r="E43" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="F43" s="25"/>
+        <v>4</v>
+      </c>
+      <c r="F43" s="8">
+        <v>5</v>
+      </c>
       <c r="G43" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="H43" s="25"/>
+        <v>4</v>
+      </c>
+      <c r="H43" s="8">
+        <v>5</v>
+      </c>
       <c r="I43" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="J43" s="25"/>
-      <c r="K43" s="23" t="s">
-        <v>114</v>
+        <v>4</v>
+      </c>
+      <c r="J43" s="8">
+        <v>2.75</v>
+      </c>
+      <c r="K43" s="24" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:11">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B44" s="25"/>
+      <c r="B44" s="25">
+        <f>B41^2/B43</f>
+        <v>50</v>
+      </c>
       <c r="C44" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="D44" s="26" t="str">
-        <f>IF(D42&gt;=D43/2,"Yes","No")</f>
-        <v>Yes</v>
-      </c>
-      <c r="E44" s="23"/>
-      <c r="F44" s="26" t="str">
-        <f>IF(F42&gt;=F43/2,"Yes","No")</f>
-        <v>Yes</v>
-      </c>
-      <c r="G44" s="23"/>
-      <c r="H44" s="26" t="str">
-        <f>IF(H42&gt;=H43/2,"Yes","No")</f>
-        <v>Yes</v>
-      </c>
-      <c r="I44" s="23"/>
-      <c r="J44" s="26" t="str">
-        <f>IF(J42&gt;=J43/2,"Yes","No")</f>
-        <v>Yes</v>
-      </c>
-      <c r="K44" s="24"/>
+      <c r="D44" s="25">
+        <f>D41^2/D43</f>
+        <v>50</v>
+      </c>
+      <c r="E44" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="F44" s="25">
+        <f>F41^2/F43</f>
+        <v>5</v>
+      </c>
+      <c r="G44" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="H44" s="25">
+        <f>H41^2/H43</f>
+        <v>5</v>
+      </c>
+      <c r="I44" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="J44" s="25">
+        <f>J41^2/J43</f>
+        <v>9.0909090909090917</v>
+      </c>
+      <c r="K44" s="23" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="45" spans="1:11">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B45" s="25"/>
+      <c r="B45" s="101">
+        <f>1-(B42/B41)</f>
+        <v>0.5</v>
+      </c>
       <c r="C45" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="D45" s="25"/>
+      <c r="D45" s="101">
+        <f>1-(D42/D41)</f>
+        <v>0.30000000000000004</v>
+      </c>
       <c r="E45" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="F45" s="25"/>
+        <v>112</v>
+      </c>
+      <c r="F45" s="101">
+        <f>1-(F42/F41)</f>
+        <v>0.5</v>
+      </c>
       <c r="G45" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="H45" s="25"/>
+        <v>112</v>
+      </c>
+      <c r="H45" s="101">
+        <f>1-(H42/H41)</f>
+        <v>0.30000000000000004</v>
+      </c>
       <c r="I45" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="J45" s="25"/>
+        <v>112</v>
+      </c>
+      <c r="J45" s="101">
+        <f>1-(J42/J41)</f>
+        <v>0.4</v>
+      </c>
       <c r="K45" s="23" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="46" spans="1:11">
       <c r="A46" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="B46" s="25"/>
+      <c r="B46" s="25">
+        <f>B43/B42</f>
+        <v>0.2</v>
+      </c>
       <c r="C46" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="D46" s="25"/>
+      <c r="D46" s="25">
+        <f>D43/D42</f>
+        <v>0.14285714285714285</v>
+      </c>
       <c r="E46" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="F46" s="25"/>
+        <v>113</v>
+      </c>
+      <c r="F46" s="25">
+        <f>F43/F42</f>
+        <v>2</v>
+      </c>
       <c r="G46" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="H46" s="25"/>
+        <v>113</v>
+      </c>
+      <c r="H46" s="25">
+        <f>H43/H42</f>
+        <v>1.4285714285714286</v>
+      </c>
       <c r="I46" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="J46" s="25"/>
+        <v>113</v>
+      </c>
+      <c r="J46" s="25">
+        <f>J43/J42</f>
+        <v>0.91666666666666663</v>
+      </c>
       <c r="K46" s="23" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="47" spans="1:11">
       <c r="A47" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="B47" s="25"/>
+      <c r="B47" s="25">
+        <f>B42*B45/($B$25*10^-6*$B$11*10^3)</f>
+        <v>0.26595744680851069</v>
+      </c>
       <c r="C47" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="D47" s="29"/>
+      <c r="D47" s="25">
+        <f>D42*D45/($B$25*10^-6*$B$11*10^3)</f>
+        <v>0.22340425531914904</v>
+      </c>
       <c r="E47" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="F47" s="29"/>
+        <v>114</v>
+      </c>
+      <c r="F47" s="25">
+        <f>F42*F45/($B$25*10^-6*$B$11*10^3)</f>
+        <v>0.26595744680851069</v>
+      </c>
       <c r="G47" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="H47" s="29"/>
+        <v>114</v>
+      </c>
+      <c r="H47" s="25">
+        <f>H42*H45/($B$25*10^-6*$B$11*10^3)</f>
+        <v>0.22340425531914904</v>
+      </c>
       <c r="I47" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="J47" s="29"/>
+        <v>114</v>
+      </c>
+      <c r="J47" s="25">
+        <f>J42*J45/($B$25*10^-6*$B$11*10^3)</f>
+        <v>0.2553191489361703</v>
+      </c>
       <c r="K47" s="23" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="48" spans="1:11">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B48" s="26" t="str">
+      <c r="B48" s="102" t="str">
         <f>IF(B46&gt;=B47/2,"Yes","No")</f>
         <v>Yes</v>
       </c>
       <c r="C48" s="23"/>
-      <c r="D48" s="29"/>
-      <c r="E48" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="F48" s="29"/>
-      <c r="G48" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="H48" s="29"/>
-      <c r="I48" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="J48" s="29"/>
-      <c r="K48" s="23" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11">
+      <c r="D48" s="26" t="str">
+        <f>IF(D46&gt;=D47/2,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="E48" s="23"/>
+      <c r="F48" s="26" t="str">
+        <f>IF(F46&gt;=F47/2,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="G48" s="23"/>
+      <c r="H48" s="26" t="str">
+        <f>IF(H46&gt;=H47/2,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="I48" s="23"/>
+      <c r="J48" s="26" t="str">
+        <f>IF(J46&gt;=J47/2,"Yes","No")</f>
+        <v>Yes</v>
+      </c>
+      <c r="K48" s="24"/>
+    </row>
+    <row r="49" spans="1:14">
       <c r="A49" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B49" s="25"/>
+      <c r="B49" s="103">
+        <f>B46+(B47/2)</f>
+        <v>0.33297872340425538</v>
+      </c>
       <c r="C49" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="D49" s="29"/>
+      <c r="D49" s="103">
+        <f>D46+(D47/2)</f>
+        <v>0.25455927051671734</v>
+      </c>
       <c r="E49" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="F49" s="103">
+        <f>F46+(F47/2)</f>
+        <v>2.1329787234042552</v>
+      </c>
+      <c r="G49" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="H49" s="103">
+        <f>H46+(H47/2)</f>
+        <v>1.540273556231003</v>
+      </c>
+      <c r="I49" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="J49" s="103">
+        <f>J46+(J47/2)</f>
+        <v>1.0443262411347518</v>
+      </c>
+      <c r="K49" s="23" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14">
+      <c r="A50" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B50" s="103">
+        <f>B46-(B47/2)</f>
+        <v>6.7021276595744667E-2</v>
+      </c>
+      <c r="C50" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D50" s="103">
+        <f>D46-(D47/2)</f>
+        <v>3.1155015197568331E-2</v>
+      </c>
+      <c r="E50" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="F50" s="103">
+        <f>F46-(F47/2)</f>
+        <v>1.8670212765957446</v>
+      </c>
+      <c r="G50" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="H50" s="103">
+        <f>H46-(H47/2)</f>
+        <v>1.3168693009118542</v>
+      </c>
+      <c r="I50" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="J50" s="103">
+        <f>J46-(J47/2)</f>
+        <v>0.78900709219858145</v>
+      </c>
+      <c r="K50" s="23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14">
+      <c r="A51" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B51" s="103">
+        <f>SQRT(B46^2 + (B47^2/12))</f>
+        <v>0.21422989277738178</v>
+      </c>
+      <c r="C51" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="D51" s="103">
+        <f>SQRT(D46^2 + (D47^2/12))</f>
+        <v>0.15673954523305453</v>
+      </c>
+      <c r="E51" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="F51" s="103">
+        <f>SQRT(F46^2 + (F47^2/12))</f>
+        <v>2.0014730692565936</v>
+      </c>
+      <c r="G51" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="H51" s="103">
+        <f>SQRT(H46^2 + (H47^2/12))</f>
+        <v>1.4300263802829551</v>
+      </c>
+      <c r="I51" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="J51" s="103">
+        <f>SQRT(J46^2 + (J47^2/12))</f>
+        <v>0.91962497796415288</v>
+      </c>
+      <c r="K51" s="23" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14">
+      <c r="A52" s="28" t="s">
+        <v>50</v>
+      </c>
+      <c r="B52" s="104">
+        <f>B41/B44</f>
+        <v>0.1</v>
+      </c>
+      <c r="C52" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="D52" s="104">
+        <f>D41/D44</f>
+        <v>0.1</v>
+      </c>
+      <c r="E52" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="F52" s="104">
+        <f>F41/F44</f>
+        <v>1</v>
+      </c>
+      <c r="G52" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="H52" s="104">
+        <f>H41/H44</f>
+        <v>1</v>
+      </c>
+      <c r="I52" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="J52" s="104">
+        <f>J41/J44</f>
+        <v>0.54999999999999993</v>
+      </c>
+      <c r="K52" s="23" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14">
+      <c r="A53" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="104">
+        <f>B51*SQRT(B45)</f>
+        <v>0.15148340991575365</v>
+      </c>
+      <c r="C53" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="D53" s="104">
+        <f>D51*SQRT(D45)</f>
+        <v>8.5849784577245306E-2</v>
+      </c>
+      <c r="E53" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="F53" s="104">
+        <f>F51*SQRT(F45)</f>
+        <v>1.4152551796335899</v>
+      </c>
+      <c r="G53" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="H53" s="104">
+        <f>H51*SQRT(H45)</f>
+        <v>0.7832577063084355</v>
+      </c>
+      <c r="I53" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="J53" s="104">
+        <f>J51*SQRT(J45)</f>
+        <v>0.58162190470977582</v>
+      </c>
+      <c r="K53" s="23" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14">
+      <c r="A54" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="B54" s="104">
+        <f>SQRT(B46^2*B45*(1-B45) + (B47^2/12))</f>
+        <v>0.12607318096807302</v>
+      </c>
+      <c r="C54" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="F49" s="29"/>
-      <c r="G49" s="23" t="s">
+      <c r="D54" s="104">
+        <f>SQRT(D46^2*D45*(1-D45) + (D47^2/12))</f>
+        <v>9.1895789132434749E-2</v>
+      </c>
+      <c r="E54" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="H49" s="29"/>
-      <c r="I49" s="23" t="s">
+      <c r="F54" s="104">
+        <f>SQRT(F46^2*F45*(1-F45) + (F47^2/12))</f>
+        <v>1.0029428931696003</v>
+      </c>
+      <c r="G54" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="J49" s="29"/>
-      <c r="K49" s="23" t="s">
+      <c r="H54" s="104">
+        <f>SQRT(H46^2*H45*(1-H45) + (H47^2/12))</f>
+        <v>0.65782258272727856</v>
+      </c>
+      <c r="I54" s="23" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="50" spans="1:11">
-      <c r="A50" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B50" s="25"/>
-      <c r="C50" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="D50" s="29"/>
-      <c r="E50" s="23" t="s">
+      <c r="J54" s="104">
+        <f>SQRT(J46^2*J45*(1-J45) + (J47^2/12))</f>
+        <v>0.45508129931305408</v>
+      </c>
+      <c r="K54" s="23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14">
+      <c r="A55" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B55" s="29">
+        <f>B41-B56</f>
+        <v>4.54</v>
+      </c>
+      <c r="C55" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="F50" s="29"/>
-      <c r="G50" s="23" t="s">
+      <c r="D55" s="29">
+        <f>D41-D56</f>
+        <v>4.54</v>
+      </c>
+      <c r="E55" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="H50" s="29"/>
-      <c r="I50" s="23" t="s">
+      <c r="F55" s="29">
+        <f>F41-F56</f>
+        <v>4.54</v>
+      </c>
+      <c r="G55" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="J50" s="29"/>
-      <c r="K50" s="23" t="s">
+      <c r="H55" s="29">
+        <f>H41-H56</f>
+        <v>4.54</v>
+      </c>
+      <c r="I55" s="23" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="51" spans="1:11">
-      <c r="A51" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="B51" s="29"/>
-      <c r="C51" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="D51" s="29"/>
-      <c r="E51" s="23" t="s">
+      <c r="J55" s="29">
+        <f>J41-J56</f>
+        <v>4.54</v>
+      </c>
+      <c r="K55" s="23" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14">
+      <c r="A56" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="B56" s="107">
+        <v>0.46</v>
+      </c>
+      <c r="C56" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="F51" s="29"/>
-      <c r="G51" s="23" t="s">
+      <c r="D56" s="107">
+        <v>0.46</v>
+      </c>
+      <c r="E56" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="H51" s="29"/>
-      <c r="I51" s="23" t="s">
+      <c r="F56" s="107">
+        <v>0.46</v>
+      </c>
+      <c r="G56" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="J51" s="29"/>
-      <c r="K51" s="23" t="s">
+      <c r="H56" s="107">
+        <v>0.46</v>
+      </c>
+      <c r="I56" s="23" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="52" spans="1:11" ht="13.9" thickBot="1">
-      <c r="A52" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="B52" s="29"/>
-      <c r="C52" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="D52" s="20"/>
-      <c r="E52" s="31" t="s">
+      <c r="J56" s="107">
+        <v>0.46</v>
+      </c>
+      <c r="K56" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="L56" s="106" t="s">
+        <v>159</v>
+      </c>
+      <c r="M56" t="s">
+        <v>160</v>
+      </c>
+      <c r="N56" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" ht="13.9" thickBot="1">
+      <c r="A57" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B57" s="105">
+        <f>10^3*B52*B45/($B$35*10^-6*$B$11*10^3)</f>
+        <v>7.3529411764705888</v>
+      </c>
+      <c r="C57" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="F52" s="20"/>
-      <c r="G52" s="31" t="s">
+      <c r="D57" s="105">
+        <f>10^3*D52*D45/($B$35*10^-6*$B$11*10^3)</f>
+        <v>4.4117647058823533</v>
+      </c>
+      <c r="E57" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="H52" s="20"/>
-      <c r="I52" s="31" t="s">
+      <c r="F57" s="105">
+        <f>10^3*F52*F45/($B$35*10^-6*$B$11*10^3)</f>
+        <v>73.529411764705884</v>
+      </c>
+      <c r="G57" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="J52" s="20"/>
-      <c r="K52" s="31" t="s">
+      <c r="H57" s="105">
+        <f>10^3*H52*H45/($B$35*10^-6*$B$11*10^3)</f>
+        <v>44.117647058823536</v>
+      </c>
+      <c r="I57" s="31" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="53" spans="1:11" ht="13.9" thickTop="1">
-      <c r="A53" s="28" t="s">
-        <v>51</v>
-      </c>
-      <c r="B53" s="29"/>
-      <c r="C53" s="23" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11">
-      <c r="A54" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B54" s="29"/>
-      <c r="C54" s="23" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11">
-      <c r="A55" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="B55" s="29"/>
-      <c r="C55" s="23" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" ht="13.9" thickBot="1">
-      <c r="A56" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B56" s="20"/>
-      <c r="C56" s="31" t="s">
+      <c r="J57" s="105">
+        <f>10^3*J52*J45/($B$35*10^-6*$B$11*10^3)</f>
+        <v>32.352941176470587</v>
+      </c>
+      <c r="K57" s="31" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
-      <c r="B57" s="33"/>
-      <c r="C57" s="34"/>
-      <c r="D57" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F57" s="3"/>
-      <c r="G57" s="3"/>
-      <c r="H57" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="I57" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J57" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="K57" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" ht="13.9" thickTop="1">
+    <row r="58" spans="1:14" ht="13.9" thickTop="1">
       <c r="B58" s="33"/>
       <c r="C58" s="34"/>
-      <c r="D58" s="8">
-        <f>D40</f>
+    </row>
+    <row r="59" spans="1:14">
+      <c r="B59" s="33"/>
+      <c r="C59" s="34"/>
+    </row>
+    <row r="60" spans="1:14" ht="17.649999999999999">
+      <c r="A60" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" ht="13.9" thickBot="1"/>
+    <row r="62" spans="1:14" ht="14.65" thickTop="1" thickBot="1">
+      <c r="A62" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E58" s="23" t="s">
+      <c r="B62" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J62" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="K62" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" ht="13.9" thickTop="1">
+      <c r="A63" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B63" s="8">
+        <f>B44</f>
+        <v>50</v>
+      </c>
+      <c r="C63" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="F58" s="8">
-        <f>F40</f>
-        <v>0</v>
-      </c>
-      <c r="G58" s="23" t="s">
+      <c r="D63" s="8">
+        <f>D44</f>
+        <v>50</v>
+      </c>
+      <c r="E63" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="H58" s="8">
-        <f>H40</f>
-        <v>0</v>
-      </c>
-      <c r="I58" s="23" t="s">
+      <c r="F63" s="8">
+        <f>F44</f>
+        <v>5</v>
+      </c>
+      <c r="G63" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="J58" s="8">
-        <f>J40</f>
-        <v>0</v>
-      </c>
-      <c r="K58" s="24" t="s">
+      <c r="H63" s="8">
+        <f>H44</f>
+        <v>5</v>
+      </c>
+      <c r="I63" s="23" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" ht="17.649999999999999">
-      <c r="A59" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D59" s="8">
-        <f>D41</f>
-        <v>0</v>
-      </c>
-      <c r="E59" s="23"/>
-      <c r="F59" s="8">
-        <f>F41</f>
-        <v>0</v>
-      </c>
-      <c r="G59" s="23"/>
-      <c r="H59" s="8">
-        <f>H41</f>
-        <v>0</v>
-      </c>
-      <c r="I59" s="23"/>
-      <c r="J59" s="8">
-        <f>J41</f>
-        <v>0</v>
-      </c>
-      <c r="K59" s="24"/>
-    </row>
-    <row r="60" spans="1:11" ht="13.9" thickBot="1">
-      <c r="D60" s="25"/>
-      <c r="E60" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="F60" s="23"/>
-      <c r="G60" s="23"/>
-      <c r="H60" s="25"/>
-      <c r="I60" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="J60" s="25"/>
-      <c r="K60" s="24" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
-      <c r="A61" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D61" s="25"/>
-      <c r="E61" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="F61" s="23"/>
-      <c r="G61" s="23"/>
-      <c r="H61" s="25"/>
-      <c r="I61" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="J61" s="25"/>
-      <c r="K61" s="24" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" ht="13.9" thickTop="1">
-      <c r="A62" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B62" s="8">
-        <f>B44</f>
-        <v>0</v>
-      </c>
-      <c r="C62" s="23" t="s">
+      <c r="J63" s="8">
+        <f>J44</f>
+        <v>9.0909090909090917</v>
+      </c>
+      <c r="K63" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="D62" s="27"/>
-      <c r="E62" s="23"/>
-      <c r="F62" s="23"/>
-      <c r="G62" s="23"/>
-      <c r="H62" s="27"/>
-      <c r="I62" s="23"/>
-      <c r="J62" s="27"/>
-      <c r="K62" s="24"/>
-    </row>
-    <row r="63" spans="1:11">
-      <c r="A63" s="7" t="s">
+    </row>
+    <row r="64" spans="1:14">
+      <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B63" s="8">
+      <c r="B64" s="8">
         <f>B45</f>
-        <v>0</v>
-      </c>
-      <c r="C63" s="23"/>
-      <c r="D63" s="27"/>
-      <c r="E63" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="F63" s="23"/>
-      <c r="G63" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="H63" s="27"/>
-      <c r="I63" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="J63" s="27"/>
-      <c r="K63" s="23" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11">
-      <c r="A64" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B64" s="25"/>
-      <c r="C64" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="D64" s="25"/>
-      <c r="E64" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="F64" s="23"/>
-      <c r="G64" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="H64" s="25"/>
-      <c r="I64" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="J64" s="25"/>
-      <c r="K64" s="23" t="s">
-        <v>21</v>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="C64" s="23"/>
+      <c r="D64" s="8">
+        <f>D45</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="E64" s="23"/>
+      <c r="F64" s="8">
+        <f>F45</f>
+        <v>0.5</v>
+      </c>
+      <c r="G64" s="23"/>
+      <c r="H64" s="8">
+        <f>H45</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="I64" s="23"/>
+      <c r="J64" s="8">
+        <f>J45</f>
+        <v>0.4</v>
+      </c>
+      <c r="K64" s="24"/>
     </row>
     <row r="65" spans="1:11">
       <c r="A65" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B65" s="25"/>
       <c r="C65" s="23" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D65" s="25"/>
       <c r="E65" s="23" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="F65" s="23"/>
-      <c r="G65" s="23" t="s">
-        <v>21</v>
-      </c>
+      <c r="G65" s="23"/>
       <c r="H65" s="25"/>
       <c r="I65" s="23" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="J65" s="25"/>
-      <c r="K65" s="23" t="s">
-        <v>21</v>
+      <c r="K65" s="24" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="66" spans="1:11">
       <c r="A66" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B66" s="25"/>
+      <c r="C66" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="D66" s="25"/>
+      <c r="E66" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="F66" s="23"/>
+      <c r="G66" s="23"/>
+      <c r="H66" s="25"/>
+      <c r="I66" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="J66" s="25"/>
+      <c r="K66" s="24" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11">
+      <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B66" s="27"/>
-      <c r="C66" s="23"/>
-      <c r="D66" s="29"/>
-      <c r="E66" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="F66" s="30"/>
-      <c r="G66" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="H66" s="29"/>
-      <c r="I66" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="J66" s="29"/>
-      <c r="K66" s="23" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11">
-      <c r="A67" s="39" t="s">
+      <c r="B67" s="27"/>
+      <c r="C67" s="23"/>
+      <c r="D67" s="27"/>
+      <c r="E67" s="23"/>
+      <c r="F67" s="23"/>
+      <c r="G67" s="23"/>
+      <c r="H67" s="27"/>
+      <c r="I67" s="23"/>
+      <c r="J67" s="27"/>
+      <c r="K67" s="24"/>
+    </row>
+    <row r="68" spans="1:11">
+      <c r="A68" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="B67" s="27"/>
-      <c r="C67" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D67" s="29"/>
-      <c r="E67" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="F67" s="30"/>
-      <c r="G67" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="H67" s="29"/>
-      <c r="I67" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="J67" s="29"/>
-      <c r="K67" s="23" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11">
-      <c r="A68" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B68" s="25"/>
+      <c r="B68" s="27"/>
       <c r="C68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D68" s="29"/>
+      <c r="D68" s="27"/>
       <c r="E68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F68" s="30"/>
+      <c r="F68" s="23"/>
       <c r="G68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H68" s="29"/>
+      <c r="H68" s="27"/>
       <c r="I68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J68" s="29"/>
+      <c r="J68" s="27"/>
       <c r="K68" s="23" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="69" spans="1:11">
       <c r="A69" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B69" s="25"/>
       <c r="C69" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D69" s="29"/>
+      <c r="D69" s="25"/>
       <c r="E69" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="F69" s="30"/>
+        <v>21</v>
+      </c>
+      <c r="F69" s="23"/>
       <c r="G69" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="H69" s="29"/>
+        <v>21</v>
+      </c>
+      <c r="H69" s="25"/>
       <c r="I69" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="J69" s="29"/>
+        <v>21</v>
+      </c>
+      <c r="J69" s="25"/>
       <c r="K69" s="23" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
     </row>
     <row r="70" spans="1:11">
-      <c r="A70" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="B70" s="29"/>
+      <c r="A70" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B70" s="25"/>
       <c r="C70" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D70" s="29"/>
-      <c r="E70" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="F70" s="30"/>
-      <c r="G70" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="H70" s="29"/>
-      <c r="I70" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="J70" s="29"/>
-      <c r="K70" s="30" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" ht="13.9" thickBot="1">
+      <c r="D70" s="25"/>
+      <c r="E70" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F70" s="23"/>
+      <c r="G70" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="H70" s="25"/>
+      <c r="I70" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="J70" s="25"/>
+      <c r="K70" s="23" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11">
       <c r="A71" s="28" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B71" s="29"/>
       <c r="C71" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D71" s="20"/>
-      <c r="E71" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="F71" s="31"/>
-      <c r="G71" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="H71" s="20"/>
-      <c r="I71" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="J71" s="20"/>
-      <c r="K71" s="31" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" ht="13.9" thickTop="1">
+      <c r="D71" s="29"/>
+      <c r="E71" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F71" s="30"/>
+      <c r="G71" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="H71" s="29"/>
+      <c r="I71" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="J71" s="29"/>
+      <c r="K71" s="23" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11">
       <c r="A72" s="28" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B72" s="29"/>
       <c r="C72" s="23" t="s">
         <v>21</v>
       </c>
+      <c r="D72" s="29"/>
+      <c r="E72" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F72" s="30"/>
+      <c r="G72" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="H72" s="29"/>
+      <c r="I72" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="J72" s="29"/>
+      <c r="K72" s="23" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="73" spans="1:11">
-      <c r="A73" s="7" t="s">
-        <v>53</v>
+      <c r="A73" s="28" t="s">
+        <v>51</v>
       </c>
       <c r="B73" s="29"/>
       <c r="C73" s="23" t="s">
-        <v>3</v>
+        <v>21</v>
+      </c>
+      <c r="D73" s="29"/>
+      <c r="E73" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="F73" s="30"/>
+      <c r="G73" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="H73" s="29"/>
+      <c r="I73" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="J73" s="29"/>
+      <c r="K73" s="23" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="74" spans="1:11">
-      <c r="A74" s="28" t="s">
+      <c r="A74" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B74" s="29"/>
+      <c r="C74" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D74" s="29"/>
+      <c r="E74" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F74" s="30"/>
+      <c r="G74" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="H74" s="29"/>
+      <c r="I74" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="J74" s="29"/>
+      <c r="K74" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11">
+      <c r="A75" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="B74" s="29"/>
-      <c r="C74" s="30" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" ht="13.9" thickBot="1">
-      <c r="A75" s="10" t="s">
+      <c r="B75" s="29"/>
+      <c r="C75" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="D75" s="29"/>
+      <c r="E75" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="F75" s="30"/>
+      <c r="G75" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="H75" s="29"/>
+      <c r="I75" s="30" t="s">
+        <v>3</v>
+      </c>
+      <c r="J75" s="29"/>
+      <c r="K75" s="30" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="13.9" thickBot="1">
+      <c r="A76" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B75" s="20"/>
-      <c r="C75" s="31" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="78" spans="1:11" ht="17.649999999999999">
-      <c r="A78" s="2" t="s">
+      <c r="B76" s="20"/>
+      <c r="C76" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="D76" s="20"/>
+      <c r="E76" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="F76" s="31"/>
+      <c r="G76" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="H76" s="20"/>
+      <c r="I76" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="J76" s="20"/>
+      <c r="K76" s="31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="13.9" thickTop="1"/>
+    <row r="79" spans="1:11" ht="17.649999999999999">
+      <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="80" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
-      <c r="A80" s="3" t="s">
+    <row r="80" spans="1:11" ht="13.9" thickBot="1"/>
+    <row r="81" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+      <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B80" s="3" t="s">
+      <c r="B81" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C80" s="3" t="s">
+      <c r="C81" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="13.9" thickTop="1">
-      <c r="A81" s="4" t="s">
+    <row r="82" spans="1:3" ht="13.9" thickTop="1">
+      <c r="A82" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B81" s="5">
+      <c r="B82" s="5">
         <v>1</v>
       </c>
-      <c r="C81" s="14" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3">
-      <c r="A82" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="B82" s="35">
-        <v>4</v>
-      </c>
-      <c r="C82" s="17" t="s">
+      <c r="C82" s="14" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="B83" s="35">
+        <v>4</v>
+      </c>
+      <c r="C83" s="17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B83" s="35">
+      <c r="B84" s="35">
         <v>2.5</v>
       </c>
-      <c r="C83" s="36" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" ht="15">
-      <c r="A84" s="53" t="s">
+      <c r="C84" s="36" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" ht="15">
+      <c r="A85" s="53" t="s">
         <v>131</v>
       </c>
-      <c r="B84" s="37">
+      <c r="B85" s="37">
         <v>22</v>
       </c>
-      <c r="C84" s="18" t="s">
+      <c r="C85" s="18" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3">
-      <c r="A85" s="53" t="s">
-        <v>130</v>
-      </c>
-      <c r="B85" s="35">
-        <v>1</v>
-      </c>
-      <c r="C85" s="18" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" s="53" t="s">
-        <v>129</v>
-      </c>
-      <c r="B86" s="16"/>
+        <v>130</v>
+      </c>
+      <c r="B86" s="35">
+        <v>1</v>
+      </c>
       <c r="C86" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" s="53" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B87" s="16"/>
       <c r="C87" s="18" t="s">
-        <v>135</v>
+        <v>26</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" s="53" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B88" s="16"/>
       <c r="C88" s="18" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" s="53" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B89" s="16"/>
       <c r="C89" s="18" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" s="53" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B90" s="16"/>
       <c r="C90" s="18" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" s="53" t="s">
-        <v>27</v>
+        <v>134</v>
       </c>
       <c r="B91" s="16"/>
       <c r="C91" s="18" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" s="53" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B92" s="16"/>
       <c r="C92" s="18" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" s="53" t="s">
-        <v>127</v>
+        <v>28</v>
       </c>
       <c r="B93" s="16"/>
       <c r="C93" s="18" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" s="53" t="s">
+        <v>127</v>
+      </c>
+      <c r="B94" s="16"/>
+      <c r="C94" s="18" t="s">
         <v>141</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3">
-      <c r="A94" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="B94" s="35">
-        <v>4.7</v>
-      </c>
-      <c r="C94" s="18" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B95" s="35">
-        <v>10</v>
+        <v>4.7</v>
       </c>
       <c r="C95" s="18" t="s">
         <v>29</v>
@@ -3254,186 +3484,193 @@
     </row>
     <row r="96" spans="1:3">
       <c r="A96" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96" s="35">
+        <v>10</v>
+      </c>
+      <c r="C96" s="18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11">
+      <c r="A97" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B96" s="16"/>
-      <c r="C96" s="18"/>
-    </row>
-    <row r="97" spans="1:11" ht="13.9" thickBot="1">
-      <c r="A97" s="10" t="s">
+      <c r="B97" s="16"/>
+      <c r="C97" s="18"/>
+    </row>
+    <row r="98" spans="1:11" ht="13.9" thickBot="1">
+      <c r="A98" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B97" s="20"/>
-      <c r="C97" s="19"/>
-    </row>
-    <row r="98" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
-      <c r="D98" s="3" t="s">
+      <c r="B98" s="20"/>
+      <c r="C98" s="19"/>
+    </row>
+    <row r="99" spans="1:11" ht="13.9" thickTop="1"/>
+    <row r="101" spans="1:11" ht="17.649999999999999">
+      <c r="A101" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" ht="13.9" thickBot="1"/>
+    <row r="103" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
+      <c r="A103" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B103" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E98" s="3" t="s">
+      <c r="C103" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F98" s="3"/>
-      <c r="G98" s="3"/>
-      <c r="H98" s="3" t="s">
+      <c r="D103" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="I98" s="3" t="s">
+      <c r="E103" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J98" s="3" t="s">
+      <c r="F103" s="3"/>
+      <c r="G103" s="3"/>
+      <c r="H103" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="K98" s="3" t="s">
+      <c r="I103" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="99" spans="1:11" ht="13.9" thickTop="1">
-      <c r="D99" s="8">
-        <f>D40</f>
-        <v>0</v>
-      </c>
-      <c r="E99" s="23" t="s">
+      <c r="J103" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="K103" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" ht="13.9" thickTop="1">
+      <c r="A104" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B104" s="8">
+        <f>B44</f>
+        <v>50</v>
+      </c>
+      <c r="C104" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="F99" s="8">
-        <f>F40</f>
-        <v>0</v>
-      </c>
-      <c r="G99" s="23" t="s">
+      <c r="D104" s="8">
+        <f>D44</f>
+        <v>50</v>
+      </c>
+      <c r="E104" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="H99" s="8">
-        <f>H40</f>
-        <v>0</v>
-      </c>
-      <c r="I99" s="23" t="s">
+      <c r="F104" s="8">
+        <f>F44</f>
+        <v>5</v>
+      </c>
+      <c r="G104" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="J99" s="8">
-        <f>J40</f>
-        <v>0</v>
-      </c>
-      <c r="K99" s="24" t="s">
+      <c r="H104" s="8">
+        <f>H44</f>
+        <v>5</v>
+      </c>
+      <c r="I104" s="23" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="100" spans="1:11" ht="17.649999999999999">
-      <c r="A100" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D100" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="E100" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="F100" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="G100" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="H100" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="I100" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="J100" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="K100" s="24" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="101" spans="1:11" ht="13.9" thickBot="1">
-      <c r="D101" s="25"/>
-      <c r="E101" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="F101" s="23"/>
-      <c r="G101" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="H101" s="25"/>
-      <c r="I101" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="J101" s="25"/>
-      <c r="K101" s="24" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="102" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
-      <c r="A102" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B102" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C102" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D102" s="20"/>
-      <c r="E102" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="F102" s="31"/>
-      <c r="G102" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="H102" s="20"/>
-      <c r="I102" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="J102" s="20"/>
-      <c r="K102" s="32" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="103" spans="1:11" ht="13.9" thickTop="1">
-      <c r="A103" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B103" s="8">
-        <f>B44</f>
-        <v>0</v>
-      </c>
-      <c r="C103" s="23" t="s">
+      <c r="J104" s="8">
+        <f>J44</f>
+        <v>9.0909090909090917</v>
+      </c>
+      <c r="K104" s="24" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11">
-      <c r="A104" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B104" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="C104" s="23" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="105" spans="1:11">
       <c r="A105" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B105" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="C105" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D105" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="E105" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F105" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="G105" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="H105" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="I105" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="J105" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="K105" s="24" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11">
+      <c r="A106" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B105" s="25"/>
-      <c r="C105" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="106" spans="1:11" ht="13.9" thickBot="1">
-      <c r="A106" s="10" t="s">
+      <c r="B106" s="25"/>
+      <c r="C106" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D106" s="25"/>
+      <c r="E106" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F106" s="23"/>
+      <c r="G106" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="H106" s="25"/>
+      <c r="I106" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="J106" s="25"/>
+      <c r="K106" s="24" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" ht="13.9" thickBot="1">
+      <c r="A107" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B106" s="20"/>
-      <c r="C106" s="31" t="s">
+      <c r="B107" s="20"/>
+      <c r="C107" s="31" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="107" spans="1:11" ht="13.9" thickTop="1"/>
+      <c r="D107" s="20"/>
+      <c r="E107" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="F107" s="31"/>
+      <c r="G107" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="H107" s="20"/>
+      <c r="I107" s="31" t="s">
+        <v>36</v>
+      </c>
+      <c r="J107" s="20"/>
+      <c r="K107" s="32" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" ht="13.9" thickTop="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3449,18 +3686,18 @@
     <col min="2" max="9" width="12.8125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21">
+    <row r="1" spans="1:3" ht="20.65">
       <c r="A1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.5">
+    <row r="3" spans="1:3" ht="17.649999999999999">
       <c r="A3" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1"/>
-    <row r="5" spans="1:3" ht="15.5" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -3483,43 +3720,43 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="14.55">
+    <row r="7" spans="1:3">
       <c r="A7" s="39" t="s">
         <v>94</v>
       </c>
       <c r="B7" s="8">
-        <f>SS_Analysis!H42</f>
-        <v>0</v>
+        <f>SS_Analysis!H46</f>
+        <v>1.4285714285714286</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="14.55">
+    <row r="8" spans="1:3">
       <c r="A8" s="39" t="s">
         <v>95</v>
       </c>
       <c r="B8" s="8">
-        <f>SS_Analysis!H45</f>
-        <v>0</v>
+        <f>SS_Analysis!H49</f>
+        <v>1.540273556231003</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="14.55">
+    <row r="9" spans="1:3">
       <c r="A9" s="39" t="s">
         <v>93</v>
       </c>
       <c r="B9" s="8">
-        <f>SS_Analysis!H46</f>
-        <v>0</v>
+        <f>SS_Analysis!H51</f>
+        <v>1.4300263802829551</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="14.55">
+    <row r="10" spans="1:3">
       <c r="A10" s="7" t="s">
         <v>63</v>
       </c>
@@ -3530,7 +3767,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1">
+    <row r="11" spans="1:3" ht="13.9" thickBot="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -3542,18 +3779,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.5" thickTop="1">
+    <row r="12" spans="1:3" ht="15.4" thickTop="1">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18.5">
+    <row r="14" spans="1:3" ht="17.649999999999999">
       <c r="A14" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="19.05" thickBot="1">
+    <row r="15" spans="1:3" ht="18" thickBot="1">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:3" ht="15.5" thickTop="1" thickBot="1">
+    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -3564,7 +3801,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1">
+    <row r="17" spans="1:3" ht="13.9" thickTop="1">
       <c r="A17" s="60" t="s">
         <v>66</v>
       </c>
@@ -3573,7 +3810,7 @@
       </c>
       <c r="C17" s="62"/>
     </row>
-    <row r="18" spans="1:3" ht="14.55">
+    <row r="18" spans="1:3">
       <c r="A18" s="63" t="s">
         <v>68</v>
       </c>
@@ -3582,7 +3819,7 @@
       </c>
       <c r="C18" s="65"/>
     </row>
-    <row r="19" spans="1:3" ht="14.55">
+    <row r="19" spans="1:3">
       <c r="A19" s="63" t="s">
         <v>70</v>
       </c>
@@ -3591,7 +3828,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="14.55">
+    <row r="20" spans="1:3">
       <c r="A20" s="63" t="s">
         <v>72</v>
       </c>
@@ -3600,7 +3837,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="14.55">
+    <row r="21" spans="1:3">
       <c r="A21" s="63" t="s">
         <v>74</v>
       </c>
@@ -3609,7 +3846,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="14.55">
+    <row r="22" spans="1:3">
       <c r="A22" s="63" t="s">
         <v>76</v>
       </c>
@@ -3618,7 +3855,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="14.55">
+    <row r="23" spans="1:3">
       <c r="A23" s="63" t="s">
         <v>77</v>
       </c>
@@ -3652,7 +3889,7 @@
       <c r="B26" s="69"/>
       <c r="C26" s="65"/>
     </row>
-    <row r="27" spans="1:3" ht="15" thickBot="1">
+    <row r="27" spans="1:3" ht="13.9" thickBot="1">
       <c r="A27" s="70" t="s">
         <v>83</v>
       </c>
@@ -3661,14 +3898,14 @@
       </c>
       <c r="C27" s="72"/>
     </row>
-    <row r="28" spans="1:3" ht="15" thickTop="1"/>
-    <row r="30" spans="1:3" ht="18.5">
+    <row r="28" spans="1:3" ht="13.9" thickTop="1"/>
+    <row r="30" spans="1:3" ht="17.649999999999999">
       <c r="A30" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickBot="1"/>
-    <row r="32" spans="1:3" ht="15.5" thickTop="1" thickBot="1">
+    <row r="31" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="32" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -3679,7 +3916,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15" thickTop="1">
+    <row r="33" spans="1:7" ht="13.9" thickTop="1">
       <c r="A33" s="60" t="s">
         <v>85</v>
       </c>
@@ -3691,7 +3928,7 @@
       </c>
       <c r="G33" s="75"/>
     </row>
-    <row r="34" spans="1:7" ht="14.55">
+    <row r="34" spans="1:7">
       <c r="A34" s="76" t="s">
         <v>86</v>
       </c>
@@ -3701,7 +3938,7 @@
       </c>
       <c r="G34" s="75"/>
     </row>
-    <row r="35" spans="1:7" ht="14.55">
+    <row r="35" spans="1:7">
       <c r="A35" s="76" t="s">
         <v>87</v>
       </c>
@@ -3712,7 +3949,7 @@
       <c r="F35" s="80"/>
       <c r="G35" s="75"/>
     </row>
-    <row r="36" spans="1:7" ht="16.05">
+    <row r="36" spans="1:7" ht="15">
       <c r="A36" s="76" t="s">
         <v>88</v>
       </c>
@@ -3725,7 +3962,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7" ht="14.55">
+    <row r="37" spans="1:7">
       <c r="A37" s="76" t="s">
         <v>89</v>
       </c>
@@ -3734,7 +3971,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="14.55">
+    <row r="38" spans="1:7">
       <c r="A38" s="83" t="s">
         <v>97</v>
       </c>

</xml_diff>

<commit_message>
Updated parameters for closed-loop control.
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6A9838-3AA0-4CF2-BCC0-2FC60A914F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A17E6D0C-E121-4CE3-9E2E-7720434B02C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="163">
   <si>
     <t>Parameter</t>
   </si>
@@ -524,6 +524,9 @@
   </si>
   <si>
     <t>0.46V (@3A)</t>
+  </si>
+  <si>
+    <t>300 - 3000</t>
   </si>
 </sst>
 </file>
@@ -1463,7 +1466,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1586,6 +1589,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -3403,7 +3407,9 @@
       <c r="A87" s="53" t="s">
         <v>129</v>
       </c>
-      <c r="B87" s="16"/>
+      <c r="B87" s="16">
+        <v>18</v>
+      </c>
       <c r="C87" s="18" t="s">
         <v>26</v>
       </c>
@@ -3412,7 +3418,9 @@
       <c r="A88" s="53" t="s">
         <v>128</v>
       </c>
-      <c r="B88" s="16"/>
+      <c r="B88" s="16">
+        <v>0.22</v>
+      </c>
       <c r="C88" s="18" t="s">
         <v>135</v>
       </c>
@@ -3421,7 +3429,9 @@
       <c r="A89" s="53" t="s">
         <v>132</v>
       </c>
-      <c r="B89" s="16"/>
+      <c r="B89" s="16">
+        <v>10</v>
+      </c>
       <c r="C89" s="18" t="s">
         <v>136</v>
       </c>
@@ -3430,7 +3440,9 @@
       <c r="A90" s="53" t="s">
         <v>133</v>
       </c>
-      <c r="B90" s="16"/>
+      <c r="B90" s="16">
+        <v>68</v>
+      </c>
       <c r="C90" s="18" t="s">
         <v>137</v>
       </c>
@@ -3439,7 +3451,9 @@
       <c r="A91" s="53" t="s">
         <v>134</v>
       </c>
-      <c r="B91" s="16"/>
+      <c r="B91" s="16">
+        <v>220</v>
+      </c>
       <c r="C91" s="18" t="s">
         <v>138</v>
       </c>
@@ -3448,7 +3462,9 @@
       <c r="A92" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="B92" s="16"/>
+      <c r="B92" s="16">
+        <v>12</v>
+      </c>
       <c r="C92" s="18" t="s">
         <v>139</v>
       </c>
@@ -3457,7 +3473,9 @@
       <c r="A93" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="B93" s="16"/>
+      <c r="B93" s="16">
+        <v>22</v>
+      </c>
       <c r="C93" s="18" t="s">
         <v>140</v>
       </c>
@@ -3466,7 +3484,9 @@
       <c r="A94" s="53" t="s">
         <v>127</v>
       </c>
-      <c r="B94" s="16"/>
+      <c r="B94" s="16">
+        <v>2200</v>
+      </c>
       <c r="C94" s="18" t="s">
         <v>141</v>
       </c>
@@ -3497,14 +3517,18 @@
       <c r="A97" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B97" s="16"/>
+      <c r="B97" s="108">
+        <v>1</v>
+      </c>
       <c r="C97" s="18"/>
     </row>
     <row r="98" spans="1:11" ht="13.9" thickBot="1">
       <c r="A98" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B98" s="20"/>
+      <c r="B98" s="20" t="s">
+        <v>162</v>
+      </c>
       <c r="C98" s="19"/>
     </row>
     <row r="99" spans="1:11" ht="13.9" thickTop="1"/>
@@ -3596,7 +3620,7 @@
         <v>3</v>
       </c>
       <c r="D105" s="8">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="E105" s="23" t="s">
         <v>3</v>
@@ -3608,13 +3632,13 @@
         <v>3</v>
       </c>
       <c r="H105" s="8">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="I105" s="23" t="s">
         <v>3</v>
       </c>
       <c r="J105" s="8">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="K105" s="24" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
Tested open loop steady-state. Simulations match calculations.
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wwei275\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A17E6D0C-E121-4CE3-9E2E-7720434B02C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA8CBFA0-FA2E-463F-95BC-A72C55469A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -30,15 +30,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="167">
   <si>
     <t>Parameter</t>
   </si>
@@ -527,20 +524,33 @@
   </si>
   <si>
     <t>300 - 3000</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Vout (avg)</t>
+  </si>
+  <si>
+    <t>Pout (avg)</t>
+  </si>
+  <si>
+    <t>mV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000E+00"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.00000"/>
     <numFmt numFmtId="168" formatCode="0.0000000"/>
+    <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1466,7 +1476,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1585,17 +1595,22 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="57" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="57" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Per cent" xfId="3" builtinId="5"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1928,26 +1943,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
   <dimension ref="A1:N108"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.4375" customWidth="1"/>
-    <col min="2" max="11" width="12.8125" customWidth="1"/>
-    <col min="12" max="12" width="17.4375" customWidth="1"/>
-    <col min="13" max="13" width="18.875" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
+    <col min="2" max="11" width="12.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.65">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.649999999999999">
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -1958,7 +1973,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="13.9" thickTop="1">
+    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="38" t="s">
         <v>37</v>
       </c>
@@ -1969,7 +1984,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
         <v>38</v>
       </c>
@@ -1980,7 +1995,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
         <v>39</v>
       </c>
@@ -1991,7 +2006,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
         <v>57</v>
       </c>
@@ -2002,7 +2017,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="39" t="s">
         <v>58</v>
       </c>
@@ -2013,7 +2028,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.9" thickBot="1">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -2024,16 +2039,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.4" thickTop="1">
+    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="17.649999999999999">
+    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -2044,7 +2059,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="13.9" thickTop="1">
+    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="46" t="s">
         <v>42</v>
       </c>
@@ -2056,7 +2071,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="48" t="s">
         <v>41</v>
       </c>
@@ -2068,7 +2083,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="57" t="s">
         <v>60</v>
       </c>
@@ -2080,7 +2095,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="50" t="s">
         <v>61</v>
       </c>
@@ -2092,7 +2107,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="53" t="s">
         <v>44</v>
       </c>
@@ -2104,7 +2119,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="53" t="s">
         <v>151</v>
       </c>
@@ -2116,7 +2131,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="53" t="s">
         <v>45</v>
       </c>
@@ -2128,7 +2143,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="96" t="s">
         <v>152</v>
       </c>
@@ -2140,7 +2155,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="13.9" thickBot="1">
+    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="88" t="s">
         <v>104</v>
       </c>
@@ -2151,14 +2166,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="13.9" thickTop="1"/>
-    <row r="28" spans="1:3" ht="17.649999999999999">
+    <row r="26" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="30" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>0</v>
       </c>
@@ -2169,7 +2184,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="13.9" thickTop="1">
+    <row r="31" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -2180,7 +2195,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="98" t="s">
         <v>153</v>
       </c>
@@ -2192,7 +2207,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -2204,7 +2219,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="28" t="s">
         <v>154</v>
       </c>
@@ -2216,7 +2231,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="13.9" thickBot="1">
+    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
@@ -2227,14 +2242,14 @@
         <v>110</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="38" spans="1:11" ht="17.649999999999999">
+    <row r="36" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="40" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
+    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>0</v>
       </c>
@@ -2269,7 +2284,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="13.9" thickTop="1">
+    <row r="41" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -2304,7 +2319,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="45" t="s">
         <v>40</v>
       </c>
@@ -2339,7 +2354,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -2375,7 +2390,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -2415,7 +2430,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="45" spans="1:11">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
@@ -2455,39 +2470,39 @@
         <v>112</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="B46" s="25">
+      <c r="B46" s="103">
         <f>B43/B42</f>
         <v>0.2</v>
       </c>
-      <c r="C46" s="23" t="s">
+      <c r="C46" s="103" t="s">
         <v>113</v>
       </c>
-      <c r="D46" s="25">
+      <c r="D46" s="103">
         <f>D43/D42</f>
         <v>0.14285714285714285</v>
       </c>
-      <c r="E46" s="23" t="s">
+      <c r="E46" s="103" t="s">
         <v>113</v>
       </c>
-      <c r="F46" s="25">
+      <c r="F46" s="103">
         <f>F43/F42</f>
         <v>2</v>
       </c>
-      <c r="G46" s="23" t="s">
+      <c r="G46" s="103" t="s">
         <v>113</v>
       </c>
-      <c r="H46" s="25">
+      <c r="H46" s="103">
         <f>H43/H42</f>
         <v>1.4285714285714286</v>
       </c>
-      <c r="I46" s="23" t="s">
+      <c r="I46" s="103" t="s">
         <v>113</v>
       </c>
-      <c r="J46" s="25">
+      <c r="J46" s="103">
         <f>J43/J42</f>
         <v>0.91666666666666663</v>
       </c>
@@ -2495,39 +2510,39 @@
         <v>113</v>
       </c>
     </row>
-    <row r="47" spans="1:11">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="B47" s="25">
+      <c r="B47" s="103">
         <f>B42*B45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.26595744680851069</v>
       </c>
-      <c r="C47" s="23" t="s">
+      <c r="C47" s="103" t="s">
         <v>114</v>
       </c>
-      <c r="D47" s="25">
+      <c r="D47" s="103">
         <f>D42*D45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.22340425531914904</v>
       </c>
-      <c r="E47" s="23" t="s">
+      <c r="E47" s="103" t="s">
         <v>114</v>
       </c>
-      <c r="F47" s="25">
+      <c r="F47" s="103">
         <f>F42*F45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.26595744680851069</v>
       </c>
-      <c r="G47" s="23" t="s">
+      <c r="G47" s="103" t="s">
         <v>114</v>
       </c>
-      <c r="H47" s="25">
+      <c r="H47" s="103">
         <f>H42*H45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.22340425531914904</v>
       </c>
-      <c r="I47" s="23" t="s">
+      <c r="I47" s="103" t="s">
         <v>114</v>
       </c>
-      <c r="J47" s="25">
+      <c r="J47" s="103">
         <f>J42*J45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.2553191489361703</v>
       </c>
@@ -2535,7 +2550,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="48" spans="1:11">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
@@ -2565,7 +2580,7 @@
       </c>
       <c r="K48" s="24"/>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>49</v>
       </c>
@@ -2605,7 +2620,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>158</v>
       </c>
@@ -2645,7 +2660,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>48</v>
       </c>
@@ -2685,7 +2700,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="28" t="s">
         <v>50</v>
       </c>
@@ -2725,7 +2740,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="28" t="s">
         <v>52</v>
       </c>
@@ -2765,116 +2780,111 @@
         <v>118</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="28" t="s">
         <v>51</v>
       </c>
       <c r="B54" s="104">
-        <f>SQRT(B46^2*B45*(1-B45) + (B47^2/12))</f>
-        <v>0.12607318096807302</v>
+        <f>SQRT(B46^2*B45*(1-B45) + (B47^2/12)*(1-B45))</f>
+        <v>0.11378586678363989</v>
       </c>
       <c r="C54" s="23" t="s">
         <v>119</v>
       </c>
       <c r="D54" s="104">
-        <f>SQRT(D46^2*D45*(1-D45) + (D47^2/12))</f>
-        <v>9.1895789132434749E-2</v>
+        <f t="shared" ref="D54:J54" si="0">SQRT(D46^2*D45*(1-D45) + (D47^2/12)*(1-D45))</f>
+        <v>8.4835720825047062E-2</v>
       </c>
       <c r="E54" s="23" t="s">
         <v>119</v>
       </c>
       <c r="F54" s="104">
-        <f>SQRT(F46^2*F45*(1-F45) + (F47^2/12))</f>
-        <v>1.0029428931696003</v>
+        <f t="shared" si="0"/>
+        <v>1.0014725275711283</v>
       </c>
       <c r="G54" s="23" t="s">
         <v>119</v>
       </c>
       <c r="H54" s="104">
-        <f>SQRT(H46^2*H45*(1-H45) + (H47^2/12))</f>
-        <v>0.65782258272727856</v>
+        <f t="shared" si="0"/>
+        <v>0.65687351431886776</v>
       </c>
       <c r="I54" s="23" t="s">
         <v>119</v>
       </c>
       <c r="J54" s="104">
-        <f>SQRT(J46^2*J45*(1-J45) + (J47^2/12))</f>
-        <v>0.45508129931305408</v>
+        <f t="shared" si="0"/>
+        <v>0.45268759653578</v>
       </c>
       <c r="K54" s="23" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>53</v>
       </c>
       <c r="B55" s="29">
-        <f>B41-B56</f>
-        <v>4.54</v>
+        <v>5</v>
       </c>
       <c r="C55" s="23" t="s">
         <v>120</v>
       </c>
       <c r="D55" s="29">
-        <f>D41-D56</f>
-        <v>4.54</v>
+        <v>5</v>
       </c>
       <c r="E55" s="23" t="s">
         <v>120</v>
       </c>
       <c r="F55" s="29">
-        <f>F41-F56</f>
-        <v>4.54</v>
+        <v>5</v>
       </c>
       <c r="G55" s="23" t="s">
         <v>120</v>
       </c>
       <c r="H55" s="29">
-        <f>H41-H56</f>
-        <v>4.54</v>
+        <v>5</v>
       </c>
       <c r="I55" s="23" t="s">
         <v>120</v>
       </c>
       <c r="J55" s="29">
-        <f>J41-J56</f>
-        <v>4.54</v>
+        <v>5</v>
       </c>
       <c r="K55" s="23" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="28" t="s">
         <v>54</v>
       </c>
       <c r="B56" s="107">
-        <v>0.46</v>
+        <v>5</v>
       </c>
       <c r="C56" s="23" t="s">
         <v>121</v>
       </c>
       <c r="D56" s="107">
-        <v>0.46</v>
+        <v>5</v>
       </c>
       <c r="E56" s="23" t="s">
         <v>121</v>
       </c>
       <c r="F56" s="107">
-        <v>0.46</v>
+        <v>5</v>
       </c>
       <c r="G56" s="23" t="s">
         <v>121</v>
       </c>
       <c r="H56" s="107">
-        <v>0.46</v>
+        <v>5</v>
       </c>
       <c r="I56" s="23" t="s">
         <v>121</v>
       </c>
       <c r="J56" s="107">
-        <v>0.46</v>
+        <v>5</v>
       </c>
       <c r="K56" s="23" t="s">
         <v>121</v>
@@ -2889,7 +2899,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="13.9" thickBot="1">
+    <row r="57" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="10" t="s">
         <v>55</v>
       </c>
@@ -2929,21 +2939,21 @@
         <v>122</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="13.9" thickTop="1">
+    <row r="58" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B58" s="33"/>
       <c r="C58" s="34"/>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B59" s="33"/>
       <c r="C59" s="34"/>
     </row>
-    <row r="60" spans="1:14" ht="17.649999999999999">
+    <row r="60" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="13.9" thickBot="1"/>
-    <row r="62" spans="1:14" ht="14.65" thickTop="1" thickBot="1">
+    <row r="61" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="62" spans="1:14" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
         <v>0</v>
       </c>
@@ -2974,7 +2984,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="13.9" thickTop="1">
+    <row r="63" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -3014,7 +3024,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -3044,300 +3054,436 @@
       </c>
       <c r="K64" s="24"/>
     </row>
-    <row r="65" spans="1:11">
-      <c r="A65" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B65" s="25"/>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A65" s="39" t="s">
+        <v>164</v>
+      </c>
+      <c r="B65" s="103">
+        <v>4.9983700000000004</v>
+      </c>
       <c r="C65" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D65" s="25"/>
+      <c r="D65" s="103">
+        <v>4.9908000000000001</v>
+      </c>
       <c r="E65" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="F65" s="23"/>
-      <c r="G65" s="23"/>
-      <c r="H65" s="25"/>
+      <c r="F65" s="108">
+        <v>4.9982800000000003</v>
+      </c>
+      <c r="G65" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="H65" s="103">
+        <v>4.9980099999999998</v>
+      </c>
       <c r="I65" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="J65" s="25"/>
+      <c r="J65" s="103">
+        <v>4.9981</v>
+      </c>
       <c r="K65" s="24" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:11">
-      <c r="A66" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B66" s="25"/>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A66" s="39" t="s">
+        <v>165</v>
+      </c>
+      <c r="B66" s="103">
+        <v>0.49967400000000001</v>
+      </c>
       <c r="C66" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="D66" s="25"/>
+      <c r="D66" s="103">
+        <v>0.49961699999999998</v>
+      </c>
       <c r="E66" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="F66" s="23"/>
-      <c r="G66" s="23"/>
-      <c r="H66" s="25"/>
+      <c r="F66" s="103">
+        <v>4.9968300000000001</v>
+      </c>
+      <c r="G66" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="H66" s="103">
+        <v>4.9961099999999998</v>
+      </c>
       <c r="I66" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="J66" s="25"/>
+      <c r="J66" s="103">
+        <v>2.7482099999999998</v>
+      </c>
       <c r="K66" s="24" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:11">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B67" s="27"/>
+      <c r="B67" s="27" t="s">
+        <v>163</v>
+      </c>
       <c r="C67" s="23"/>
-      <c r="D67" s="27"/>
+      <c r="D67" s="108" t="s">
+        <v>163</v>
+      </c>
       <c r="E67" s="23"/>
-      <c r="F67" s="23"/>
+      <c r="F67" s="108" t="s">
+        <v>163</v>
+      </c>
       <c r="G67" s="23"/>
-      <c r="H67" s="27"/>
+      <c r="H67" s="108" t="s">
+        <v>163</v>
+      </c>
       <c r="I67" s="23"/>
-      <c r="J67" s="27"/>
+      <c r="J67" s="108" t="s">
+        <v>163</v>
+      </c>
       <c r="K67" s="24"/>
     </row>
-    <row r="68" spans="1:11">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="B68" s="27"/>
+      <c r="B68" s="108">
+        <f>0.332881-0.0669235</f>
+        <v>0.26595749999999996</v>
+      </c>
       <c r="C68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D68" s="27"/>
+      <c r="D68" s="108">
+        <f>0.254488-0.0310839</f>
+        <v>0.22340409999999999</v>
+      </c>
       <c r="E68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F68" s="23"/>
+      <c r="F68" s="103">
+        <f>2.13197-1.86601</f>
+        <v>0.26595999999999997</v>
+      </c>
       <c r="G68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H68" s="27"/>
+      <c r="H68" s="108">
+        <f>1.53955-1.31615</f>
+        <v>0.22340000000000004</v>
+      </c>
       <c r="I68" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J68" s="27"/>
+      <c r="J68" s="108">
+        <f>1.04393-0.788614</f>
+        <v>0.25531599999999999</v>
+      </c>
       <c r="K68" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:11">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B69" s="25"/>
+      <c r="B69" s="103">
+        <v>0.33288099999999998</v>
+      </c>
       <c r="C69" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D69" s="25"/>
+      <c r="D69" s="103">
+        <v>0.25448799999999999</v>
+      </c>
       <c r="E69" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F69" s="23"/>
+      <c r="F69" s="103">
+        <v>2.1319699999999999</v>
+      </c>
       <c r="G69" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H69" s="25"/>
+      <c r="H69" s="103">
+        <v>1.53955</v>
+      </c>
       <c r="I69" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J69" s="25"/>
+      <c r="J69" s="103">
+        <v>1.04393</v>
+      </c>
       <c r="K69" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:11">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B70" s="25"/>
+      <c r="B70" s="103">
+        <v>0.214139</v>
+      </c>
       <c r="C70" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D70" s="25"/>
+      <c r="D70" s="103">
+        <v>0.15667500000000001</v>
+      </c>
       <c r="E70" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F70" s="23"/>
+      <c r="F70" s="103">
+        <v>2.0004599999999999</v>
+      </c>
       <c r="G70" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H70" s="25"/>
+      <c r="H70" s="103">
+        <f>1.42931</f>
+        <v>1.4293100000000001</v>
+      </c>
       <c r="I70" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J70" s="25"/>
+      <c r="J70" s="103">
+        <v>0.91923299999999997</v>
+      </c>
       <c r="K70" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:11">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" s="28" t="s">
         <v>50</v>
       </c>
-      <c r="B71" s="29"/>
+      <c r="B71" s="109">
+        <v>9.9967399999999998E-2</v>
+      </c>
       <c r="C71" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D71" s="29"/>
+      <c r="D71" s="104">
+        <v>9.9942699999999995E-2</v>
+      </c>
       <c r="E71" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F71" s="30"/>
+      <c r="F71" s="103">
+        <v>0.99965599999999999</v>
+      </c>
       <c r="G71" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H71" s="29"/>
+      <c r="H71" s="104">
+        <v>0.99960099999999996</v>
+      </c>
       <c r="I71" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J71" s="29"/>
+      <c r="J71" s="104">
+        <v>0.54984599999999995</v>
+      </c>
       <c r="K71" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:11">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="B72" s="29"/>
+      <c r="B72" s="104">
+        <v>0.151419</v>
+      </c>
       <c r="C72" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D72" s="29"/>
+      <c r="D72" s="104">
+        <v>8.5814299999999996E-2</v>
+      </c>
       <c r="E72" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F72" s="30"/>
+      <c r="F72" s="109">
+        <v>1.4145399999999999</v>
+      </c>
       <c r="G72" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H72" s="29"/>
+      <c r="H72" s="104">
+        <v>0.78286299999999998</v>
+      </c>
       <c r="I72" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J72" s="29"/>
+      <c r="J72" s="104">
+        <v>0.58137399999999995</v>
+      </c>
       <c r="K72" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:11">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="B73" s="29"/>
+      <c r="B73" s="104">
+        <v>0.113757</v>
+      </c>
       <c r="C73" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D73" s="29"/>
+      <c r="D73" s="104">
+        <v>8.4824099999999999E-2</v>
+      </c>
       <c r="E73" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="F73" s="30"/>
+      <c r="F73" s="104">
+        <v>1.0011399999999999</v>
+      </c>
       <c r="G73" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="H73" s="29"/>
+      <c r="H73" s="104">
+        <v>0.65672399999999997</v>
+      </c>
       <c r="I73" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="J73" s="29"/>
+      <c r="J73" s="104">
+        <v>0.452598</v>
+      </c>
       <c r="K73" s="23" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="74" spans="1:11">
+      <c r="L73" s="110"/>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B74" s="29"/>
+      <c r="B74" s="104">
+        <v>5.00204</v>
+      </c>
       <c r="C74" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D74" s="29"/>
+      <c r="D74" s="104">
+        <v>5.0002899999999997</v>
+      </c>
       <c r="E74" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="F74" s="30"/>
+      <c r="F74" s="104">
+        <v>5.0350299999999999</v>
+      </c>
       <c r="G74" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="H74" s="29"/>
+      <c r="H74" s="104">
+        <v>5.02006</v>
+      </c>
       <c r="I74" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="J74" s="29"/>
+      <c r="J74" s="104">
+        <v>5.0142699999999998</v>
+      </c>
       <c r="K74" s="23" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:11">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="B75" s="29"/>
+      <c r="B75" s="104">
+        <v>5.00204</v>
+      </c>
       <c r="C75" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="D75" s="29"/>
+      <c r="D75" s="104">
+        <v>5.0002899999999997</v>
+      </c>
       <c r="E75" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="F75" s="30"/>
+      <c r="F75" s="104">
+        <v>5.0350299999999999</v>
+      </c>
       <c r="G75" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="H75" s="29"/>
+      <c r="H75" s="104">
+        <v>5.02006</v>
+      </c>
       <c r="I75" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="J75" s="29"/>
+      <c r="J75" s="104">
+        <v>5.0142699999999998</v>
+      </c>
       <c r="K75" s="30" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="13.9" thickBot="1">
+    <row r="76" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B76" s="20"/>
+      <c r="B76" s="105">
+        <f>(5.00204-4.99469)*10^3</f>
+        <v>7.3499999999997456</v>
+      </c>
       <c r="C76" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="D76" s="20"/>
+        <v>166</v>
+      </c>
+      <c r="D76" s="105">
+        <f>(5.00029 - 4.99588)*10^3</f>
+        <v>4.410000000000025</v>
+      </c>
       <c r="E76" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="F76" s="31"/>
+        <v>166</v>
+      </c>
+      <c r="F76" s="105">
+        <f>(5.03503-4.96153)*10^3</f>
+        <v>73.500000000000114</v>
+      </c>
       <c r="G76" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="H76" s="20"/>
+        <v>166</v>
+      </c>
+      <c r="H76" s="105">
+        <f>(5.02006-4.97596)*10^3</f>
+        <v>44.10000000000025</v>
+      </c>
       <c r="I76" s="31" t="s">
-        <v>3</v>
-      </c>
-      <c r="J76" s="20"/>
+        <v>166</v>
+      </c>
+      <c r="J76" s="105">
+        <f>(5.01427-4.98192)*10^3</f>
+        <v>32.350000000000101</v>
+      </c>
       <c r="K76" s="31" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="79" spans="1:11" ht="17.649999999999999">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="81" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="80" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="81" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
@@ -3348,7 +3494,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="13.9" thickTop="1">
+    <row r="82" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>125</v>
       </c>
@@ -3359,7 +3505,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
         <v>126</v>
       </c>
@@ -3370,7 +3516,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -3381,7 +3527,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15">
+    <row r="85" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="53" t="s">
         <v>131</v>
       </c>
@@ -3392,7 +3538,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="53" t="s">
         <v>130</v>
       </c>
@@ -3403,7 +3549,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="53" t="s">
         <v>129</v>
       </c>
@@ -3414,7 +3560,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="53" t="s">
         <v>128</v>
       </c>
@@ -3425,7 +3571,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="53" t="s">
         <v>132</v>
       </c>
@@ -3436,7 +3582,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="53" t="s">
         <v>133</v>
       </c>
@@ -3447,7 +3593,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="53" t="s">
         <v>134</v>
       </c>
@@ -3458,7 +3604,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="53" t="s">
         <v>27</v>
       </c>
@@ -3469,7 +3615,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="53" t="s">
         <v>28</v>
       </c>
@@ -3480,7 +3626,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="53" t="s">
         <v>127</v>
       </c>
@@ -3491,7 +3637,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="15" t="s">
         <v>123</v>
       </c>
@@ -3502,7 +3648,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="15" t="s">
         <v>124</v>
       </c>
@@ -3513,16 +3659,16 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B97" s="108">
-        <v>1</v>
+      <c r="B97" s="111">
+        <v>0.1</v>
       </c>
       <c r="C97" s="18"/>
     </row>
-    <row r="98" spans="1:11" ht="13.9" thickBot="1">
+    <row r="98" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="10" t="s">
         <v>31</v>
       </c>
@@ -3531,14 +3677,14 @@
       </c>
       <c r="C98" s="19"/>
     </row>
-    <row r="99" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="101" spans="1:11" ht="17.649999999999999">
+    <row r="99" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="102" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="103" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
+    <row r="102" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="103" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
         <v>0</v>
       </c>
@@ -3569,7 +3715,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="104" spans="1:11" ht="13.9" thickTop="1">
+    <row r="104" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A104" s="7" t="s">
         <v>16</v>
       </c>
@@ -3609,7 +3755,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="105" spans="1:11">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105" s="7" t="s">
         <v>33</v>
       </c>
@@ -3644,7 +3790,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="1:11">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106" s="7" t="s">
         <v>34</v>
       </c>
@@ -3669,7 +3815,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:11" ht="13.9" thickBot="1">
+    <row r="107" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" s="10" t="s">
         <v>35</v>
       </c>
@@ -3694,7 +3840,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="108" spans="1:11" ht="13.9" thickTop="1"/>
+    <row r="108" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3704,24 +3850,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.4375" customWidth="1"/>
-    <col min="2" max="9" width="12.8125" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="2" max="9" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.65">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.649999999999999">
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -3732,7 +3878,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="13.9" thickTop="1">
+    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="38" t="s">
         <v>104</v>
       </c>
@@ -3744,7 +3890,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
         <v>94</v>
       </c>
@@ -3756,7 +3902,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="39" t="s">
         <v>95</v>
       </c>
@@ -3768,7 +3914,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="39" t="s">
         <v>93</v>
       </c>
@@ -3780,7 +3926,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>63</v>
       </c>
@@ -3791,7 +3937,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.9" thickBot="1">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -3803,18 +3949,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.4" thickTop="1">
+    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="17.649999999999999">
+    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18" thickBot="1">
+    <row r="15" spans="1:3" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -3825,7 +3971,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="13.9" thickTop="1">
+    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="60" t="s">
         <v>66</v>
       </c>
@@ -3834,7 +3980,7 @@
       </c>
       <c r="C17" s="62"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="63" t="s">
         <v>68</v>
       </c>
@@ -3843,7 +3989,7 @@
       </c>
       <c r="C18" s="65"/>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="63" t="s">
         <v>70</v>
       </c>
@@ -3852,7 +3998,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="63" t="s">
         <v>72</v>
       </c>
@@ -3861,7 +4007,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="63" t="s">
         <v>74</v>
       </c>
@@ -3870,7 +4016,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="63" t="s">
         <v>76</v>
       </c>
@@ -3879,7 +4025,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="63" t="s">
         <v>77</v>
       </c>
@@ -3888,7 +4034,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="63" t="s">
         <v>78</v>
       </c>
@@ -3897,7 +4043,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="63" t="s">
         <v>80</v>
       </c>
@@ -3906,14 +4052,14 @@
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="68" t="s">
         <v>82</v>
       </c>
       <c r="B26" s="69"/>
       <c r="C26" s="65"/>
     </row>
-    <row r="27" spans="1:3" ht="13.9" thickBot="1">
+    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="70" t="s">
         <v>83</v>
       </c>
@@ -3922,14 +4068,14 @@
       </c>
       <c r="C27" s="72"/>
     </row>
-    <row r="28" spans="1:3" ht="13.9" thickTop="1"/>
-    <row r="30" spans="1:3" ht="17.649999999999999">
+    <row r="28" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="32" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -3940,7 +4086,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="13.9" thickTop="1">
+    <row r="33" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A33" s="60" t="s">
         <v>85</v>
       </c>
@@ -3952,7 +4098,7 @@
       </c>
       <c r="G33" s="75"/>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="76" t="s">
         <v>86</v>
       </c>
@@ -3962,7 +4108,7 @@
       </c>
       <c r="G34" s="75"/>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="76" t="s">
         <v>87</v>
       </c>
@@ -3973,7 +4119,7 @@
       <c r="F35" s="80"/>
       <c r="G35" s="75"/>
     </row>
-    <row r="36" spans="1:7" ht="15">
+    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="76" t="s">
         <v>88</v>
       </c>
@@ -3986,7 +4132,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="76" t="s">
         <v>89</v>
       </c>
@@ -3995,7 +4141,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="83" t="s">
         <v>97</v>
       </c>
@@ -4006,7 +4152,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="83" t="s">
         <v>96</v>
       </c>
@@ -4015,7 +4161,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="83" t="s">
         <v>98</v>
       </c>
@@ -4024,7 +4170,7 @@
       </c>
       <c r="C40" s="78"/>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="83" t="s">
         <v>99</v>
       </c>
@@ -4033,7 +4179,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="13.9" thickBot="1">
+    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="85" t="s">
         <v>90</v>
       </c>
@@ -4042,16 +4188,16 @@
         <v>149</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="13.9" thickTop="1">
+    <row r="43" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B43" s="75"/>
     </row>
-    <row r="45" spans="1:7" ht="17.649999999999999">
+    <row r="45" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="13.9" thickBot="1"/>
-    <row r="47" spans="1:7" ht="14.65" thickTop="1" thickBot="1">
+    <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>0</v>
       </c>
@@ -4062,7 +4208,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="13.9" thickTop="1">
+    <row r="48" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A48" s="83" t="s">
         <v>101</v>
       </c>
@@ -4071,7 +4217,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="76" t="s">
         <v>87</v>
       </c>
@@ -4080,7 +4226,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="83" t="s">
         <v>150</v>
       </c>
@@ -4089,7 +4235,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="13.9" thickBot="1">
+    <row r="51" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="84" t="s">
         <v>102</v>
       </c>
@@ -4098,7 +4244,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="13.9" thickTop="1"/>
+    <row r="52" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Finalised parameters. Closed loop feedback works as intended.
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wwei275\Documents\GitHub\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/wwei275_uoa_auckland_ac_nz/Documents/Documents/GitHub/311/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA8CBFA0-FA2E-463F-95BC-A72C55469A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="13_ncr:1_{AA8CBFA0-FA2E-463F-95BC-A72C55469A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E42D3796-6CCB-4E70-92C7-B89FBA87668C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="166">
   <si>
     <t>Parameter</t>
   </si>
@@ -139,9 +139,6 @@
     <t>Vref</t>
   </si>
   <si>
-    <t>Steady State Vout</t>
-  </si>
-  <si>
     <t>Settling Time (+/- 5%)</t>
   </si>
   <si>
@@ -523,9 +520,6 @@
     <t>0.46V (@3A)</t>
   </si>
   <si>
-    <t>300 - 3000</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -536,6 +530,9 @@
   </si>
   <si>
     <t>mV</t>
+  </si>
+  <si>
+    <t>Steady State Vout (avg)</t>
   </si>
 </sst>
 </file>
@@ -643,7 +640,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="59">
+  <borders count="62">
     <border>
       <left/>
       <right/>
@@ -1467,6 +1464,51 @@
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1476,7 +1518,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1497,7 +1539,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1602,9 +1643,17 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="60" xfId="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="61" xfId="2" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -1623,6 +1672,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>184785</xdr:colOff>
+      <xdr:row>97</xdr:row>
+      <xdr:rowOff>116205</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06663EDE-5E45-D283-182E-D291825479CA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3352800" y="16101060"/>
+          <a:ext cx="3362325" cy="3171825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1953,12 +2051,12 @@
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -1974,8 +2072,8 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="38" t="s">
-        <v>37</v>
+      <c r="A6" s="37" t="s">
+        <v>36</v>
       </c>
       <c r="B6" s="5">
         <v>3.5</v>
@@ -1985,8 +2083,8 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="39" t="s">
-        <v>38</v>
+      <c r="A7" s="38" t="s">
+        <v>37</v>
       </c>
       <c r="B7" s="8">
         <v>2.5</v>
@@ -1996,8 +2094,8 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="39" t="s">
-        <v>39</v>
+      <c r="A8" s="38" t="s">
+        <v>38</v>
       </c>
       <c r="B8" s="8">
         <v>5</v>
@@ -2007,8 +2105,8 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="39" t="s">
-        <v>57</v>
+      <c r="A9" s="38" t="s">
+        <v>56</v>
       </c>
       <c r="B9" s="8">
         <v>5</v>
@@ -2018,13 +2116,13 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="39" t="s">
-        <v>58</v>
-      </c>
-      <c r="B10" s="40">
+      <c r="A10" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="39">
         <v>0.5</v>
       </c>
-      <c r="C10" s="41" t="s">
+      <c r="C10" s="40" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2044,7 +2142,7 @@
     </row>
     <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -2060,106 +2158,106 @@
       </c>
     </row>
     <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="46" t="s">
-        <v>42</v>
-      </c>
-      <c r="B17" s="92">
+      <c r="A17" s="45" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="91">
         <f>1-(B7/B8)</f>
         <v>0.5</v>
       </c>
-      <c r="C17" s="47" t="s">
-        <v>105</v>
+      <c r="C17" s="46" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="48" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="93">
+      <c r="A18" s="47" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="92">
         <f>1-(B6/B9)</f>
         <v>0.30000000000000004</v>
       </c>
-      <c r="C18" s="49" t="s">
-        <v>106</v>
+      <c r="C18" s="48" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="57" t="s">
-        <v>60</v>
-      </c>
-      <c r="B19" s="58">
+      <c r="A19" s="56" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" s="57">
         <f>B9/B7</f>
         <v>2</v>
       </c>
-      <c r="C19" s="59" t="s">
-        <v>107</v>
+      <c r="C19" s="58" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="50" t="s">
-        <v>61</v>
-      </c>
-      <c r="B20" s="51">
+      <c r="A20" s="49" t="s">
+        <v>60</v>
+      </c>
+      <c r="B20" s="50">
         <f>B10/B6</f>
         <v>0.14285714285714285</v>
       </c>
-      <c r="C20" s="52" t="s">
-        <v>108</v>
+      <c r="C20" s="51" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="53" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21" s="94">
+      <c r="A21" s="52" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" s="93">
         <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="53" t="s">
-        <v>151</v>
-      </c>
-      <c r="B22" s="95">
+      <c r="A22" s="52" t="s">
+        <v>150</v>
+      </c>
+      <c r="B22" s="94">
         <f>B8^2/B10</f>
         <v>50</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="53" t="s">
-        <v>45</v>
+      <c r="A23" s="52" t="s">
+        <v>44</v>
       </c>
       <c r="B23" s="16">
         <f>10^6*B22*B21*(1-B21)^2/(2*B11*10^3)</f>
         <v>37.037037037037045</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="96" t="s">
-        <v>152</v>
-      </c>
-      <c r="B24" s="29">
+      <c r="A24" s="95" t="s">
+        <v>151</v>
+      </c>
+      <c r="B24" s="28">
         <f>B23*1.2</f>
         <v>44.44444444444445</v>
       </c>
-      <c r="C24" s="36" t="s">
+      <c r="C24" s="35" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="88" t="s">
-        <v>104</v>
-      </c>
-      <c r="B25" s="97">
+      <c r="A25" s="87" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" s="96">
         <v>47</v>
       </c>
       <c r="C25" s="19" t="s">
@@ -2196,15 +2294,15 @@
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="98" t="s">
-        <v>153</v>
-      </c>
-      <c r="B32" s="99">
+      <c r="A32" s="97" t="s">
+        <v>152</v>
+      </c>
+      <c r="B32" s="98">
         <f>B9/B8</f>
         <v>1</v>
       </c>
-      <c r="C32" s="36" t="s">
-        <v>43</v>
+      <c r="C32" s="35" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2212,34 +2310,34 @@
         <v>11</v>
       </c>
       <c r="B33" s="16">
-        <f>10^6*B32*B17/(B11*10^3*B31)</f>
-        <v>50</v>
+        <f>10^6*B32*B17/(B11/20*10^3*B31)</f>
+        <v>1000</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" s="28" t="s">
-        <v>154</v>
-      </c>
-      <c r="B34" s="29">
+      <c r="A34" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="B34" s="28">
         <f>B33*1.2</f>
-        <v>60</v>
-      </c>
-      <c r="C34" s="100" t="s">
-        <v>110</v>
+        <v>1200</v>
+      </c>
+      <c r="C34" s="99" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B35" s="97">
-        <v>68</v>
+      <c r="B35" s="96">
+        <v>1500</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -2291,66 +2389,66 @@
       <c r="B41" s="5">
         <v>5</v>
       </c>
-      <c r="C41" s="21" t="s">
+      <c r="C41" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="D41" s="54">
+      <c r="D41" s="53">
         <v>5</v>
       </c>
-      <c r="E41" s="21" t="s">
+      <c r="E41" s="20" t="s">
         <v>3</v>
       </c>
       <c r="F41" s="5">
         <v>5</v>
       </c>
-      <c r="G41" s="21" t="s">
+      <c r="G41" s="20" t="s">
         <v>3</v>
       </c>
       <c r="H41" s="5">
         <v>5</v>
       </c>
-      <c r="I41" s="21" t="s">
+      <c r="I41" s="20" t="s">
         <v>3</v>
       </c>
       <c r="J41" s="5">
         <v>5</v>
       </c>
-      <c r="K41" s="22" t="s">
+      <c r="K41" s="21" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" s="45" t="s">
-        <v>40</v>
-      </c>
-      <c r="B42" s="42">
+      <c r="A42" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="B42" s="41">
         <v>2.5</v>
       </c>
-      <c r="C42" s="43" t="s">
+      <c r="C42" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="D42" s="55">
+      <c r="D42" s="54">
         <v>3.5</v>
       </c>
-      <c r="E42" s="43" t="s">
+      <c r="E42" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="F42" s="42">
+      <c r="F42" s="41">
         <v>2.5</v>
       </c>
-      <c r="G42" s="43" t="s">
+      <c r="G42" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="H42" s="42">
+      <c r="H42" s="41">
         <v>3.5</v>
       </c>
-      <c r="I42" s="43" t="s">
+      <c r="I42" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="J42" s="42">
+      <c r="J42" s="41">
         <v>3</v>
       </c>
-      <c r="K42" s="44" t="s">
+      <c r="K42" s="43" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2362,31 +2460,31 @@
         <f>B10</f>
         <v>0.5</v>
       </c>
-      <c r="C43" s="23" t="s">
+      <c r="C43" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D43" s="56">
+      <c r="D43" s="55">
         <v>0.5</v>
       </c>
-      <c r="E43" s="23" t="s">
+      <c r="E43" s="22" t="s">
         <v>4</v>
       </c>
       <c r="F43" s="8">
         <v>5</v>
       </c>
-      <c r="G43" s="23" t="s">
+      <c r="G43" s="22" t="s">
         <v>4</v>
       </c>
       <c r="H43" s="8">
         <v>5</v>
       </c>
-      <c r="I43" s="23" t="s">
+      <c r="I43" s="22" t="s">
         <v>4</v>
       </c>
       <c r="J43" s="8">
         <v>2.75</v>
       </c>
-      <c r="K43" s="24" t="s">
+      <c r="K43" s="23" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2394,593 +2492,592 @@
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B44" s="25">
+      <c r="B44" s="24">
         <f>B41^2/B43</f>
         <v>50</v>
       </c>
-      <c r="C44" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="D44" s="25">
+      <c r="C44" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="D44" s="24">
         <f>D41^2/D43</f>
         <v>50</v>
       </c>
-      <c r="E44" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="F44" s="25">
+      <c r="E44" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="F44" s="24">
         <f>F41^2/F43</f>
         <v>5</v>
       </c>
-      <c r="G44" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="H44" s="25">
+      <c r="G44" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="H44" s="24">
         <f>H41^2/H43</f>
         <v>5</v>
       </c>
-      <c r="I44" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="J44" s="25">
+      <c r="I44" s="22" t="s">
+        <v>110</v>
+      </c>
+      <c r="J44" s="24">
         <f>J41^2/J43</f>
         <v>9.0909090909090917</v>
       </c>
-      <c r="K44" s="23" t="s">
-        <v>111</v>
+      <c r="K44" s="22" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B45" s="101">
+      <c r="B45" s="100">
         <f>1-(B42/B41)</f>
         <v>0.5</v>
       </c>
-      <c r="C45" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="D45" s="101">
+      <c r="C45" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="D45" s="100">
         <f>1-(D42/D41)</f>
         <v>0.30000000000000004</v>
       </c>
-      <c r="E45" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="F45" s="101">
+      <c r="E45" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="F45" s="100">
         <f>1-(F42/F41)</f>
         <v>0.5</v>
       </c>
-      <c r="G45" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="H45" s="101">
+      <c r="G45" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="H45" s="100">
         <f>1-(H42/H41)</f>
         <v>0.30000000000000004</v>
       </c>
-      <c r="I45" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="J45" s="101">
+      <c r="I45" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="J45" s="100">
         <f>1-(J42/J41)</f>
         <v>0.4</v>
       </c>
-      <c r="K45" s="23" t="s">
-        <v>112</v>
+      <c r="K45" s="22" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" s="39" t="s">
-        <v>47</v>
-      </c>
-      <c r="B46" s="103">
+      <c r="A46" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="B46" s="102">
         <f>B43/B42</f>
         <v>0.2</v>
       </c>
-      <c r="C46" s="103" t="s">
-        <v>113</v>
-      </c>
-      <c r="D46" s="103">
+      <c r="C46" s="102" t="s">
+        <v>112</v>
+      </c>
+      <c r="D46" s="102">
         <f>D43/D42</f>
         <v>0.14285714285714285</v>
       </c>
-      <c r="E46" s="103" t="s">
-        <v>113</v>
-      </c>
-      <c r="F46" s="103">
+      <c r="E46" s="102" t="s">
+        <v>112</v>
+      </c>
+      <c r="F46" s="102">
         <f>F43/F42</f>
         <v>2</v>
       </c>
-      <c r="G46" s="103" t="s">
-        <v>113</v>
-      </c>
-      <c r="H46" s="103">
+      <c r="G46" s="102" t="s">
+        <v>112</v>
+      </c>
+      <c r="H46" s="102">
         <f>H43/H42</f>
         <v>1.4285714285714286</v>
       </c>
-      <c r="I46" s="103" t="s">
-        <v>113</v>
-      </c>
-      <c r="J46" s="103">
+      <c r="I46" s="102" t="s">
+        <v>112</v>
+      </c>
+      <c r="J46" s="102">
         <f>J43/J42</f>
         <v>0.91666666666666663</v>
       </c>
-      <c r="K46" s="23" t="s">
-        <v>113</v>
+      <c r="K46" s="22" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" s="39" t="s">
-        <v>46</v>
-      </c>
-      <c r="B47" s="103">
+      <c r="A47" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="B47" s="102">
         <f>B42*B45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.26595744680851069</v>
       </c>
-      <c r="C47" s="103" t="s">
-        <v>114</v>
-      </c>
-      <c r="D47" s="103">
+      <c r="C47" s="102" t="s">
+        <v>113</v>
+      </c>
+      <c r="D47" s="102">
         <f>D42*D45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.22340425531914904</v>
       </c>
-      <c r="E47" s="103" t="s">
-        <v>114</v>
-      </c>
-      <c r="F47" s="103">
+      <c r="E47" s="102" t="s">
+        <v>113</v>
+      </c>
+      <c r="F47" s="102">
         <f>F42*F45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.26595744680851069</v>
       </c>
-      <c r="G47" s="103" t="s">
-        <v>114</v>
-      </c>
-      <c r="H47" s="103">
+      <c r="G47" s="102" t="s">
+        <v>113</v>
+      </c>
+      <c r="H47" s="102">
         <f>H42*H45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.22340425531914904</v>
       </c>
-      <c r="I47" s="103" t="s">
-        <v>114</v>
-      </c>
-      <c r="J47" s="103">
+      <c r="I47" s="102" t="s">
+        <v>113</v>
+      </c>
+      <c r="J47" s="102">
         <f>J42*J45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.2553191489361703</v>
       </c>
-      <c r="K47" s="23" t="s">
-        <v>114</v>
+      <c r="K47" s="22" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B48" s="102" t="str">
+      <c r="B48" s="101" t="str">
         <f>IF(B46&gt;=B47/2,"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="C48" s="23"/>
-      <c r="D48" s="26" t="str">
+      <c r="C48" s="22"/>
+      <c r="D48" s="25" t="str">
         <f>IF(D46&gt;=D47/2,"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="E48" s="23"/>
-      <c r="F48" s="26" t="str">
+      <c r="E48" s="22"/>
+      <c r="F48" s="25" t="str">
         <f>IF(F46&gt;=F47/2,"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="G48" s="23"/>
-      <c r="H48" s="26" t="str">
+      <c r="G48" s="22"/>
+      <c r="H48" s="25" t="str">
         <f>IF(H46&gt;=H47/2,"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="I48" s="23"/>
-      <c r="J48" s="26" t="str">
+      <c r="I48" s="22"/>
+      <c r="J48" s="25" t="str">
         <f>IF(J46&gt;=J47/2,"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="K48" s="24"/>
+      <c r="K48" s="23"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B49" s="103">
+        <v>48</v>
+      </c>
+      <c r="B49" s="102">
         <f>B46+(B47/2)</f>
         <v>0.33297872340425538</v>
       </c>
-      <c r="C49" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="D49" s="103">
+      <c r="C49" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="D49" s="102">
         <f>D46+(D47/2)</f>
         <v>0.25455927051671734</v>
       </c>
-      <c r="E49" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="F49" s="103">
+      <c r="E49" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="F49" s="102">
         <f>F46+(F47/2)</f>
         <v>2.1329787234042552</v>
       </c>
-      <c r="G49" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="H49" s="103">
+      <c r="G49" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="H49" s="102">
         <f>H46+(H47/2)</f>
         <v>1.540273556231003</v>
       </c>
-      <c r="I49" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="J49" s="103">
+      <c r="I49" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="J49" s="102">
         <f>J46+(J47/2)</f>
         <v>1.0443262411347518</v>
       </c>
-      <c r="K49" s="23" t="s">
-        <v>115</v>
+      <c r="K49" s="22" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="B50" s="103">
+        <v>157</v>
+      </c>
+      <c r="B50" s="102">
         <f>B46-(B47/2)</f>
         <v>6.7021276595744667E-2</v>
       </c>
-      <c r="C50" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D50" s="103">
+      <c r="C50" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="D50" s="102">
         <f>D46-(D47/2)</f>
         <v>3.1155015197568331E-2</v>
       </c>
-      <c r="E50" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="F50" s="103">
+      <c r="E50" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="F50" s="102">
         <f>F46-(F47/2)</f>
         <v>1.8670212765957446</v>
       </c>
-      <c r="G50" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="H50" s="103">
+      <c r="G50" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="H50" s="102">
         <f>H46-(H47/2)</f>
         <v>1.3168693009118542</v>
       </c>
-      <c r="I50" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="J50" s="103">
+      <c r="I50" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="J50" s="102">
         <f>J46-(J47/2)</f>
         <v>0.78900709219858145</v>
       </c>
-      <c r="K50" s="23" t="s">
-        <v>43</v>
+      <c r="K50" s="22" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B51" s="103">
+        <v>47</v>
+      </c>
+      <c r="B51" s="102">
         <f>SQRT(B46^2 + (B47^2/12))</f>
         <v>0.21422989277738178</v>
       </c>
-      <c r="C51" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="D51" s="103">
+      <c r="C51" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="D51" s="102">
         <f>SQRT(D46^2 + (D47^2/12))</f>
         <v>0.15673954523305453</v>
       </c>
-      <c r="E51" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="F51" s="103">
+      <c r="E51" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="F51" s="102">
         <f>SQRT(F46^2 + (F47^2/12))</f>
         <v>2.0014730692565936</v>
       </c>
-      <c r="G51" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="H51" s="103">
+      <c r="G51" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="H51" s="102">
         <f>SQRT(H46^2 + (H47^2/12))</f>
         <v>1.4300263802829551</v>
       </c>
-      <c r="I51" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="J51" s="103">
+      <c r="I51" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="J51" s="102">
         <f>SQRT(J46^2 + (J47^2/12))</f>
         <v>0.91962497796415288</v>
       </c>
-      <c r="K51" s="23" t="s">
-        <v>116</v>
+      <c r="K51" s="22" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A52" s="28" t="s">
-        <v>50</v>
-      </c>
-      <c r="B52" s="104">
+      <c r="A52" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="B52" s="103">
         <f>B41/B44</f>
         <v>0.1</v>
       </c>
-      <c r="C52" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="D52" s="104">
+      <c r="C52" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="D52" s="103">
         <f>D41/D44</f>
         <v>0.1</v>
       </c>
-      <c r="E52" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="F52" s="104">
+      <c r="E52" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="F52" s="103">
         <f>F41/F44</f>
         <v>1</v>
       </c>
-      <c r="G52" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="H52" s="104">
+      <c r="G52" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="H52" s="103">
         <f>H41/H44</f>
         <v>1</v>
       </c>
-      <c r="I52" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="J52" s="104">
+      <c r="I52" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="J52" s="103">
         <f>J41/J44</f>
         <v>0.54999999999999993</v>
       </c>
-      <c r="K52" s="23" t="s">
-        <v>117</v>
+      <c r="K52" s="22" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A53" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="B53" s="104">
+      <c r="A53" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B53" s="103">
         <f>B51*SQRT(B45)</f>
         <v>0.15148340991575365</v>
       </c>
-      <c r="C53" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="D53" s="104">
+      <c r="C53" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="D53" s="103">
         <f>D51*SQRT(D45)</f>
         <v>8.5849784577245306E-2</v>
       </c>
-      <c r="E53" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="F53" s="104">
+      <c r="E53" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="F53" s="103">
         <f>F51*SQRT(F45)</f>
         <v>1.4152551796335899</v>
       </c>
-      <c r="G53" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="H53" s="104">
+      <c r="G53" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="H53" s="103">
         <f>H51*SQRT(H45)</f>
         <v>0.7832577063084355</v>
       </c>
-      <c r="I53" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="J53" s="104">
+      <c r="I53" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="J53" s="103">
         <f>J51*SQRT(J45)</f>
         <v>0.58162190470977582</v>
       </c>
-      <c r="K53" s="23" t="s">
-        <v>118</v>
+      <c r="K53" s="22" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A54" s="28" t="s">
-        <v>51</v>
-      </c>
-      <c r="B54" s="104">
+      <c r="A54" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="B54" s="103">
         <f>SQRT(B46^2*B45*(1-B45) + (B47^2/12)*(1-B45))</f>
         <v>0.11378586678363989</v>
       </c>
-      <c r="C54" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="D54" s="104">
+      <c r="C54" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="D54" s="103">
         <f t="shared" ref="D54:J54" si="0">SQRT(D46^2*D45*(1-D45) + (D47^2/12)*(1-D45))</f>
         <v>8.4835720825047062E-2</v>
       </c>
-      <c r="E54" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="F54" s="104">
+      <c r="E54" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="F54" s="103">
         <f t="shared" si="0"/>
         <v>1.0014725275711283</v>
       </c>
-      <c r="G54" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="H54" s="104">
+      <c r="G54" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="H54" s="103">
         <f t="shared" si="0"/>
         <v>0.65687351431886776</v>
       </c>
-      <c r="I54" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="J54" s="104">
+      <c r="I54" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="J54" s="103">
         <f t="shared" si="0"/>
         <v>0.45268759653578</v>
       </c>
-      <c r="K54" s="23" t="s">
-        <v>119</v>
+      <c r="K54" s="22" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B55" s="28">
+        <v>5</v>
+      </c>
+      <c r="C55" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="D55" s="28">
+        <v>5</v>
+      </c>
+      <c r="E55" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="F55" s="28">
+        <v>5</v>
+      </c>
+      <c r="G55" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="H55" s="28">
+        <v>5</v>
+      </c>
+      <c r="I55" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="J55" s="28">
+        <v>5</v>
+      </c>
+      <c r="K55" s="22" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="B55" s="29">
+      <c r="B56" s="106">
         <v>5</v>
       </c>
-      <c r="C55" s="23" t="s">
+      <c r="C56" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="D55" s="29">
+      <c r="D56" s="106">
         <v>5</v>
       </c>
-      <c r="E55" s="23" t="s">
+      <c r="E56" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="F55" s="29">
+      <c r="F56" s="106">
         <v>5</v>
       </c>
-      <c r="G55" s="23" t="s">
+      <c r="G56" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="H55" s="29">
+      <c r="H56" s="106">
         <v>5</v>
       </c>
-      <c r="I55" s="23" t="s">
+      <c r="I56" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="J55" s="29">
+      <c r="J56" s="106">
         <v>5</v>
       </c>
-      <c r="K55" s="23" t="s">
+      <c r="K56" s="22" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A56" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="B56" s="107">
-        <v>5</v>
-      </c>
-      <c r="C56" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="D56" s="107">
-        <v>5</v>
-      </c>
-      <c r="E56" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="F56" s="107">
-        <v>5</v>
-      </c>
-      <c r="G56" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="H56" s="107">
-        <v>5</v>
-      </c>
-      <c r="I56" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="J56" s="107">
-        <v>5</v>
-      </c>
-      <c r="K56" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="L56" s="106" t="s">
+      <c r="L56" s="105" t="s">
+        <v>158</v>
+      </c>
+      <c r="M56" t="s">
         <v>159</v>
       </c>
-      <c r="M56" t="s">
+      <c r="N56" t="s">
         <v>160</v>
-      </c>
-      <c r="N56" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="57" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B57" s="105">
+        <v>54</v>
+      </c>
+      <c r="B57" s="104">
         <f>10^3*B52*B45/($B$35*10^-6*$B$11*10^3)</f>
-        <v>7.3529411764705888</v>
-      </c>
-      <c r="C57" s="31" t="s">
-        <v>122</v>
-      </c>
-      <c r="D57" s="105">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C57" s="30" t="s">
+        <v>121</v>
+      </c>
+      <c r="D57" s="104">
         <f>10^3*D52*D45/($B$35*10^-6*$B$11*10^3)</f>
-        <v>4.4117647058823533</v>
-      </c>
-      <c r="E57" s="31" t="s">
-        <v>122</v>
-      </c>
-      <c r="F57" s="105">
+        <v>0.2</v>
+      </c>
+      <c r="E57" s="30" t="s">
+        <v>121</v>
+      </c>
+      <c r="F57" s="104">
         <f>10^3*F52*F45/($B$35*10^-6*$B$11*10^3)</f>
-        <v>73.529411764705884</v>
-      </c>
-      <c r="G57" s="31" t="s">
-        <v>122</v>
-      </c>
-      <c r="H57" s="105">
+        <v>3.3333333333333335</v>
+      </c>
+      <c r="G57" s="30" t="s">
+        <v>121</v>
+      </c>
+      <c r="H57" s="104">
         <f>10^3*H52*H45/($B$35*10^-6*$B$11*10^3)</f>
-        <v>44.117647058823536</v>
-      </c>
-      <c r="I57" s="31" t="s">
-        <v>122</v>
-      </c>
-      <c r="J57" s="105">
+        <v>2.0000000000000004</v>
+      </c>
+      <c r="I57" s="30" t="s">
+        <v>121</v>
+      </c>
+      <c r="J57" s="104">
         <f>10^3*J52*J45/($B$35*10^-6*$B$11*10^3)</f>
-        <v>32.352941176470587</v>
-      </c>
-      <c r="K57" s="31" t="s">
-        <v>122</v>
+        <v>1.4666666666666666</v>
+      </c>
+      <c r="K57" s="30" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="58" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="33"/>
-      <c r="C58" s="34"/>
+      <c r="B58" s="32"/>
+      <c r="C58" s="33"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B59" s="33"/>
-      <c r="C59" s="34"/>
+      <c r="B59" s="32"/>
+      <c r="C59" s="33"/>
     </row>
     <row r="60" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="1:14" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="3" t="s">
+    <row r="62" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="115" t="s">
         <v>0</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="B62" s="115" t="s">
         <v>1</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="115" t="s">
         <v>7</v>
       </c>
-      <c r="D62" s="3" t="s">
+      <c r="D62" s="115" t="s">
         <v>1</v>
       </c>
-      <c r="E62" s="3" t="s">
+      <c r="E62" s="115" t="s">
         <v>7</v>
       </c>
-      <c r="F62" s="3"/>
-      <c r="G62" s="3"/>
-      <c r="H62" s="3" t="s">
+      <c r="F62" s="115"/>
+      <c r="G62" s="115"/>
+      <c r="H62" s="115" t="s">
         <v>1</v>
       </c>
-      <c r="I62" s="3" t="s">
+      <c r="I62" s="115" t="s">
         <v>7</v>
       </c>
-      <c r="J62" s="3" t="s">
+      <c r="J62" s="115" t="s">
         <v>1</v>
       </c>
-      <c r="K62" s="3" t="s">
+      <c r="K62" s="115" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2992,35 +3089,35 @@
         <f>B44</f>
         <v>50</v>
       </c>
-      <c r="C63" s="23" t="s">
+      <c r="C63" s="22" t="s">
         <v>20</v>
       </c>
       <c r="D63" s="8">
         <f>D44</f>
         <v>50</v>
       </c>
-      <c r="E63" s="23" t="s">
+      <c r="E63" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F63" s="8">
         <f>F44</f>
         <v>5</v>
       </c>
-      <c r="G63" s="23" t="s">
+      <c r="G63" s="22" t="s">
         <v>20</v>
       </c>
       <c r="H63" s="8">
         <f>H44</f>
         <v>5</v>
       </c>
-      <c r="I63" s="23" t="s">
+      <c r="I63" s="22" t="s">
         <v>20</v>
       </c>
       <c r="J63" s="8">
         <f>J44</f>
         <v>9.0909090909090917</v>
       </c>
-      <c r="K63" s="24" t="s">
+      <c r="K63" s="23" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3032,95 +3129,95 @@
         <f>B45</f>
         <v>0.5</v>
       </c>
-      <c r="C64" s="23"/>
+      <c r="C64" s="22"/>
       <c r="D64" s="8">
         <f>D45</f>
         <v>0.30000000000000004</v>
       </c>
-      <c r="E64" s="23"/>
+      <c r="E64" s="22"/>
       <c r="F64" s="8">
         <f>F45</f>
         <v>0.5</v>
       </c>
-      <c r="G64" s="23"/>
+      <c r="G64" s="22"/>
       <c r="H64" s="8">
         <f>H45</f>
         <v>0.30000000000000004</v>
       </c>
-      <c r="I64" s="23"/>
+      <c r="I64" s="22"/>
       <c r="J64" s="8">
         <f>J45</f>
         <v>0.4</v>
       </c>
-      <c r="K64" s="24"/>
+      <c r="K64" s="23"/>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A65" s="39" t="s">
-        <v>164</v>
-      </c>
-      <c r="B65" s="103">
+      <c r="A65" s="38" t="s">
+        <v>162</v>
+      </c>
+      <c r="B65" s="102">
         <v>4.9983700000000004</v>
       </c>
-      <c r="C65" s="23" t="s">
+      <c r="C65" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D65" s="103">
+      <c r="D65" s="102">
         <v>4.9908000000000001</v>
       </c>
-      <c r="E65" s="23" t="s">
+      <c r="E65" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="F65" s="108">
+      <c r="F65" s="107">
         <v>4.9982800000000003</v>
       </c>
-      <c r="G65" s="23" t="s">
+      <c r="G65" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="H65" s="103">
+      <c r="H65" s="102">
         <v>4.9980099999999998</v>
       </c>
-      <c r="I65" s="23" t="s">
+      <c r="I65" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="J65" s="103">
+      <c r="J65" s="102">
         <v>4.9981</v>
       </c>
-      <c r="K65" s="24" t="s">
+      <c r="K65" s="23" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A66" s="39" t="s">
-        <v>165</v>
-      </c>
-      <c r="B66" s="103">
+      <c r="A66" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="B66" s="102">
         <v>0.49967400000000001</v>
       </c>
-      <c r="C66" s="23" t="s">
+      <c r="C66" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D66" s="103">
+      <c r="D66" s="102">
         <v>0.49961699999999998</v>
       </c>
-      <c r="E66" s="23" t="s">
+      <c r="E66" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="F66" s="103">
+      <c r="F66" s="102">
         <v>4.9968300000000001</v>
       </c>
-      <c r="G66" s="23" t="s">
+      <c r="G66" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="H66" s="103">
+      <c r="H66" s="102">
         <v>4.9961099999999998</v>
       </c>
-      <c r="I66" s="23" t="s">
+      <c r="I66" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="J66" s="103">
+      <c r="J66" s="102">
         <v>2.7482099999999998</v>
       </c>
-      <c r="K66" s="24" t="s">
+      <c r="K66" s="23" t="s">
         <v>4</v>
       </c>
     </row>
@@ -3128,352 +3225,352 @@
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B67" s="27" t="s">
-        <v>163</v>
-      </c>
-      <c r="C67" s="23"/>
-      <c r="D67" s="108" t="s">
-        <v>163</v>
-      </c>
-      <c r="E67" s="23"/>
-      <c r="F67" s="108" t="s">
-        <v>163</v>
-      </c>
-      <c r="G67" s="23"/>
-      <c r="H67" s="108" t="s">
-        <v>163</v>
-      </c>
-      <c r="I67" s="23"/>
-      <c r="J67" s="108" t="s">
-        <v>163</v>
-      </c>
-      <c r="K67" s="24"/>
+      <c r="B67" s="26" t="s">
+        <v>161</v>
+      </c>
+      <c r="C67" s="22"/>
+      <c r="D67" s="107" t="s">
+        <v>161</v>
+      </c>
+      <c r="E67" s="22"/>
+      <c r="F67" s="107" t="s">
+        <v>161</v>
+      </c>
+      <c r="G67" s="22"/>
+      <c r="H67" s="107" t="s">
+        <v>161</v>
+      </c>
+      <c r="I67" s="22"/>
+      <c r="J67" s="107" t="s">
+        <v>161</v>
+      </c>
+      <c r="K67" s="23"/>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A68" s="39" t="s">
-        <v>46</v>
-      </c>
-      <c r="B68" s="108">
+      <c r="A68" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="B68" s="107">
         <f>0.332881-0.0669235</f>
         <v>0.26595749999999996</v>
       </c>
-      <c r="C68" s="23" t="s">
+      <c r="C68" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D68" s="108">
+      <c r="D68" s="107">
         <f>0.254488-0.0310839</f>
         <v>0.22340409999999999</v>
       </c>
-      <c r="E68" s="23" t="s">
+      <c r="E68" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F68" s="103">
+      <c r="F68" s="102">
         <f>2.13197-1.86601</f>
         <v>0.26595999999999997</v>
       </c>
-      <c r="G68" s="23" t="s">
+      <c r="G68" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H68" s="108">
+      <c r="H68" s="107">
         <f>1.53955-1.31615</f>
         <v>0.22340000000000004</v>
       </c>
-      <c r="I68" s="23" t="s">
+      <c r="I68" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="J68" s="108">
+      <c r="J68" s="107">
         <f>1.04393-0.788614</f>
         <v>0.25531599999999999</v>
       </c>
-      <c r="K68" s="23" t="s">
+      <c r="K68" s="22" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B69" s="103">
+        <v>48</v>
+      </c>
+      <c r="B69" s="102">
         <v>0.33288099999999998</v>
       </c>
-      <c r="C69" s="23" t="s">
+      <c r="C69" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D69" s="103">
+      <c r="D69" s="102">
         <v>0.25448799999999999</v>
       </c>
-      <c r="E69" s="23" t="s">
+      <c r="E69" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F69" s="103">
+      <c r="F69" s="102">
         <v>2.1319699999999999</v>
       </c>
-      <c r="G69" s="23" t="s">
+      <c r="G69" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H69" s="103">
+      <c r="H69" s="102">
         <v>1.53955</v>
       </c>
-      <c r="I69" s="23" t="s">
+      <c r="I69" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="J69" s="103">
+      <c r="J69" s="102">
         <v>1.04393</v>
       </c>
-      <c r="K69" s="23" t="s">
+      <c r="K69" s="22" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B70" s="103">
+        <v>47</v>
+      </c>
+      <c r="B70" s="102">
         <v>0.214139</v>
       </c>
-      <c r="C70" s="23" t="s">
+      <c r="C70" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D70" s="103">
+      <c r="D70" s="102">
         <v>0.15667500000000001</v>
       </c>
-      <c r="E70" s="23" t="s">
+      <c r="E70" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F70" s="103">
+      <c r="F70" s="102">
         <v>2.0004599999999999</v>
       </c>
-      <c r="G70" s="23" t="s">
+      <c r="G70" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H70" s="103">
+      <c r="H70" s="102">
         <f>1.42931</f>
         <v>1.4293100000000001</v>
       </c>
-      <c r="I70" s="23" t="s">
+      <c r="I70" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="J70" s="103">
+      <c r="J70" s="102">
         <v>0.91923299999999997</v>
       </c>
-      <c r="K70" s="23" t="s">
+      <c r="K70" s="22" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A71" s="28" t="s">
+      <c r="A71" s="27" t="s">
+        <v>49</v>
+      </c>
+      <c r="B71" s="116">
+        <v>9.9967399999999998E-2</v>
+      </c>
+      <c r="C71" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="D71" s="103">
+        <v>9.9942699999999995E-2</v>
+      </c>
+      <c r="E71" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="F71" s="102">
+        <v>0.99965599999999999</v>
+      </c>
+      <c r="G71" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="H71" s="103">
+        <v>0.99960099999999996</v>
+      </c>
+      <c r="I71" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="J71" s="103">
+        <v>0.54984599999999995</v>
+      </c>
+      <c r="K71" s="22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A72" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="B72" s="103">
+        <v>0.151419</v>
+      </c>
+      <c r="C72" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="D72" s="103">
+        <v>8.5814299999999996E-2</v>
+      </c>
+      <c r="E72" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="F72" s="116">
+        <v>1.4145399999999999</v>
+      </c>
+      <c r="G72" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="H72" s="103">
+        <v>0.78286299999999998</v>
+      </c>
+      <c r="I72" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="J72" s="103">
+        <v>0.58137399999999995</v>
+      </c>
+      <c r="K72" s="22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="B71" s="109">
-        <v>9.9967399999999998E-2</v>
-      </c>
-      <c r="C71" s="23" t="s">
+      <c r="B73" s="103">
+        <v>0.113757</v>
+      </c>
+      <c r="C73" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D71" s="104">
-        <v>9.9942699999999995E-2</v>
-      </c>
-      <c r="E71" s="23" t="s">
+      <c r="D73" s="103">
+        <v>8.4824099999999999E-2</v>
+      </c>
+      <c r="E73" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F71" s="103">
-        <v>0.99965599999999999</v>
-      </c>
-      <c r="G71" s="23" t="s">
+      <c r="F73" s="103">
+        <v>1.0011399999999999</v>
+      </c>
+      <c r="G73" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H71" s="104">
-        <v>0.99960099999999996</v>
-      </c>
-      <c r="I71" s="23" t="s">
+      <c r="H73" s="103">
+        <v>0.65672399999999997</v>
+      </c>
+      <c r="I73" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="J71" s="104">
-        <v>0.54984599999999995</v>
-      </c>
-      <c r="K71" s="23" t="s">
+      <c r="J73" s="103">
+        <v>0.452598</v>
+      </c>
+      <c r="K73" s="22" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A72" s="28" t="s">
-        <v>52</v>
-      </c>
-      <c r="B72" s="104">
-        <v>0.151419</v>
-      </c>
-      <c r="C72" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D72" s="104">
-        <v>8.5814299999999996E-2</v>
-      </c>
-      <c r="E72" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="F72" s="109">
-        <v>1.4145399999999999</v>
-      </c>
-      <c r="G72" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="H72" s="104">
-        <v>0.78286299999999998</v>
-      </c>
-      <c r="I72" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="J72" s="104">
-        <v>0.58137399999999995</v>
-      </c>
-      <c r="K72" s="23" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A73" s="28" t="s">
-        <v>51</v>
-      </c>
-      <c r="B73" s="104">
-        <v>0.113757</v>
-      </c>
-      <c r="C73" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D73" s="104">
-        <v>8.4824099999999999E-2</v>
-      </c>
-      <c r="E73" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="F73" s="104">
-        <v>1.0011399999999999</v>
-      </c>
-      <c r="G73" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="H73" s="104">
-        <v>0.65672399999999997</v>
-      </c>
-      <c r="I73" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="J73" s="104">
-        <v>0.452598</v>
-      </c>
-      <c r="K73" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="L73" s="110"/>
+      <c r="L73" s="108"/>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B74" s="103">
+        <v>5.00204</v>
+      </c>
+      <c r="C74" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D74" s="103">
+        <v>5.0002899999999997</v>
+      </c>
+      <c r="E74" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F74" s="103">
+        <v>5.0350299999999999</v>
+      </c>
+      <c r="G74" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="H74" s="103">
+        <v>5.02006</v>
+      </c>
+      <c r="I74" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="J74" s="103">
+        <v>5.0142699999999998</v>
+      </c>
+      <c r="K74" s="22" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="B74" s="104">
+      <c r="B75" s="103">
         <v>5.00204</v>
       </c>
-      <c r="C74" s="23" t="s">
+      <c r="C75" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="D74" s="104">
+      <c r="D75" s="103">
         <v>5.0002899999999997</v>
       </c>
-      <c r="E74" s="23" t="s">
+      <c r="E75" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="F74" s="104">
+      <c r="F75" s="103">
         <v>5.0350299999999999</v>
       </c>
-      <c r="G74" s="23" t="s">
+      <c r="G75" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="H74" s="104">
+      <c r="H75" s="103">
         <v>5.02006</v>
       </c>
-      <c r="I74" s="23" t="s">
+      <c r="I75" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="J74" s="104">
+      <c r="J75" s="103">
         <v>5.0142699999999998</v>
       </c>
-      <c r="K74" s="23" t="s">
+      <c r="K75" s="29" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A75" s="28" t="s">
+    <row r="76" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="117" t="s">
         <v>54</v>
       </c>
-      <c r="B75" s="104">
-        <v>5.00204</v>
-      </c>
-      <c r="C75" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="D75" s="104">
-        <v>5.0002899999999997</v>
-      </c>
-      <c r="E75" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="F75" s="104">
-        <v>5.0350299999999999</v>
-      </c>
-      <c r="G75" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="H75" s="104">
-        <v>5.02006</v>
-      </c>
-      <c r="I75" s="30" t="s">
-        <v>3</v>
-      </c>
-      <c r="J75" s="104">
-        <v>5.0142699999999998</v>
-      </c>
-      <c r="K75" s="30" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="76" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B76" s="105">
+      <c r="B76" s="118">
         <f>(5.00204-4.99469)*10^3</f>
         <v>7.3499999999997456</v>
       </c>
-      <c r="C76" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="D76" s="105">
+      <c r="C76" s="114" t="s">
+        <v>164</v>
+      </c>
+      <c r="D76" s="118">
         <f>(5.00029 - 4.99588)*10^3</f>
         <v>4.410000000000025</v>
       </c>
-      <c r="E76" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="F76" s="105">
+      <c r="E76" s="114" t="s">
+        <v>164</v>
+      </c>
+      <c r="F76" s="118">
         <f>(5.03503-4.96153)*10^3</f>
         <v>73.500000000000114</v>
       </c>
-      <c r="G76" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="H76" s="105">
+      <c r="G76" s="114" t="s">
+        <v>164</v>
+      </c>
+      <c r="H76" s="118">
         <f>(5.02006-4.97596)*10^3</f>
         <v>44.10000000000025</v>
       </c>
-      <c r="I76" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="J76" s="105">
+      <c r="I76" s="114" t="s">
+        <v>164</v>
+      </c>
+      <c r="J76" s="118">
         <f>(5.01427-4.98192)*10^3</f>
         <v>32.350000000000101</v>
       </c>
-      <c r="K76" s="31" t="s">
-        <v>166</v>
+      <c r="K76" s="114" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="77" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -3496,7 +3593,7 @@
     </row>
     <row r="82" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B82" s="5">
         <v>1</v>
@@ -3507,9 +3604,9 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="B83" s="35">
+        <v>125</v>
+      </c>
+      <c r="B83" s="34">
         <v>4</v>
       </c>
       <c r="C83" s="17" t="s">
@@ -3520,18 +3617,18 @@
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B84" s="35">
+      <c r="B84" s="34">
         <v>2.5</v>
       </c>
-      <c r="C84" s="36" t="s">
+      <c r="C84" s="35" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A85" s="53" t="s">
-        <v>131</v>
-      </c>
-      <c r="B85" s="37">
+      <c r="A85" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="B85" s="36">
         <v>22</v>
       </c>
       <c r="C85" s="18" t="s">
@@ -3539,10 +3636,10 @@
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A86" s="53" t="s">
-        <v>130</v>
-      </c>
-      <c r="B86" s="35">
+      <c r="A86" s="52" t="s">
+        <v>129</v>
+      </c>
+      <c r="B86" s="34">
         <v>1</v>
       </c>
       <c r="C86" s="18" t="s">
@@ -3550,8 +3647,8 @@
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87" s="53" t="s">
-        <v>129</v>
+      <c r="A87" s="52" t="s">
+        <v>128</v>
       </c>
       <c r="B87" s="16">
         <v>18</v>
@@ -3561,87 +3658,87 @@
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A88" s="53" t="s">
-        <v>128</v>
+      <c r="A88" s="52" t="s">
+        <v>127</v>
       </c>
       <c r="B88" s="16">
         <v>0.22</v>
       </c>
       <c r="C88" s="18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A89" s="53" t="s">
-        <v>132</v>
+      <c r="A89" s="52" t="s">
+        <v>131</v>
       </c>
       <c r="B89" s="16">
         <v>10</v>
       </c>
       <c r="C89" s="18" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A90" s="53" t="s">
-        <v>133</v>
+      <c r="A90" s="52" t="s">
+        <v>132</v>
       </c>
       <c r="B90" s="16">
         <v>68</v>
       </c>
       <c r="C90" s="18" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A91" s="53" t="s">
-        <v>134</v>
+      <c r="A91" s="52" t="s">
+        <v>133</v>
       </c>
       <c r="B91" s="16">
         <v>220</v>
       </c>
       <c r="C91" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="B92" s="16">
+        <v>22</v>
+      </c>
+      <c r="C92" s="18" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A92" s="53" t="s">
-        <v>27</v>
-      </c>
-      <c r="B92" s="16">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="B93" s="16">
         <v>12</v>
       </c>
-      <c r="C92" s="18" t="s">
+      <c r="C93" s="18" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A93" s="53" t="s">
-        <v>28</v>
-      </c>
-      <c r="B93" s="16">
-        <v>22</v>
-      </c>
-      <c r="C93" s="18" t="s">
-        <v>140</v>
-      </c>
-    </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A94" s="53" t="s">
-        <v>127</v>
+      <c r="A94" s="52" t="s">
+        <v>126</v>
       </c>
       <c r="B94" s="16">
         <v>2200</v>
       </c>
       <c r="C94" s="18" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="B95" s="35">
+        <v>122</v>
+      </c>
+      <c r="B95" s="34">
         <v>4.7</v>
       </c>
       <c r="C95" s="18" t="s">
@@ -3650,9 +3747,9 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="B96" s="35">
+        <v>123</v>
+      </c>
+      <c r="B96" s="34">
         <v>10</v>
       </c>
       <c r="C96" s="18" t="s">
@@ -3663,8 +3760,8 @@
       <c r="A97" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B97" s="111">
-        <v>0.1</v>
+      <c r="B97" s="110">
+        <v>5</v>
       </c>
       <c r="C97" s="18"/>
     </row>
@@ -3672,8 +3769,8 @@
       <c r="A98" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B98" s="20" t="s">
-        <v>162</v>
+      <c r="B98" s="111">
+        <v>1000</v>
       </c>
       <c r="C98" s="19"/>
     </row>
@@ -3723,35 +3820,35 @@
         <f>B44</f>
         <v>50</v>
       </c>
-      <c r="C104" s="23" t="s">
+      <c r="C104" s="22" t="s">
         <v>20</v>
       </c>
       <c r="D104" s="8">
         <f>D44</f>
         <v>50</v>
       </c>
-      <c r="E104" s="23" t="s">
+      <c r="E104" s="22" t="s">
         <v>20</v>
       </c>
       <c r="F104" s="8">
         <f>F44</f>
         <v>5</v>
       </c>
-      <c r="G104" s="23" t="s">
+      <c r="G104" s="22" t="s">
         <v>20</v>
       </c>
       <c r="H104" s="8">
         <f>H44</f>
         <v>5</v>
       </c>
-      <c r="I104" s="23" t="s">
+      <c r="I104" s="22" t="s">
         <v>20</v>
       </c>
       <c r="J104" s="8">
         <f>J44</f>
         <v>9.0909090909090917</v>
       </c>
-      <c r="K104" s="24" t="s">
+      <c r="K104" s="23" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3762,88 +3859,109 @@
       <c r="B105" s="8">
         <v>2.5</v>
       </c>
-      <c r="C105" s="23" t="s">
+      <c r="C105" s="22" t="s">
         <v>3</v>
       </c>
       <c r="D105" s="8">
         <v>3.5</v>
       </c>
-      <c r="E105" s="23" t="s">
+      <c r="E105" s="22" t="s">
         <v>3</v>
       </c>
       <c r="F105" s="8">
         <v>2.5</v>
       </c>
-      <c r="G105" s="23" t="s">
+      <c r="G105" s="22" t="s">
         <v>3</v>
       </c>
       <c r="H105" s="8">
         <v>3.5</v>
       </c>
-      <c r="I105" s="23" t="s">
+      <c r="I105" s="22" t="s">
         <v>3</v>
       </c>
       <c r="J105" s="8">
         <v>3</v>
       </c>
-      <c r="K105" s="24" t="s">
+      <c r="K105" s="23" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A106" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B106" s="25"/>
-      <c r="C106" s="23" t="s">
+      <c r="A106" s="38" t="s">
+        <v>165</v>
+      </c>
+      <c r="B106" s="102">
+        <v>4.9581299999999997</v>
+      </c>
+      <c r="C106" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D106" s="25"/>
-      <c r="E106" s="23" t="s">
+      <c r="D106" s="102">
+        <v>4.9572399999999996</v>
+      </c>
+      <c r="E106" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="F106" s="23"/>
-      <c r="G106" s="23" t="s">
+      <c r="F106" s="102">
+        <v>4.9486999999999997</v>
+      </c>
+      <c r="G106" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="H106" s="25"/>
-      <c r="I106" s="23" t="s">
+      <c r="H106" s="102">
+        <v>4.9558900000000001</v>
+      </c>
+      <c r="I106" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="J106" s="25"/>
-      <c r="K106" s="24" t="s">
+      <c r="J106" s="24">
+        <v>4.9549200000000004</v>
+      </c>
+      <c r="K106" s="23" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B107" s="109">
+        <v>12.7</v>
+      </c>
+      <c r="C107" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="B107" s="20"/>
-      <c r="C107" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="D107" s="20"/>
-      <c r="E107" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="F107" s="31"/>
-      <c r="G107" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="H107" s="20"/>
-      <c r="I107" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="J107" s="20"/>
-      <c r="K107" s="32" t="s">
-        <v>36</v>
+      <c r="D107" s="109">
+        <v>29.2</v>
+      </c>
+      <c r="E107" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="F107" s="112">
+        <v>16.3</v>
+      </c>
+      <c r="G107" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="H107" s="109">
+        <v>3.6</v>
+      </c>
+      <c r="I107" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="J107" s="113">
+        <v>10.3</v>
+      </c>
+      <c r="K107" s="31" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3858,12 +3976,12 @@
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -3879,8 +3997,8 @@
       </c>
     </row>
     <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="38" t="s">
-        <v>104</v>
+      <c r="A6" s="37" t="s">
+        <v>103</v>
       </c>
       <c r="B6" s="5">
         <f>SS_Analysis!B25</f>
@@ -3891,50 +4009,50 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="39" t="s">
-        <v>94</v>
+      <c r="A7" s="38" t="s">
+        <v>93</v>
       </c>
       <c r="B7" s="8">
         <f>SS_Analysis!H46</f>
         <v>1.4285714285714286</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="39" t="s">
-        <v>95</v>
+      <c r="A8" s="38" t="s">
+        <v>94</v>
       </c>
       <c r="B8" s="8">
         <f>SS_Analysis!H49</f>
         <v>1.540273556231003</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="39" t="s">
-        <v>93</v>
+      <c r="A9" s="38" t="s">
+        <v>92</v>
       </c>
       <c r="B9" s="8">
         <f>SS_Analysis!H51</f>
         <v>1.4300263802829551</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B10" s="8">
         <v>0.25</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3954,7 +4072,7 @@
     </row>
     <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -3972,106 +4090,106 @@
       </c>
     </row>
     <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="60" t="s">
+      <c r="A17" s="59" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="60" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="61" t="s">
+      <c r="C17" s="61"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="62"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="63" t="s">
+      <c r="B18" s="63" t="s">
         <v>68</v>
       </c>
-      <c r="B18" s="64" t="s">
+      <c r="C18" s="64"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="65"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="63" t="s">
+      <c r="B19" s="65"/>
+      <c r="C19" s="64" t="s">
         <v>70</v>
       </c>
-      <c r="B19" s="66"/>
-      <c r="C19" s="65" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="63" t="s">
+      <c r="B20" s="65"/>
+      <c r="C20" s="64" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="66"/>
-      <c r="C20" s="65" t="s">
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="63" t="s">
+      <c r="B21" s="65"/>
+      <c r="C21" s="64" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="66"/>
-      <c r="C21" s="65" t="s">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="63" t="s">
+      <c r="B22" s="65"/>
+      <c r="C22" s="64" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="66"/>
-      <c r="C22" s="65" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="63" t="s">
+      <c r="B23" s="65"/>
+      <c r="C23" s="64" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="66"/>
-      <c r="C23" s="65" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="63" t="s">
+      <c r="B24" s="66"/>
+      <c r="C24" s="64" t="s">
         <v>78</v>
       </c>
-      <c r="B24" s="67"/>
-      <c r="C24" s="65" t="s">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="63" t="s">
+      <c r="B25" s="66"/>
+      <c r="C25" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="B25" s="67"/>
-      <c r="C25" s="65" t="s">
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="68" t="s">
+      <c r="B26" s="68"/>
+      <c r="C26" s="64"/>
+    </row>
+    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="B26" s="69"/>
-      <c r="C26" s="65"/>
-    </row>
-    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="70" t="s">
-        <v>83</v>
-      </c>
-      <c r="B27" s="71">
+      <c r="B27" s="70">
         <v>0.65</v>
       </c>
-      <c r="C27" s="72"/>
+      <c r="C27" s="71"/>
     </row>
     <row r="28" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="30" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -4087,113 +4205,113 @@
       </c>
     </row>
     <row r="33" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="60" t="s">
+      <c r="A33" s="59" t="s">
+        <v>84</v>
+      </c>
+      <c r="B33" s="72">
+        <v>0.1</v>
+      </c>
+      <c r="C33" s="73" t="s">
+        <v>142</v>
+      </c>
+      <c r="G33" s="74"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="75" t="s">
         <v>85</v>
       </c>
-      <c r="B33" s="73">
-        <v>0.1</v>
-      </c>
-      <c r="C33" s="74" t="s">
+      <c r="B34" s="76"/>
+      <c r="C34" s="77" t="s">
         <v>143</v>
       </c>
-      <c r="G33" s="75"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="76" t="s">
+      <c r="G34" s="74"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="75" t="s">
         <v>86</v>
       </c>
-      <c r="B34" s="77"/>
-      <c r="C34" s="78" t="s">
+      <c r="B35" s="78"/>
+      <c r="C35" s="77" t="s">
         <v>144</v>
       </c>
-      <c r="G34" s="75"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="76" t="s">
+      <c r="F35" s="79"/>
+      <c r="G35" s="74"/>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="75" t="s">
         <v>87</v>
       </c>
-      <c r="B35" s="79"/>
-      <c r="C35" s="78" t="s">
-        <v>145</v>
-      </c>
-      <c r="F35" s="80"/>
-      <c r="G35" s="75"/>
-    </row>
-    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="76" t="s">
-        <v>88</v>
-      </c>
-      <c r="B36" s="81" t="str">
+      <c r="B36" s="80" t="str">
         <f>IF(B35&lt;=B10,"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="C36" s="78"/>
+      <c r="C36" s="77"/>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="76" t="s">
+      <c r="A37" s="75" t="s">
+        <v>88</v>
+      </c>
+      <c r="B37" s="76"/>
+      <c r="C37" s="77" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="82" t="s">
+        <v>96</v>
+      </c>
+      <c r="B38" s="81">
+        <v>0.5</v>
+      </c>
+      <c r="C38" s="77" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="82" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="76"/>
+      <c r="C39" s="77" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="82" t="s">
+        <v>97</v>
+      </c>
+      <c r="B40" s="81">
+        <v>5</v>
+      </c>
+      <c r="C40" s="77"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="82" t="s">
+        <v>98</v>
+      </c>
+      <c r="B41" s="76"/>
+      <c r="C41" s="77" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="84" t="s">
         <v>89</v>
       </c>
-      <c r="B37" s="77"/>
-      <c r="C37" s="78" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="83" t="s">
-        <v>97</v>
-      </c>
-      <c r="B38" s="82">
-        <v>0.5</v>
-      </c>
-      <c r="C38" s="78" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="83" t="s">
-        <v>96</v>
-      </c>
-      <c r="B39" s="77"/>
-      <c r="C39" s="78" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="83" t="s">
-        <v>98</v>
-      </c>
-      <c r="B40" s="82">
-        <v>5</v>
-      </c>
-      <c r="C40" s="78"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="83" t="s">
-        <v>99</v>
-      </c>
-      <c r="B41" s="77"/>
-      <c r="C41" s="78" t="s">
+      <c r="B42" s="85"/>
+      <c r="C42" s="86" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="85" t="s">
-        <v>90</v>
-      </c>
-      <c r="B42" s="86"/>
-      <c r="C42" s="87" t="s">
-        <v>149</v>
-      </c>
-    </row>
     <row r="43" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="75"/>
+      <c r="B43" s="74"/>
     </row>
     <row r="45" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -4209,39 +4327,39 @@
       </c>
     </row>
     <row r="48" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="83" t="s">
+      <c r="A48" s="82" t="s">
+        <v>100</v>
+      </c>
+      <c r="B48" s="76"/>
+      <c r="C48" s="77" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="75" t="s">
+        <v>86</v>
+      </c>
+      <c r="B49" s="90"/>
+      <c r="C49" s="64" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="82" t="s">
+        <v>149</v>
+      </c>
+      <c r="B50" s="90"/>
+      <c r="C50" s="64" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="83" t="s">
         <v>101</v>
       </c>
-      <c r="B48" s="77"/>
-      <c r="C48" s="78" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="76" t="s">
-        <v>87</v>
-      </c>
-      <c r="B49" s="91"/>
-      <c r="C49" s="65" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="83" t="s">
-        <v>150</v>
-      </c>
-      <c r="B50" s="91"/>
-      <c r="C50" s="65" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="84" t="s">
+      <c r="B51" s="88"/>
+      <c r="C51" s="89" t="s">
         <v>102</v>
-      </c>
-      <c r="B51" s="89"/>
-      <c r="C51" s="90" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Updated boost converter parameters. Simulated with closed loop control. Improved output.
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/wwei275_uoa_auckland_ac_nz/Documents/Documents/GitHub/311/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69A63D3B-2827-4D8F-A7BD-6B49D3215CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="141" documentId="13_ncr:1_{AA8CBFA0-FA2E-463F-95BC-A72C55469A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{668C1007-B3FE-4D6F-9FD9-2255C3B87768}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -30,15 +30,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="169">
   <si>
     <t>Parameter</t>
   </si>
@@ -536,6 +533,15 @@
   </si>
   <si>
     <t>Steady State Vout (avg)</t>
+  </si>
+  <si>
+    <t>Rv</t>
+  </si>
+  <si>
+    <t>Rc2</t>
+  </si>
+  <si>
+    <t>pF</t>
   </si>
 </sst>
 </file>
@@ -550,7 +556,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1650,11 +1656,11 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="60" xfId="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="61" xfId="2" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
@@ -1662,7 +1668,7 @@
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Per cent" xfId="3" builtinId="5"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1688,7 +1694,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>189547</xdr:colOff>
+      <xdr:colOff>184785</xdr:colOff>
       <xdr:row>97</xdr:row>
       <xdr:rowOff>116205</xdr:rowOff>
     </xdr:to>
@@ -2043,27 +2049,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
-  <dimension ref="A1:N108"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
+  <dimension ref="A1:N110"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.4375" customWidth="1"/>
+    <col min="1" max="1" width="20.375" customWidth="1"/>
     <col min="2" max="11" width="12.875" customWidth="1"/>
-    <col min="12" max="12" width="17.4375" customWidth="1"/>
+    <col min="12" max="12" width="17.375" customWidth="1"/>
     <col min="13" max="13" width="18.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.65">
+    <row r="1" spans="1:3" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.649999999999999">
+    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -2074,7 +2080,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="13.9" thickTop="1">
+    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A6" s="37" t="s">
         <v>36</v>
       </c>
@@ -2085,7 +2091,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="38" t="s">
         <v>37</v>
       </c>
@@ -2096,7 +2102,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
         <v>38</v>
       </c>
@@ -2107,7 +2113,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="38" t="s">
         <v>56</v>
       </c>
@@ -2118,7 +2124,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="38" t="s">
         <v>57</v>
       </c>
@@ -2129,7 +2135,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.9" thickBot="1">
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -2140,16 +2146,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.4" thickTop="1">
+    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="17.649999999999999">
+    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -2160,7 +2166,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="13.9" thickTop="1">
+    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A17" s="45" t="s">
         <v>41</v>
       </c>
@@ -2172,7 +2178,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="47" t="s">
         <v>40</v>
       </c>
@@ -2184,7 +2190,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="56" t="s">
         <v>59</v>
       </c>
@@ -2196,7 +2202,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="49" t="s">
         <v>60</v>
       </c>
@@ -2208,7 +2214,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="52" t="s">
         <v>43</v>
       </c>
@@ -2220,7 +2226,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="52" t="s">
         <v>150</v>
       </c>
@@ -2232,7 +2238,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="52" t="s">
         <v>44</v>
       </c>
@@ -2244,7 +2250,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="95" t="s">
         <v>151</v>
       </c>
@@ -2256,7 +2262,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="13.9" thickBot="1">
+    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="87" t="s">
         <v>103</v>
       </c>
@@ -2267,14 +2273,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="13.9" thickTop="1"/>
-    <row r="28" spans="1:3" ht="17.649999999999999">
+    <row r="26" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="30" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="29" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>0</v>
       </c>
@@ -2285,7 +2291,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="13.9" thickTop="1">
+    <row r="31" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -2296,7 +2302,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="97" t="s">
         <v>152</v>
       </c>
@@ -2308,7 +2314,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -2320,7 +2326,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="27" t="s">
         <v>153</v>
       </c>
@@ -2332,25 +2338,25 @@
         <v>109</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="13.9" thickBot="1">
+    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B35" s="11">
-        <v>220</v>
+      <c r="B35" s="96">
+        <v>560</v>
       </c>
       <c r="C35" s="19" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="38" spans="1:11" ht="17.649999999999999">
+    <row r="36" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="1:11" ht="18" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="40" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
+    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>0</v>
       </c>
@@ -2385,7 +2391,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="13.9" thickTop="1">
+    <row r="41" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -2420,7 +2426,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="44" t="s">
         <v>39</v>
       </c>
@@ -2455,7 +2461,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -2491,7 +2497,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -2531,7 +2537,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="45" spans="1:11">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
@@ -2571,7 +2577,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="38" t="s">
         <v>46</v>
       </c>
@@ -2611,7 +2617,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="47" spans="1:11">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" s="38" t="s">
         <v>45</v>
       </c>
@@ -2651,7 +2657,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="48" spans="1:11">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
@@ -2681,7 +2687,7 @@
       </c>
       <c r="K48" s="23"/>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
         <v>48</v>
       </c>
@@ -2721,7 +2727,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
         <v>157</v>
       </c>
@@ -2761,7 +2767,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
         <v>47</v>
       </c>
@@ -2801,7 +2807,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="27" t="s">
         <v>49</v>
       </c>
@@ -2841,7 +2847,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="27" t="s">
         <v>51</v>
       </c>
@@ -2881,7 +2887,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" s="27" t="s">
         <v>50</v>
       </c>
@@ -2921,7 +2927,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
         <v>52</v>
       </c>
@@ -2956,7 +2962,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
@@ -3000,60 +3006,60 @@
         <v>160</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="13.9" thickBot="1">
+    <row r="57" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>54</v>
       </c>
       <c r="B57" s="104">
         <f>10^3*B52*B45/($B$35*10^-6*$B$11*10^3)</f>
-        <v>2.2727272727272729</v>
+        <v>0.89285714285714302</v>
       </c>
       <c r="C57" s="30" t="s">
         <v>121</v>
       </c>
       <c r="D57" s="104">
         <f>10^3*D52*D45/($B$35*10^-6*$B$11*10^3)</f>
-        <v>1.3636363636363638</v>
+        <v>0.53571428571428581</v>
       </c>
       <c r="E57" s="30" t="s">
         <v>121</v>
       </c>
       <c r="F57" s="104">
         <f>10^3*F52*F45/($B$35*10^-6*$B$11*10^3)</f>
-        <v>22.727272727272727</v>
+        <v>8.9285714285714288</v>
       </c>
       <c r="G57" s="30" t="s">
         <v>121</v>
       </c>
       <c r="H57" s="104">
         <f>10^3*H52*H45/($B$35*10^-6*$B$11*10^3)</f>
-        <v>13.636363636363638</v>
+        <v>5.3571428571428585</v>
       </c>
       <c r="I57" s="30" t="s">
         <v>121</v>
       </c>
       <c r="J57" s="104">
         <f>10^3*J52*J45/($B$35*10^-6*$B$11*10^3)</f>
-        <v>9.9999999999999982</v>
+        <v>3.9285714285714284</v>
       </c>
       <c r="K57" s="30" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="13.9" thickTop="1">
+    <row r="58" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B58" s="32"/>
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B59" s="32"/>
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="1:14" ht="17.649999999999999">
+    <row r="60" spans="1:14" ht="18" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="14.25" thickBot="1">
+    <row r="62" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="115" t="s">
         <v>0</v>
       </c>
@@ -3084,7 +3090,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="13.9" thickTop="1">
+    <row r="63" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -3124,7 +3130,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -3154,7 +3160,7 @@
       </c>
       <c r="K64" s="23"/>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A65" s="38" t="s">
         <v>162</v>
       </c>
@@ -3189,7 +3195,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A66" s="38" t="s">
         <v>163</v>
       </c>
@@ -3224,7 +3230,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:12">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
@@ -3249,7 +3255,7 @@
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:12">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A68" s="38" t="s">
         <v>45</v>
       </c>
@@ -3289,7 +3295,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
         <v>48</v>
       </c>
@@ -3324,7 +3330,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
@@ -3360,7 +3366,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:12">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A71" s="27" t="s">
         <v>49</v>
       </c>
@@ -3395,7 +3401,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:12">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" s="27" t="s">
         <v>51</v>
       </c>
@@ -3430,7 +3436,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
@@ -3466,7 +3472,7 @@
       </c>
       <c r="L73" s="108"/>
     </row>
-    <row r="74" spans="1:12">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
         <v>52</v>
       </c>
@@ -3501,7 +3507,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
@@ -3536,7 +3542,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="13.9" thickBot="1">
+    <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A76" s="117" t="s">
         <v>54</v>
       </c>
@@ -3576,14 +3582,14 @@
         <v>164</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="13.9" thickTop="1"/>
-    <row r="79" spans="1:12" ht="17.649999999999999">
+    <row r="77" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="79" spans="1:12" ht="18" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="13.9" thickBot="1"/>
-    <row r="81" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="80" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
@@ -3594,7 +3600,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="13.9" thickTop="1">
+    <row r="82" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
         <v>124</v>
       </c>
@@ -3605,7 +3611,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" s="15" t="s">
         <v>125</v>
       </c>
@@ -3616,7 +3622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -3627,7 +3633,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15">
+    <row r="85" spans="1:3" ht="15" x14ac:dyDescent="0.2">
       <c r="A85" s="52" t="s">
         <v>130</v>
       </c>
@@ -3638,7 +3644,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" s="52" t="s">
         <v>129</v>
       </c>
@@ -3649,7 +3655,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" s="52" t="s">
         <v>128</v>
       </c>
@@ -3660,7 +3666,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="52" t="s">
         <v>127</v>
       </c>
@@ -3671,276 +3677,317 @@
         <v>134</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="52" t="s">
+        <v>166</v>
+      </c>
+      <c r="B89" s="16">
+        <v>0.22</v>
+      </c>
+      <c r="C89" s="18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90" s="52" t="s">
         <v>131</v>
       </c>
-      <c r="B89" s="16">
+      <c r="B90" s="16">
+        <v>47</v>
+      </c>
+      <c r="C90" s="18" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91" s="52" t="s">
+        <v>132</v>
+      </c>
+      <c r="B91" s="16">
+        <v>100</v>
+      </c>
+      <c r="C91" s="18" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A92" s="52" t="s">
+        <v>133</v>
+      </c>
+      <c r="B92" s="16">
+        <v>1500</v>
+      </c>
+      <c r="C92" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="B93" s="16">
+        <v>100</v>
+      </c>
+      <c r="C93" s="18" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A94" s="52" t="s">
+        <v>28</v>
+      </c>
+      <c r="B94" s="16">
+        <v>100</v>
+      </c>
+      <c r="C94" s="18" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95" s="52" t="s">
+        <v>126</v>
+      </c>
+      <c r="B95" s="16">
+        <v>3300</v>
+      </c>
+      <c r="C95" s="18" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A96" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="B96" s="34">
         <v>4.7</v>
-      </c>
-      <c r="C89" s="18" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3">
-      <c r="A90" s="52" t="s">
-        <v>132</v>
-      </c>
-      <c r="B90" s="16">
-        <v>10</v>
-      </c>
-      <c r="C90" s="18" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3">
-      <c r="A91" s="52" t="s">
-        <v>133</v>
-      </c>
-      <c r="B91" s="16">
-        <v>1500</v>
-      </c>
-      <c r="C91" s="18" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3">
-      <c r="A92" s="52" t="s">
-        <v>27</v>
-      </c>
-      <c r="B92" s="16">
-        <v>22</v>
-      </c>
-      <c r="C92" s="18" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3">
-      <c r="A93" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="B93" s="16">
-        <v>12</v>
-      </c>
-      <c r="C93" s="18" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3">
-      <c r="A94" s="52" t="s">
-        <v>126</v>
-      </c>
-      <c r="B94" s="16">
-        <v>2200</v>
-      </c>
-      <c r="C94" s="18" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3">
-      <c r="A95" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="B95" s="34">
-        <v>4.7</v>
-      </c>
-      <c r="C95" s="18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3">
-      <c r="A96" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="B96" s="34">
-        <v>10</v>
       </c>
       <c r="C96" s="18" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="B97" s="34">
+        <v>10</v>
+      </c>
+      <c r="C97" s="18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A98" s="52" t="s">
+        <v>167</v>
+      </c>
+      <c r="B98" s="34">
+        <v>150</v>
+      </c>
+      <c r="C98" s="18" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A99" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B97" s="110">
+      <c r="B99" s="110">
+        <v>5</v>
+      </c>
+      <c r="C99" s="18"/>
+    </row>
+    <row r="100" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B100" s="111">
+        <v>1000</v>
+      </c>
+      <c r="C100" s="19"/>
+    </row>
+    <row r="101" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="103" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A103" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B105" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C97" s="18"/>
-    </row>
-    <row r="98" spans="1:11" ht="13.9" thickBot="1">
-      <c r="A98" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B98" s="111">
-        <v>500</v>
-      </c>
-      <c r="C98" s="19"/>
-    </row>
-    <row r="99" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="101" spans="1:11" ht="17.649999999999999">
-      <c r="A101" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="102" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="103" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
-      <c r="A103" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B103" s="3" t="s">
+      <c r="C105" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D105" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C103" s="3" t="s">
+      <c r="E105" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D103" s="3" t="s">
+      <c r="F105" s="3"/>
+      <c r="G105" s="3"/>
+      <c r="H105" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E103" s="3" t="s">
+      <c r="I105" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F103" s="3"/>
-      <c r="G103" s="3"/>
-      <c r="H103" s="3" t="s">
+      <c r="J105" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="I103" s="3" t="s">
+      <c r="K105" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J103" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="K103" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11" ht="13.9" thickTop="1">
-      <c r="A104" s="7" t="s">
+    </row>
+    <row r="106" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A106" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B104" s="8">
+      <c r="B106" s="8">
         <f>B44</f>
         <v>50</v>
       </c>
-      <c r="C104" s="22" t="s">
+      <c r="C106" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="D104" s="8">
+      <c r="D106" s="8">
         <f>D44</f>
         <v>50</v>
       </c>
-      <c r="E104" s="22" t="s">
+      <c r="E106" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="F104" s="8">
+      <c r="F106" s="8">
         <f>F44</f>
         <v>5</v>
       </c>
-      <c r="G104" s="22" t="s">
+      <c r="G106" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="H104" s="8">
+      <c r="H106" s="8">
         <f>H44</f>
         <v>5</v>
       </c>
-      <c r="I104" s="22" t="s">
+      <c r="I106" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="J104" s="8">
-        <f>J44</f>
-        <v>9.0909090909090917</v>
-      </c>
-      <c r="K104" s="23" t="s">
+      <c r="J106" s="8">
+        <v>10</v>
+      </c>
+      <c r="K106" s="23" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="105" spans="1:11">
-      <c r="A105" s="7" t="s">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A107" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B105" s="8">
+      <c r="B107" s="8">
         <v>2.5</v>
       </c>
-      <c r="C105" s="22" t="s">
+      <c r="C107" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D105" s="8">
+      <c r="D107" s="8">
         <v>3.5</v>
       </c>
-      <c r="E105" s="22" t="s">
+      <c r="E107" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="F105" s="8">
+      <c r="F107" s="8">
         <v>2.5</v>
       </c>
-      <c r="G105" s="22" t="s">
+      <c r="G107" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="H105" s="8">
+      <c r="H107" s="8">
         <v>3.5</v>
       </c>
-      <c r="I105" s="22" t="s">
+      <c r="I107" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="J105" s="8">
+      <c r="J107" s="8">
         <v>3</v>
       </c>
-      <c r="K105" s="23" t="s">
+      <c r="K107" s="23" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="1:11">
-      <c r="A106" s="38" t="s">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A108" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="B106" s="102"/>
-      <c r="C106" s="22" t="s">
+      <c r="B108" s="102">
+        <v>4.9987000000000004</v>
+      </c>
+      <c r="C108" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D106" s="102"/>
-      <c r="E106" s="22" t="s">
+      <c r="D108" s="102">
+        <v>4.9998500000000003</v>
+      </c>
+      <c r="E108" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="F106" s="102"/>
-      <c r="G106" s="22" t="s">
+      <c r="F108" s="102">
+        <v>4.9988000000000001</v>
+      </c>
+      <c r="G108" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="H106" s="102"/>
-      <c r="I106" s="22" t="s">
+      <c r="H108" s="102">
+        <v>4.9996700000000001</v>
+      </c>
+      <c r="I108" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="J106" s="24"/>
-      <c r="K106" s="23" t="s">
+      <c r="J108" s="102">
+        <v>4.9985900000000001</v>
+      </c>
+      <c r="K108" s="23" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:11" ht="13.9" thickBot="1">
-      <c r="A107" s="10" t="s">
+    <row r="109" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A109" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B107" s="109"/>
-      <c r="C107" s="30" t="s">
+      <c r="B109" s="109">
+        <v>8.9</v>
+      </c>
+      <c r="C109" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="D107" s="109"/>
-      <c r="E107" s="30" t="s">
+      <c r="D109" s="109">
+        <v>7.7</v>
+      </c>
+      <c r="E109" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="F107" s="112"/>
-      <c r="G107" s="30" t="s">
+      <c r="F109" s="112">
+        <v>12.2</v>
+      </c>
+      <c r="G109" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="H107" s="109"/>
-      <c r="I107" s="30" t="s">
+      <c r="H109" s="109">
+        <v>1.2</v>
+      </c>
+      <c r="I109" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="J107" s="113"/>
-      <c r="K107" s="31" t="s">
+      <c r="J109" s="113">
+        <v>4.8</v>
+      </c>
+      <c r="K109" s="31" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="108" spans="1:11" ht="13.9" thickTop="1"/>
+    <row r="110" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3951,24 +3998,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.4375" customWidth="1"/>
+    <col min="1" max="1" width="24.375" customWidth="1"/>
     <col min="2" max="9" width="12.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.65">
+    <row r="1" spans="1:3" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.649999999999999">
+    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -3979,7 +4026,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="13.9" thickTop="1">
+    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A6" s="37" t="s">
         <v>103</v>
       </c>
@@ -3991,7 +4038,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="38" t="s">
         <v>93</v>
       </c>
@@ -4003,7 +4050,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
         <v>94</v>
       </c>
@@ -4015,7 +4062,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="38" t="s">
         <v>92</v>
       </c>
@@ -4027,7 +4074,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -4038,7 +4085,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.9" thickBot="1">
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -4050,18 +4097,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.4" thickTop="1">
+    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="17.649999999999999">
+    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18" thickBot="1">
+    <row r="15" spans="1:3" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -4072,7 +4119,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="13.9" thickTop="1">
+    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A17" s="59" t="s">
         <v>65</v>
       </c>
@@ -4081,7 +4128,7 @@
       </c>
       <c r="C17" s="61"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
@@ -4090,7 +4137,7 @@
       </c>
       <c r="C18" s="64"/>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
@@ -4099,7 +4146,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
@@ -4108,7 +4155,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
@@ -4117,7 +4164,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
@@ -4126,7 +4173,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
@@ -4135,7 +4182,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
@@ -4144,7 +4191,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
@@ -4153,14 +4200,14 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
       <c r="B26" s="68"/>
       <c r="C26" s="64"/>
     </row>
-    <row r="27" spans="1:3" ht="13.9" thickBot="1">
+    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="69" t="s">
         <v>82</v>
       </c>
@@ -4169,14 +4216,14 @@
       </c>
       <c r="C27" s="71"/>
     </row>
-    <row r="28" spans="1:3" ht="13.9" thickTop="1"/>
-    <row r="30" spans="1:3" ht="17.649999999999999">
+    <row r="28" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="32" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="31" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -4187,7 +4234,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="13.9" thickTop="1">
+    <row r="33" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A33" s="59" t="s">
         <v>84</v>
       </c>
@@ -4199,7 +4246,7 @@
       </c>
       <c r="G33" s="74"/>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="75" t="s">
         <v>85</v>
       </c>
@@ -4209,7 +4256,7 @@
       </c>
       <c r="G34" s="74"/>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="75" t="s">
         <v>86</v>
       </c>
@@ -4220,7 +4267,7 @@
       <c r="F35" s="79"/>
       <c r="G35" s="74"/>
     </row>
-    <row r="36" spans="1:7" ht="15">
+    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="75" t="s">
         <v>87</v>
       </c>
@@ -4233,7 +4280,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="75" t="s">
         <v>88</v>
       </c>
@@ -4242,7 +4289,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="82" t="s">
         <v>96</v>
       </c>
@@ -4253,7 +4300,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="82" t="s">
         <v>95</v>
       </c>
@@ -4262,7 +4309,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="82" t="s">
         <v>97</v>
       </c>
@@ -4271,7 +4318,7 @@
       </c>
       <c r="C40" s="77"/>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="82" t="s">
         <v>98</v>
       </c>
@@ -4280,7 +4327,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="13.9" thickBot="1">
+    <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="84" t="s">
         <v>89</v>
       </c>
@@ -4289,16 +4336,16 @@
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="13.9" thickTop="1">
+    <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B43" s="74"/>
     </row>
-    <row r="45" spans="1:7" ht="17.649999999999999">
+    <row r="45" spans="1:7" ht="18" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="13.9" thickBot="1"/>
-    <row r="47" spans="1:7" ht="14.65" thickTop="1" thickBot="1">
+    <row r="46" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>0</v>
       </c>
@@ -4309,7 +4356,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="13.9" thickTop="1">
+    <row r="48" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A48" s="82" t="s">
         <v>100</v>
       </c>
@@ -4318,7 +4365,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="75" t="s">
         <v>86</v>
       </c>
@@ -4327,7 +4374,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="82" t="s">
         <v>149</v>
       </c>
@@ -4336,7 +4383,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="13.9" thickBot="1">
+    <row r="51" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="83" t="s">
         <v>101</v>
       </c>
@@ -4345,7 +4392,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="13.9" thickTop="1"/>
+    <row r="52" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Changed curent sense resistor at output smaller.
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/wwei275_uoa_auckland_ac_nz/Documents/Documents/GitHub/311/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wwei275\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="141" documentId="13_ncr:1_{AA8CBFA0-FA2E-463F-95BC-A72C55469A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{668C1007-B3FE-4D6F-9FD9-2255C3B87768}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D57C3655-3732-451F-A711-849C8939EA28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -1527,7 +1527,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1663,6 +1663,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="61" xfId="2" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -2050,25 +2051,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
   <dimension ref="A1:N110"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.375" customWidth="1"/>
-    <col min="2" max="11" width="12.875" customWidth="1"/>
-    <col min="12" max="12" width="17.375" customWidth="1"/>
-    <col min="13" max="13" width="18.875" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
+    <col min="2" max="11" width="12.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
@@ -2080,7 +2081,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="s">
         <v>36</v>
       </c>
@@ -2091,7 +2092,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
         <v>37</v>
       </c>
@@ -2102,7 +2103,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
         <v>38</v>
       </c>
@@ -2113,7 +2114,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
         <v>56</v>
       </c>
@@ -2124,7 +2125,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
         <v>57</v>
       </c>
@@ -2135,7 +2136,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -2149,12 +2150,12 @@
     <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
@@ -2166,7 +2167,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="45" t="s">
         <v>41</v>
       </c>
@@ -2178,7 +2179,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="47" t="s">
         <v>40</v>
       </c>
@@ -2190,7 +2191,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="56" t="s">
         <v>59</v>
       </c>
@@ -2202,7 +2203,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="49" t="s">
         <v>60</v>
       </c>
@@ -2214,7 +2215,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="52" t="s">
         <v>43</v>
       </c>
@@ -2226,7 +2227,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="52" t="s">
         <v>150</v>
       </c>
@@ -2238,7 +2239,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="52" t="s">
         <v>44</v>
       </c>
@@ -2250,7 +2251,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="95" t="s">
         <v>151</v>
       </c>
@@ -2262,7 +2263,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="87" t="s">
         <v>103</v>
       </c>
@@ -2273,13 +2274,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="28" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="30" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>0</v>
@@ -2291,7 +2292,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -2302,7 +2303,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="97" t="s">
         <v>152</v>
       </c>
@@ -2314,7 +2315,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -2326,7 +2327,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="27" t="s">
         <v>153</v>
       </c>
@@ -2338,7 +2339,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
@@ -2349,13 +2350,13 @@
         <v>109</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="1:11" ht="18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="40" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>0</v>
@@ -2391,7 +2392,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -2426,7 +2427,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="44" t="s">
         <v>39</v>
       </c>
@@ -2461,7 +2462,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -2497,7 +2498,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -2537,7 +2538,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
@@ -2577,7 +2578,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="38" t="s">
         <v>46</v>
       </c>
@@ -2617,7 +2618,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="38" t="s">
         <v>45</v>
       </c>
@@ -2657,7 +2658,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
@@ -2687,7 +2688,7 @@
       </c>
       <c r="K48" s="23"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>48</v>
       </c>
@@ -2727,7 +2728,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>157</v>
       </c>
@@ -2767,7 +2768,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>47</v>
       </c>
@@ -2807,7 +2808,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="27" t="s">
         <v>49</v>
       </c>
@@ -2847,7 +2848,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="27" t="s">
         <v>51</v>
       </c>
@@ -2887,7 +2888,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>50</v>
       </c>
@@ -2927,7 +2928,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>52</v>
       </c>
@@ -2962,7 +2963,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
@@ -3006,7 +3007,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="10" t="s">
         <v>54</v>
       </c>
@@ -3046,15 +3047,15 @@
         <v>121</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B58" s="32"/>
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B59" s="32"/>
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="1:14" ht="18" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
@@ -3090,7 +3091,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -3130,7 +3131,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -3160,7 +3161,7 @@
       </c>
       <c r="K64" s="23"/>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="38" t="s">
         <v>162</v>
       </c>
@@ -3195,7 +3196,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="38" t="s">
         <v>163</v>
       </c>
@@ -3230,7 +3231,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
@@ -3255,7 +3256,7 @@
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" s="38" t="s">
         <v>45</v>
       </c>
@@ -3295,7 +3296,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>48</v>
       </c>
@@ -3330,7 +3331,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
@@ -3366,7 +3367,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" s="27" t="s">
         <v>49</v>
       </c>
@@ -3401,7 +3402,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="27" t="s">
         <v>51</v>
       </c>
@@ -3436,7 +3437,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
@@ -3472,7 +3473,7 @@
       </c>
       <c r="L73" s="108"/>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
         <v>52</v>
       </c>
@@ -3507,7 +3508,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
@@ -3542,7 +3543,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="117" t="s">
         <v>54</v>
       </c>
@@ -3582,13 +3583,13 @@
         <v>164</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="79" spans="1:12" ht="18" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="81" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
         <v>0</v>
@@ -3600,7 +3601,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
         <v>124</v>
       </c>
@@ -3611,7 +3612,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
         <v>125</v>
       </c>
@@ -3622,7 +3623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -3633,7 +3634,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="52" t="s">
         <v>130</v>
       </c>
@@ -3644,7 +3645,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="52" t="s">
         <v>129</v>
       </c>
@@ -3655,7 +3656,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="52" t="s">
         <v>128</v>
       </c>
@@ -3666,7 +3667,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="52" t="s">
         <v>127</v>
       </c>
@@ -3677,18 +3678,18 @@
         <v>134</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="52" t="s">
         <v>166</v>
       </c>
-      <c r="B89" s="16">
-        <v>0.22</v>
+      <c r="B89" s="119">
+        <v>4.7E-2</v>
       </c>
       <c r="C89" s="18" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="52" t="s">
         <v>131</v>
       </c>
@@ -3699,7 +3700,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="52" t="s">
         <v>132</v>
       </c>
@@ -3710,7 +3711,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="52" t="s">
         <v>133</v>
       </c>
@@ -3721,7 +3722,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="52" t="s">
         <v>27</v>
       </c>
@@ -3732,7 +3733,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="52" t="s">
         <v>28</v>
       </c>
@@ -3743,7 +3744,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="52" t="s">
         <v>126</v>
       </c>
@@ -3754,7 +3755,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="15" t="s">
         <v>122</v>
       </c>
@@ -3765,7 +3766,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97" s="15" t="s">
         <v>123</v>
       </c>
@@ -3776,7 +3777,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" s="52" t="s">
         <v>167</v>
       </c>
@@ -3787,7 +3788,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99" s="15" t="s">
         <v>30</v>
       </c>
@@ -3796,7 +3797,7 @@
       </c>
       <c r="C99" s="18"/>
     </row>
-    <row r="100" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="10" t="s">
         <v>31</v>
       </c>
@@ -3805,13 +3806,13 @@
       </c>
       <c r="C100" s="19"/>
     </row>
-    <row r="101" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="101" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="103" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="104" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="105" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="3" t="s">
         <v>0</v>
@@ -3843,7 +3844,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="106" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A106" s="7" t="s">
         <v>16</v>
       </c>
@@ -3882,7 +3883,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107" s="7" t="s">
         <v>33</v>
       </c>
@@ -3917,7 +3918,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108" s="38" t="s">
         <v>165</v>
       </c>
@@ -3952,7 +3953,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A109" s="10" t="s">
         <v>34</v>
       </c>
@@ -3987,7 +3988,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="110" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="110" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3998,23 +3999,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.375" customWidth="1"/>
-    <col min="2" max="9" width="12.875" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="2" max="9" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
@@ -4026,7 +4027,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="s">
         <v>103</v>
       </c>
@@ -4038,7 +4039,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
         <v>93</v>
       </c>
@@ -4050,7 +4051,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
         <v>94</v>
       </c>
@@ -4062,7 +4063,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
         <v>92</v>
       </c>
@@ -4074,7 +4075,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -4085,7 +4086,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -4100,12 +4101,12 @@
     <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
     </row>
     <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4119,7 +4120,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="59" t="s">
         <v>65</v>
       </c>
@@ -4128,7 +4129,7 @@
       </c>
       <c r="C17" s="61"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
@@ -4137,7 +4138,7 @@
       </c>
       <c r="C18" s="64"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
@@ -4146,7 +4147,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
@@ -4155,7 +4156,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
@@ -4164,7 +4165,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
@@ -4173,7 +4174,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
@@ -4182,7 +4183,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
@@ -4191,7 +4192,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
@@ -4200,14 +4201,14 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
       <c r="B26" s="68"/>
       <c r="C26" s="64"/>
     </row>
-    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="69" t="s">
         <v>82</v>
       </c>
@@ -4216,13 +4217,13 @@
       </c>
       <c r="C27" s="71"/>
     </row>
-    <row r="28" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>0</v>
@@ -4234,7 +4235,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A33" s="59" t="s">
         <v>84</v>
       </c>
@@ -4246,7 +4247,7 @@
       </c>
       <c r="G33" s="74"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="75" t="s">
         <v>85</v>
       </c>
@@ -4256,7 +4257,7 @@
       </c>
       <c r="G34" s="74"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="75" t="s">
         <v>86</v>
       </c>
@@ -4280,7 +4281,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="75" t="s">
         <v>88</v>
       </c>
@@ -4289,7 +4290,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="82" t="s">
         <v>96</v>
       </c>
@@ -4300,7 +4301,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="82" t="s">
         <v>95</v>
       </c>
@@ -4309,7 +4310,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="82" t="s">
         <v>97</v>
       </c>
@@ -4318,7 +4319,7 @@
       </c>
       <c r="C40" s="77"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="82" t="s">
         <v>98</v>
       </c>
@@ -4327,7 +4328,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="84" t="s">
         <v>89</v>
       </c>
@@ -4336,15 +4337,15 @@
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B43" s="74"/>
     </row>
-    <row r="45" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>0</v>
@@ -4356,7 +4357,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A48" s="82" t="s">
         <v>100</v>
       </c>
@@ -4365,7 +4366,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="75" t="s">
         <v>86</v>
       </c>
@@ -4374,7 +4375,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="82" t="s">
         <v>149</v>
       </c>
@@ -4383,7 +4384,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="83" t="s">
         <v>101</v>
       </c>
@@ -4392,7 +4393,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="52" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Using 10V_DC to power OPAMP instead.
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wwei275\Documents\GitHub\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D57C3655-3732-451F-A711-849C8939EA28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BABF3E0-2D4E-41C2-BB41-E755756E6BF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -30,6 +30,9 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -538,10 +541,10 @@
     <t>Rv</t>
   </si>
   <si>
-    <t>Rc2</t>
-  </si>
-  <si>
     <t>pF</t>
+  </si>
+  <si>
+    <t>Cf</t>
   </si>
 </sst>
 </file>
@@ -556,7 +559,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1669,7 +1672,7 @@
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2051,26 +2054,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
   <dimension ref="A1:N110"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" customWidth="1"/>
-    <col min="2" max="11" width="12.85546875" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" customWidth="1"/>
-    <col min="13" max="13" width="18.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.4375" customWidth="1"/>
+    <col min="2" max="11" width="12.875" customWidth="1"/>
+    <col min="12" max="12" width="17.4375" customWidth="1"/>
+    <col min="13" max="13" width="18.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="20.65">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="17.649999999999999">
       <c r="A3" s="2" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -2081,7 +2084,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="13.9" thickTop="1">
       <c r="A6" s="37" t="s">
         <v>36</v>
       </c>
@@ -2092,7 +2095,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" s="38" t="s">
         <v>37</v>
       </c>
@@ -2103,7 +2106,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" s="38" t="s">
         <v>38</v>
       </c>
@@ -2114,7 +2117,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" s="38" t="s">
         <v>56</v>
       </c>
@@ -2125,7 +2128,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" s="38" t="s">
         <v>57</v>
       </c>
@@ -2136,7 +2139,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.9" thickBot="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -2147,16 +2150,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="15.4" thickTop="1">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="17.649999999999999">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -2167,7 +2170,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="13.9" thickTop="1">
       <c r="A17" s="45" t="s">
         <v>41</v>
       </c>
@@ -2179,7 +2182,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18" s="47" t="s">
         <v>40</v>
       </c>
@@ -2191,7 +2194,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19" s="56" t="s">
         <v>59</v>
       </c>
@@ -2203,7 +2206,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3">
       <c r="A20" s="49" t="s">
         <v>60</v>
       </c>
@@ -2215,7 +2218,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3">
       <c r="A21" s="52" t="s">
         <v>43</v>
       </c>
@@ -2227,7 +2230,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3">
       <c r="A22" s="52" t="s">
         <v>150</v>
       </c>
@@ -2239,7 +2242,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3">
       <c r="A23" s="52" t="s">
         <v>44</v>
       </c>
@@ -2251,7 +2254,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3">
       <c r="A24" s="95" t="s">
         <v>151</v>
       </c>
@@ -2263,7 +2266,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="13.9" thickBot="1">
       <c r="A25" s="87" t="s">
         <v>103</v>
       </c>
@@ -2274,14 +2277,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="13.9" thickTop="1"/>
+    <row r="28" spans="1:3" ht="17.649999999999999">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="30" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A30" s="3" t="s">
         <v>0</v>
       </c>
@@ -2292,7 +2295,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="13.9" thickTop="1">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -2303,7 +2306,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3">
       <c r="A32" s="97" t="s">
         <v>152</v>
       </c>
@@ -2315,7 +2318,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -2327,7 +2330,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11">
       <c r="A34" s="27" t="s">
         <v>153</v>
       </c>
@@ -2339,7 +2342,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="13.9" thickBot="1">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
@@ -2350,14 +2353,14 @@
         <v>109</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="13.9" thickTop="1"/>
+    <row r="38" spans="1:11" ht="17.649999999999999">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="40" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="13.9" thickBot="1"/>
+    <row r="40" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
       <c r="A40" s="3" t="s">
         <v>0</v>
       </c>
@@ -2392,7 +2395,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="13.9" thickTop="1">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -2427,7 +2430,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11">
       <c r="A42" s="44" t="s">
         <v>39</v>
       </c>
@@ -2462,7 +2465,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -2498,7 +2501,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -2538,7 +2541,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
@@ -2578,7 +2581,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11">
       <c r="A46" s="38" t="s">
         <v>46</v>
       </c>
@@ -2618,7 +2621,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11">
       <c r="A47" s="38" t="s">
         <v>45</v>
       </c>
@@ -2658,7 +2661,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
@@ -2688,7 +2691,7 @@
       </c>
       <c r="K48" s="23"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14">
       <c r="A49" s="7" t="s">
         <v>48</v>
       </c>
@@ -2728,7 +2731,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14">
       <c r="A50" s="7" t="s">
         <v>157</v>
       </c>
@@ -2768,7 +2771,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14">
       <c r="A51" s="7" t="s">
         <v>47</v>
       </c>
@@ -2808,7 +2811,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14">
       <c r="A52" s="27" t="s">
         <v>49</v>
       </c>
@@ -2848,7 +2851,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14">
       <c r="A53" s="27" t="s">
         <v>51</v>
       </c>
@@ -2888,7 +2891,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14">
       <c r="A54" s="27" t="s">
         <v>50</v>
       </c>
@@ -2928,7 +2931,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14">
       <c r="A55" s="7" t="s">
         <v>52</v>
       </c>
@@ -2963,7 +2966,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14">
       <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
@@ -3007,7 +3010,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" ht="13.9" thickBot="1">
       <c r="A57" s="10" t="s">
         <v>54</v>
       </c>
@@ -3047,20 +3050,20 @@
         <v>121</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="13.9" thickTop="1">
       <c r="B58" s="32"/>
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14">
       <c r="B59" s="32"/>
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:14" ht="17.649999999999999">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:14" ht="14.25" thickBot="1">
       <c r="A62" s="115" t="s">
         <v>0</v>
       </c>
@@ -3091,7 +3094,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" ht="13.9" thickTop="1">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -3131,7 +3134,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -3161,7 +3164,7 @@
       </c>
       <c r="K64" s="23"/>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:12">
       <c r="A65" s="38" t="s">
         <v>162</v>
       </c>
@@ -3196,7 +3199,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:12">
       <c r="A66" s="38" t="s">
         <v>163</v>
       </c>
@@ -3231,7 +3234,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:12">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
@@ -3256,7 +3259,7 @@
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:12">
       <c r="A68" s="38" t="s">
         <v>45</v>
       </c>
@@ -3296,7 +3299,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:12">
       <c r="A69" s="7" t="s">
         <v>48</v>
       </c>
@@ -3331,7 +3334,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:12">
       <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
@@ -3367,7 +3370,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:12">
       <c r="A71" s="27" t="s">
         <v>49</v>
       </c>
@@ -3402,7 +3405,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:12">
       <c r="A72" s="27" t="s">
         <v>51</v>
       </c>
@@ -3437,7 +3440,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:12">
       <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
@@ -3473,7 +3476,7 @@
       </c>
       <c r="L73" s="108"/>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:12">
       <c r="A74" s="7" t="s">
         <v>52</v>
       </c>
@@ -3508,7 +3511,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:12">
       <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
@@ -3543,7 +3546,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" ht="13.9" thickBot="1">
       <c r="A76" s="117" t="s">
         <v>54</v>
       </c>
@@ -3583,14 +3586,14 @@
         <v>164</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:12" ht="13.9" thickTop="1"/>
+    <row r="79" spans="1:12" ht="17.649999999999999">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="81" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:12" ht="13.9" thickBot="1"/>
+    <row r="81" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
@@ -3601,7 +3604,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" ht="13.9" thickTop="1">
       <c r="A82" s="4" t="s">
         <v>124</v>
       </c>
@@ -3612,7 +3615,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3">
       <c r="A83" s="15" t="s">
         <v>125</v>
       </c>
@@ -3623,7 +3626,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -3634,7 +3637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" ht="15">
       <c r="A85" s="52" t="s">
         <v>130</v>
       </c>
@@ -3645,7 +3648,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3">
       <c r="A86" s="52" t="s">
         <v>129</v>
       </c>
@@ -3656,7 +3659,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3">
       <c r="A87" s="52" t="s">
         <v>128</v>
       </c>
@@ -3667,7 +3670,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3">
       <c r="A88" s="52" t="s">
         <v>127</v>
       </c>
@@ -3678,7 +3681,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3">
       <c r="A89" s="52" t="s">
         <v>166</v>
       </c>
@@ -3689,7 +3692,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3">
       <c r="A90" s="52" t="s">
         <v>131</v>
       </c>
@@ -3700,7 +3703,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3">
       <c r="A91" s="52" t="s">
         <v>132</v>
       </c>
@@ -3711,7 +3714,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3">
       <c r="A92" s="52" t="s">
         <v>133</v>
       </c>
@@ -3722,7 +3725,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3">
       <c r="A93" s="52" t="s">
         <v>27</v>
       </c>
@@ -3733,7 +3736,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3">
       <c r="A94" s="52" t="s">
         <v>28</v>
       </c>
@@ -3744,7 +3747,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3">
       <c r="A95" s="52" t="s">
         <v>126</v>
       </c>
@@ -3755,7 +3758,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3">
       <c r="A96" s="15" t="s">
         <v>122</v>
       </c>
@@ -3766,7 +3769,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11">
       <c r="A97" s="15" t="s">
         <v>123</v>
       </c>
@@ -3777,18 +3780,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11">
       <c r="A98" s="52" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B98" s="34">
         <v>150</v>
       </c>
       <c r="C98" s="18" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11">
       <c r="A99" s="15" t="s">
         <v>30</v>
       </c>
@@ -3797,7 +3800,7 @@
       </c>
       <c r="C99" s="18"/>
     </row>
-    <row r="100" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" ht="13.9" thickBot="1">
       <c r="A100" s="10" t="s">
         <v>31</v>
       </c>
@@ -3806,14 +3809,14 @@
       </c>
       <c r="C100" s="19"/>
     </row>
-    <row r="101" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" ht="13.9" thickTop="1"/>
+    <row r="103" spans="1:11" ht="17.649999999999999">
       <c r="A103" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="104" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="105" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" ht="13.9" thickBot="1"/>
+    <row r="105" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
       <c r="A105" s="3" t="s">
         <v>0</v>
       </c>
@@ -3844,7 +3847,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="106" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" ht="13.9" thickTop="1">
       <c r="A106" s="7" t="s">
         <v>16</v>
       </c>
@@ -3883,7 +3886,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11">
       <c r="A107" s="7" t="s">
         <v>33</v>
       </c>
@@ -3918,7 +3921,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11">
       <c r="A108" s="38" t="s">
         <v>165</v>
       </c>
@@ -3953,7 +3956,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" ht="13.9" thickBot="1">
       <c r="A109" s="10" t="s">
         <v>34</v>
       </c>
@@ -3988,7 +3991,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="110" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="1:11" ht="13.9" thickTop="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3999,24 +4002,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
-    <col min="2" max="9" width="12.85546875" customWidth="1"/>
+    <col min="1" max="1" width="24.4375" customWidth="1"/>
+    <col min="2" max="9" width="12.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="20.65">
       <c r="A1" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="17.649999999999999">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -4027,7 +4030,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="13.9" thickTop="1">
       <c r="A6" s="37" t="s">
         <v>103</v>
       </c>
@@ -4039,7 +4042,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" s="38" t="s">
         <v>93</v>
       </c>
@@ -4051,7 +4054,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" s="38" t="s">
         <v>94</v>
       </c>
@@ -4063,7 +4066,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" s="38" t="s">
         <v>92</v>
       </c>
@@ -4075,7 +4078,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -4086,7 +4089,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.9" thickBot="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -4098,18 +4101,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="15.4" thickTop="1">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="17.649999999999999">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="18" thickBot="1">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -4120,7 +4123,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="13.9" thickTop="1">
       <c r="A17" s="59" t="s">
         <v>65</v>
       </c>
@@ -4129,7 +4132,7 @@
       </c>
       <c r="C17" s="61"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
@@ -4138,7 +4141,7 @@
       </c>
       <c r="C18" s="64"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
@@ -4147,7 +4150,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3">
       <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
@@ -4156,7 +4159,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3">
       <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
@@ -4165,7 +4168,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3">
       <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
@@ -4174,7 +4177,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3">
       <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
@@ -4183,7 +4186,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3">
       <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
@@ -4192,7 +4195,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3">
       <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
@@ -4201,14 +4204,14 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3">
       <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
       <c r="B26" s="68"/>
       <c r="C26" s="64"/>
     </row>
-    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="13.9" thickBot="1">
       <c r="A27" s="69" t="s">
         <v>82</v>
       </c>
@@ -4217,14 +4220,14 @@
       </c>
       <c r="C27" s="71"/>
     </row>
-    <row r="28" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" ht="13.9" thickTop="1"/>
+    <row r="30" spans="1:3" ht="17.649999999999999">
       <c r="A30" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="32" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -4235,7 +4238,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="13.9" thickTop="1">
       <c r="A33" s="59" t="s">
         <v>84</v>
       </c>
@@ -4247,7 +4250,7 @@
       </c>
       <c r="G33" s="74"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7">
       <c r="A34" s="75" t="s">
         <v>85</v>
       </c>
@@ -4257,7 +4260,7 @@
       </c>
       <c r="G34" s="74"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7">
       <c r="A35" s="75" t="s">
         <v>86</v>
       </c>
@@ -4268,7 +4271,7 @@
       <c r="F35" s="79"/>
       <c r="G35" s="74"/>
     </row>
-    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="15">
       <c r="A36" s="75" t="s">
         <v>87</v>
       </c>
@@ -4281,7 +4284,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7">
       <c r="A37" s="75" t="s">
         <v>88</v>
       </c>
@@ -4290,7 +4293,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7">
       <c r="A38" s="82" t="s">
         <v>96</v>
       </c>
@@ -4301,7 +4304,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7">
       <c r="A39" s="82" t="s">
         <v>95</v>
       </c>
@@ -4310,7 +4313,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7">
       <c r="A40" s="82" t="s">
         <v>97</v>
       </c>
@@ -4319,7 +4322,7 @@
       </c>
       <c r="C40" s="77"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7">
       <c r="A41" s="82" t="s">
         <v>98</v>
       </c>
@@ -4328,7 +4331,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" ht="13.9" thickBot="1">
       <c r="A42" s="84" t="s">
         <v>89</v>
       </c>
@@ -4337,16 +4340,16 @@
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="13.9" thickTop="1">
       <c r="B43" s="74"/>
     </row>
-    <row r="45" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" ht="17.649999999999999">
       <c r="A45" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="47" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" ht="13.9" thickBot="1"/>
+    <row r="47" spans="1:7" ht="14.65" thickTop="1" thickBot="1">
       <c r="A47" s="3" t="s">
         <v>0</v>
       </c>
@@ -4357,7 +4360,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" ht="13.9" thickTop="1">
       <c r="A48" s="82" t="s">
         <v>100</v>
       </c>
@@ -4366,7 +4369,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3">
       <c r="A49" s="75" t="s">
         <v>86</v>
       </c>
@@ -4375,7 +4378,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3">
       <c r="A50" s="82" t="s">
         <v>149</v>
       </c>
@@ -4384,7 +4387,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" ht="13.9" thickBot="1">
       <c r="A51" s="83" t="s">
         <v>101</v>
       </c>
@@ -4393,7 +4396,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="1:3" ht="13.9" thickTop="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Boost Converter Design Params.xlsx
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BABF3E0-2D4E-41C2-BB41-E755756E6BF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09E95DFE-5A27-435F-8E2C-A5ECAD43F8C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -30,15 +30,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="181">
   <si>
     <t>Parameter</t>
   </si>
@@ -545,6 +542,42 @@
   </si>
   <si>
     <t>Cf</t>
+  </si>
+  <si>
+    <t>Evaluating Coupling &amp; Pass Capacitors</t>
+  </si>
+  <si>
+    <t>Calculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1/C3/C4 </t>
+  </si>
+  <si>
+    <t>Placement Reasoning</t>
+  </si>
+  <si>
+    <t>Placement Location</t>
+  </si>
+  <si>
+    <t>Input side to the MOSFET</t>
+  </si>
+  <si>
+    <t>C12</t>
+  </si>
+  <si>
+    <t>UC3843 output//Rop1/op2</t>
+  </si>
+  <si>
+    <t>C10</t>
+  </si>
+  <si>
+    <t>RC/CT Circuit near Rrt</t>
+  </si>
+  <si>
+    <t>C5/C6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extras on output side of MOSFET </t>
   </si>
 </sst>
 </file>
@@ -559,7 +592,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -614,6 +647,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1530,7 +1569,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1667,12 +1706,13 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="61" xfId="2" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Per cent" xfId="3" builtinId="5"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2053,27 +2093,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
-  <dimension ref="A1:N110"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
+  <dimension ref="A1:N119"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.4375" customWidth="1"/>
-    <col min="2" max="11" width="12.875" customWidth="1"/>
-    <col min="12" max="12" width="17.4375" customWidth="1"/>
-    <col min="13" max="13" width="18.875" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="4" max="11" width="12.88671875" customWidth="1"/>
+    <col min="12" max="12" width="17.44140625" customWidth="1"/>
+    <col min="13" max="13" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.65">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.649999999999999">
+    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -2084,7 +2126,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="13.9" thickTop="1">
+    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A6" s="37" t="s">
         <v>36</v>
       </c>
@@ -2095,7 +2137,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="38" t="s">
         <v>37</v>
       </c>
@@ -2106,7 +2148,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="38" t="s">
         <v>38</v>
       </c>
@@ -2117,7 +2159,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="38" t="s">
         <v>56</v>
       </c>
@@ -2128,7 +2170,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="38" t="s">
         <v>57</v>
       </c>
@@ -2139,7 +2181,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.9" thickBot="1">
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -2150,16 +2192,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.4" thickTop="1">
+    <row r="12" spans="1:3" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="17.649999999999999">
+    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -2170,7 +2212,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="13.9" thickTop="1">
+    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A17" s="45" t="s">
         <v>41</v>
       </c>
@@ -2182,7 +2224,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="47" t="s">
         <v>40</v>
       </c>
@@ -2194,7 +2236,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="56" t="s">
         <v>59</v>
       </c>
@@ -2206,7 +2248,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="49" t="s">
         <v>60</v>
       </c>
@@ -2218,7 +2260,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="52" t="s">
         <v>43</v>
       </c>
@@ -2230,7 +2272,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="52" t="s">
         <v>150</v>
       </c>
@@ -2242,7 +2284,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="52" t="s">
         <v>44</v>
       </c>
@@ -2254,7 +2296,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="95" t="s">
         <v>151</v>
       </c>
@@ -2266,7 +2308,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="13.9" thickBot="1">
+    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="87" t="s">
         <v>103</v>
       </c>
@@ -2277,14 +2319,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="13.9" thickTop="1"/>
-    <row r="28" spans="1:3" ht="17.649999999999999">
+    <row r="26" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="30" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="29" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>0</v>
       </c>
@@ -2295,7 +2337,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="13.9" thickTop="1">
+    <row r="31" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -2306,7 +2348,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="97" t="s">
         <v>152</v>
       </c>
@@ -2318,7 +2360,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -2330,7 +2372,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="27" t="s">
         <v>153</v>
       </c>
@@ -2342,7 +2384,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="13.9" thickBot="1">
+    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
@@ -2353,14 +2395,14 @@
         <v>109</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="38" spans="1:11" ht="17.649999999999999">
+    <row r="36" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="40" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
+    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="40" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>0</v>
       </c>
@@ -2395,7 +2437,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="13.9" thickTop="1">
+    <row r="41" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -2430,7 +2472,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="44" t="s">
         <v>39</v>
       </c>
@@ -2465,7 +2507,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -2501,7 +2543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -2541,7 +2583,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="45" spans="1:11">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
@@ -2581,7 +2623,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="46" spans="1:11">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" s="38" t="s">
         <v>46</v>
       </c>
@@ -2621,7 +2663,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="47" spans="1:11">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" s="38" t="s">
         <v>45</v>
       </c>
@@ -2661,7 +2703,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="48" spans="1:11">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
@@ -2691,7 +2733,7 @@
       </c>
       <c r="K48" s="23"/>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="7" t="s">
         <v>48</v>
       </c>
@@ -2731,7 +2773,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" s="7" t="s">
         <v>157</v>
       </c>
@@ -2771,7 +2813,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" s="7" t="s">
         <v>47</v>
       </c>
@@ -2811,7 +2853,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" s="27" t="s">
         <v>49</v>
       </c>
@@ -2851,7 +2893,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="27" t="s">
         <v>51</v>
       </c>
@@ -2891,7 +2933,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="27" t="s">
         <v>50</v>
       </c>
@@ -2931,7 +2973,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55" s="7" t="s">
         <v>52</v>
       </c>
@@ -2966,7 +3008,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
@@ -3010,7 +3052,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="13.9" thickBot="1">
+    <row r="57" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
         <v>54</v>
       </c>
@@ -3050,20 +3092,20 @@
         <v>121</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="13.9" thickTop="1">
+    <row r="58" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B58" s="32"/>
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B59" s="32"/>
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="1:14" ht="17.649999999999999">
+    <row r="60" spans="1:14" ht="18" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="14.25" thickBot="1">
+    <row r="62" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="115" t="s">
         <v>0</v>
       </c>
@@ -3094,7 +3136,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="13.9" thickTop="1">
+    <row r="63" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -3134,7 +3176,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -3164,7 +3206,7 @@
       </c>
       <c r="K64" s="23"/>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A65" s="38" t="s">
         <v>162</v>
       </c>
@@ -3199,7 +3241,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A66" s="38" t="s">
         <v>163</v>
       </c>
@@ -3234,7 +3276,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:12">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
@@ -3259,7 +3301,7 @@
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:12">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A68" s="38" t="s">
         <v>45</v>
       </c>
@@ -3299,7 +3341,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A69" s="7" t="s">
         <v>48</v>
       </c>
@@ -3334,7 +3376,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
@@ -3370,7 +3412,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:12">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A71" s="27" t="s">
         <v>49</v>
       </c>
@@ -3405,7 +3447,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:12">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A72" s="27" t="s">
         <v>51</v>
       </c>
@@ -3440,7 +3482,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
@@ -3476,7 +3518,7 @@
       </c>
       <c r="L73" s="108"/>
     </row>
-    <row r="74" spans="1:12">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A74" s="7" t="s">
         <v>52</v>
       </c>
@@ -3511,7 +3553,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
@@ -3546,7 +3588,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="13.9" thickBot="1">
+    <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A76" s="117" t="s">
         <v>54</v>
       </c>
@@ -3586,14 +3628,14 @@
         <v>164</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="13.9" thickTop="1"/>
-    <row r="79" spans="1:12" ht="17.649999999999999">
+    <row r="77" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="79" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="13.9" thickBot="1"/>
-    <row r="81" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="80" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="81" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
@@ -3604,7 +3646,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="13.9" thickTop="1">
+    <row r="82" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>124</v>
       </c>
@@ -3615,7 +3657,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" s="15" t="s">
         <v>125</v>
       </c>
@@ -3626,7 +3668,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -3637,7 +3679,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15">
+    <row r="85" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="52" t="s">
         <v>130</v>
       </c>
@@ -3648,7 +3690,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" s="52" t="s">
         <v>129</v>
       </c>
@@ -3659,7 +3701,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" s="52" t="s">
         <v>128</v>
       </c>
@@ -3670,7 +3712,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" s="52" t="s">
         <v>127</v>
       </c>
@@ -3681,7 +3723,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="52" t="s">
         <v>166</v>
       </c>
@@ -3692,7 +3734,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" s="52" t="s">
         <v>131</v>
       </c>
@@ -3703,7 +3745,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" s="52" t="s">
         <v>132</v>
       </c>
@@ -3714,7 +3756,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" s="52" t="s">
         <v>133</v>
       </c>
@@ -3725,7 +3767,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="52" t="s">
         <v>27</v>
       </c>
@@ -3736,7 +3778,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" s="52" t="s">
         <v>28</v>
       </c>
@@ -3747,7 +3789,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" s="52" t="s">
         <v>126</v>
       </c>
@@ -3758,7 +3800,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" s="15" t="s">
         <v>122</v>
       </c>
@@ -3769,7 +3811,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97" s="15" t="s">
         <v>123</v>
       </c>
@@ -3780,7 +3822,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="98" spans="1:11">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A98" s="52" t="s">
         <v>168</v>
       </c>
@@ -3791,7 +3833,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="99" spans="1:11">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A99" s="15" t="s">
         <v>30</v>
       </c>
@@ -3800,7 +3842,7 @@
       </c>
       <c r="C99" s="18"/>
     </row>
-    <row r="100" spans="1:11" ht="13.9" thickBot="1">
+    <row r="100" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A100" s="10" t="s">
         <v>31</v>
       </c>
@@ -3809,14 +3851,14 @@
       </c>
       <c r="C100" s="19"/>
     </row>
-    <row r="101" spans="1:11" ht="13.9" thickTop="1"/>
-    <row r="103" spans="1:11" ht="17.649999999999999">
+    <row r="101" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="103" spans="1:11" ht="18" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="104" spans="1:11" ht="13.9" thickBot="1"/>
-    <row r="105" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
+    <row r="104" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="105" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A105" s="3" t="s">
         <v>0</v>
       </c>
@@ -3847,7 +3889,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="106" spans="1:11" ht="13.9" thickTop="1">
+    <row r="106" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A106" s="7" t="s">
         <v>16</v>
       </c>
@@ -3886,7 +3928,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="107" spans="1:11">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" s="7" t="s">
         <v>33</v>
       </c>
@@ -3921,7 +3963,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:11">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108" s="38" t="s">
         <v>165</v>
       </c>
@@ -3956,7 +3998,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="13.9" thickBot="1">
+    <row r="109" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A109" s="10" t="s">
         <v>34</v>
       </c>
@@ -3991,8 +4033,87 @@
         <v>35</v>
       </c>
     </row>
-    <row r="110" spans="1:11" ht="13.9" thickTop="1"/>
+    <row r="110" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="112" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+      <c r="A112" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="114" spans="1:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A114" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C114" s="3"/>
+      <c r="D114" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="E114" s="3"/>
+      <c r="F114" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="G114" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="38" t="s">
+        <v>171</v>
+      </c>
+      <c r="B115" s="120" t="s">
+        <v>174</v>
+      </c>
+      <c r="C115" s="22"/>
+      <c r="D115" s="22"/>
+      <c r="E115" s="22"/>
+      <c r="F115" s="22"/>
+      <c r="G115" s="22"/>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A116" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="B116" t="s">
+        <v>180</v>
+      </c>
+      <c r="C116" s="22"/>
+      <c r="D116" s="22"/>
+      <c r="E116" s="22"/>
+      <c r="F116" s="22"/>
+      <c r="G116" s="22"/>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A117" s="38" t="s">
+        <v>175</v>
+      </c>
+      <c r="B117" s="120" t="s">
+        <v>176</v>
+      </c>
+      <c r="C117" s="22"/>
+      <c r="D117" s="22"/>
+      <c r="E117" s="22"/>
+      <c r="F117" s="22"/>
+      <c r="G117" s="22"/>
+    </row>
+    <row r="118" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A118" s="87" t="s">
+        <v>177</v>
+      </c>
+      <c r="B118" s="102" t="s">
+        <v>178</v>
+      </c>
+      <c r="C118" s="30"/>
+      <c r="D118" s="30"/>
+      <c r="E118" s="30"/>
+      <c r="F118" s="30"/>
+      <c r="G118" s="30"/>
+    </row>
+    <row r="119" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -4002,24 +4123,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.4375" customWidth="1"/>
-    <col min="2" max="9" width="12.875" customWidth="1"/>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
+    <col min="2" max="9" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.65">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.649999999999999">
+    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -4030,7 +4151,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="13.9" thickTop="1">
+    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A6" s="37" t="s">
         <v>103</v>
       </c>
@@ -4042,7 +4163,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="38" t="s">
         <v>93</v>
       </c>
@@ -4054,7 +4175,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="38" t="s">
         <v>94</v>
       </c>
@@ -4066,7 +4187,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="38" t="s">
         <v>92</v>
       </c>
@@ -4078,7 +4199,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -4089,7 +4210,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="13.9" thickBot="1">
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -4101,18 +4222,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.4" thickTop="1">
+    <row r="12" spans="1:3" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="17.649999999999999">
+    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18" thickBot="1">
+    <row r="15" spans="1:3" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="16" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -4123,7 +4244,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="13.9" thickTop="1">
+    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A17" s="59" t="s">
         <v>65</v>
       </c>
@@ -4132,7 +4253,7 @@
       </c>
       <c r="C17" s="61"/>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
@@ -4141,7 +4262,7 @@
       </c>
       <c r="C18" s="64"/>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
@@ -4150,7 +4271,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
@@ -4159,7 +4280,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
@@ -4168,7 +4289,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
@@ -4177,7 +4298,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
@@ -4186,7 +4307,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
@@ -4195,7 +4316,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
@@ -4204,14 +4325,14 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
       <c r="B26" s="68"/>
       <c r="C26" s="64"/>
     </row>
-    <row r="27" spans="1:3" ht="13.9" thickBot="1">
+    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="69" t="s">
         <v>82</v>
       </c>
@@ -4220,14 +4341,14 @@
       </c>
       <c r="C27" s="71"/>
     </row>
-    <row r="28" spans="1:3" ht="13.9" thickTop="1"/>
-    <row r="30" spans="1:3" ht="17.649999999999999">
+    <row r="28" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="13.9" thickBot="1"/>
-    <row r="32" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+    <row r="31" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="32" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -4238,7 +4359,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="13.9" thickTop="1">
+    <row r="33" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A33" s="59" t="s">
         <v>84</v>
       </c>
@@ -4250,7 +4371,7 @@
       </c>
       <c r="G33" s="74"/>
     </row>
-    <row r="34" spans="1:7">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="75" t="s">
         <v>85</v>
       </c>
@@ -4260,7 +4381,7 @@
       </c>
       <c r="G34" s="74"/>
     </row>
-    <row r="35" spans="1:7">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="75" t="s">
         <v>86</v>
       </c>
@@ -4271,7 +4392,7 @@
       <c r="F35" s="79"/>
       <c r="G35" s="74"/>
     </row>
-    <row r="36" spans="1:7" ht="15">
+    <row r="36" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="75" t="s">
         <v>87</v>
       </c>
@@ -4284,7 +4405,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="75" t="s">
         <v>88</v>
       </c>
@@ -4293,7 +4414,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="82" t="s">
         <v>96</v>
       </c>
@@ -4304,7 +4425,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="82" t="s">
         <v>95</v>
       </c>
@@ -4313,7 +4434,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="40" spans="1:7">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="82" t="s">
         <v>97</v>
       </c>
@@ -4322,7 +4443,7 @@
       </c>
       <c r="C40" s="77"/>
     </row>
-    <row r="41" spans="1:7">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="82" t="s">
         <v>98</v>
       </c>
@@ -4331,7 +4452,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="13.9" thickBot="1">
+    <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="84" t="s">
         <v>89</v>
       </c>
@@ -4340,16 +4461,16 @@
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="13.9" thickTop="1">
+    <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="B43" s="74"/>
     </row>
-    <row r="45" spans="1:7" ht="17.649999999999999">
+    <row r="45" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="13.9" thickBot="1"/>
-    <row r="47" spans="1:7" ht="14.65" thickTop="1" thickBot="1">
+    <row r="46" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="47" spans="1:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
         <v>0</v>
       </c>
@@ -4360,7 +4481,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="13.9" thickTop="1">
+    <row r="48" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A48" s="82" t="s">
         <v>100</v>
       </c>
@@ -4369,7 +4490,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="75" t="s">
         <v>86</v>
       </c>
@@ -4378,7 +4499,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="50" spans="1:3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="82" t="s">
         <v>149</v>
       </c>
@@ -4387,7 +4508,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="13.9" thickBot="1">
+    <row r="51" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="83" t="s">
         <v>101</v>
       </c>
@@ -4396,7 +4517,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="13.9" thickTop="1"/>
+    <row r="52" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added relevant capacitor values, and added to Altium
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09E95DFE-5A27-435F-8E2C-A5ECAD43F8C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92E6E483-78DD-45F1-B264-6A9D83423984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="191">
   <si>
     <t>Parameter</t>
   </si>
@@ -547,9 +547,6 @@
     <t>Evaluating Coupling &amp; Pass Capacitors</t>
   </si>
   <si>
-    <t>Calculation</t>
-  </si>
-  <si>
     <t xml:space="preserve">C1/C3/C4 </t>
   </si>
   <si>
@@ -562,9 +559,6 @@
     <t>Input side to the MOSFET</t>
   </si>
   <si>
-    <t>C12</t>
-  </si>
-  <si>
     <t>UC3843 output//Rop1/op2</t>
   </si>
   <si>
@@ -578,6 +572,42 @@
   </si>
   <si>
     <t xml:space="preserve">Extras on output side of MOSFET </t>
+  </si>
+  <si>
+    <t>Calculation//Formulae</t>
+  </si>
+  <si>
+    <t>Vref bypass capacitor</t>
+  </si>
+  <si>
+    <t>= 0.1uF as per datasheet</t>
+  </si>
+  <si>
+    <t>0.1uf//100nF</t>
+  </si>
+  <si>
+    <t>C12/R21</t>
+  </si>
+  <si>
+    <t>Low pass noise filter to MCU_PI sig</t>
+  </si>
+  <si>
+    <t>Smooth input ripple</t>
+  </si>
+  <si>
+    <t>Act as bypass capacitors</t>
+  </si>
+  <si>
+    <t>- To be done</t>
+  </si>
+  <si>
+    <t>fp = 1/2piRC @ 10kHz corner</t>
+  </si>
+  <si>
+    <t>R21 = 37k, C12 = 3.3nF</t>
+  </si>
+  <si>
+    <t>0 - short</t>
   </si>
 </sst>
 </file>
@@ -592,7 +622,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -653,6 +683,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1569,7 +1606,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1707,6 +1744,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -2099,7 +2137,9 @@
     <col min="1" max="1" width="20.44140625" customWidth="1"/>
     <col min="2" max="2" width="13.5546875" customWidth="1"/>
     <col min="3" max="3" width="13.33203125" customWidth="1"/>
-    <col min="4" max="11" width="12.88671875" customWidth="1"/>
+    <col min="4" max="7" width="12.88671875" customWidth="1"/>
+    <col min="8" max="8" width="19.21875" customWidth="1"/>
+    <col min="9" max="11" width="12.88671875" customWidth="1"/>
     <col min="12" max="12" width="17.44140625" customWidth="1"/>
     <col min="13" max="13" width="18.88671875" customWidth="1"/>
   </cols>
@@ -4039,79 +4079,108 @@
         <v>169</v>
       </c>
     </row>
-    <row r="113" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="114" spans="1:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="114" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A114" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C114" s="3"/>
       <c r="D114" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E114" s="3"/>
       <c r="F114" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="G114" s="3"/>
+      <c r="H114" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A115" s="38" t="s">
         <v>170</v>
       </c>
-      <c r="G114" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="38" t="s">
-        <v>171</v>
-      </c>
       <c r="B115" s="120" t="s">
+        <v>173</v>
+      </c>
+      <c r="C115" s="22"/>
+      <c r="D115" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="E115" s="22"/>
+      <c r="F115" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="G115" s="22"/>
+      <c r="H115" s="22" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A116" s="38" t="s">
+        <v>177</v>
+      </c>
+      <c r="B116" t="s">
+        <v>178</v>
+      </c>
+      <c r="C116" s="22"/>
+      <c r="D116" t="s">
+        <v>186</v>
+      </c>
+      <c r="E116" s="22"/>
+      <c r="F116" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="G116" s="22"/>
+      <c r="H116" s="22" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A117" s="38" t="s">
+        <v>183</v>
+      </c>
+      <c r="B117" s="120" t="s">
         <v>174</v>
       </c>
-      <c r="C115" s="22"/>
-      <c r="D115" s="22"/>
-      <c r="E115" s="22"/>
-      <c r="F115" s="22"/>
-      <c r="G115" s="22"/>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A116" s="38" t="s">
-        <v>179</v>
-      </c>
-      <c r="B116" t="s">
+      <c r="C117" s="22"/>
+      <c r="D117" s="121" t="s">
+        <v>184</v>
+      </c>
+      <c r="E117" s="22"/>
+      <c r="F117" s="22" t="s">
+        <v>188</v>
+      </c>
+      <c r="G117" s="22"/>
+      <c r="H117" s="22" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A118" s="87" t="s">
+        <v>175</v>
+      </c>
+      <c r="B118" s="102" t="s">
+        <v>176</v>
+      </c>
+      <c r="C118" s="30"/>
+      <c r="D118" s="30" t="s">
         <v>180</v>
       </c>
-      <c r="C116" s="22"/>
-      <c r="D116" s="22"/>
-      <c r="E116" s="22"/>
-      <c r="F116" s="22"/>
-      <c r="G116" s="22"/>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A117" s="38" t="s">
-        <v>175</v>
-      </c>
-      <c r="B117" s="120" t="s">
-        <v>176</v>
-      </c>
-      <c r="C117" s="22"/>
-      <c r="D117" s="22"/>
-      <c r="E117" s="22"/>
-      <c r="F117" s="22"/>
-      <c r="G117" s="22"/>
-    </row>
-    <row r="118" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A118" s="87" t="s">
-        <v>177</v>
-      </c>
-      <c r="B118" s="102" t="s">
-        <v>178</v>
-      </c>
-      <c r="C118" s="30"/>
-      <c r="D118" s="30"/>
       <c r="E118" s="30"/>
-      <c r="F118" s="30"/>
+      <c r="F118" s="30" t="s">
+        <v>181</v>
+      </c>
       <c r="G118" s="30"/>
-    </row>
-    <row r="119" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="H118" s="30" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
More protection capacitor values changed in boost converter Excel
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92E6E483-78DD-45F1-B264-6A9D83423984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47F0A5C-A65C-49C0-8650-1A625C142098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="196">
   <si>
     <t>Parameter</t>
   </si>
@@ -608,6 +608,21 @@
   </si>
   <si>
     <t>0 - short</t>
+  </si>
+  <si>
+    <t>C15/C16/C17</t>
+  </si>
+  <si>
+    <t>Close by all major elect 'hubs'</t>
+  </si>
+  <si>
+    <t>Respond to local high f noise</t>
+  </si>
+  <si>
+    <t>100nF @ 15.9mOhm per C</t>
+  </si>
+  <si>
+    <t>C = (Idelt)/(delV) = (0.05*10e-6)/0.5. &amp; Xc = 1/(2pifC)</t>
   </si>
 </sst>
 </file>
@@ -2131,14 +2146,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
-  <dimension ref="A1:N119"/>
+  <dimension ref="A1:N120"/>
   <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.44140625" customWidth="1"/>
     <col min="2" max="2" width="13.5546875" customWidth="1"/>
     <col min="3" max="3" width="13.33203125" customWidth="1"/>
     <col min="4" max="7" width="12.88671875" customWidth="1"/>
-    <col min="8" max="8" width="19.21875" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
     <col min="9" max="11" width="12.88671875" customWidth="1"/>
     <col min="12" max="12" width="17.44140625" customWidth="1"/>
     <col min="13" max="13" width="18.88671875" customWidth="1"/>
@@ -4180,7 +4195,27 @@
         <v>182</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="119" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A119" s="87" t="s">
+        <v>191</v>
+      </c>
+      <c r="B119" s="102" t="s">
+        <v>192</v>
+      </c>
+      <c r="C119" s="30"/>
+      <c r="D119" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="E119" s="30"/>
+      <c r="F119" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="G119" s="30"/>
+      <c r="H119" s="30" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated current sense signal processing to use appropriate cutoff frequency. Updated simulation results. Confirmed inductor design meets requirements.
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tytom\Documents\GitHub\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wwei275\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B47F0A5C-A65C-49C0-8650-1A625C142098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CFF7BB6-10F2-4CF5-BF41-862A5BB5013A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="203">
   <si>
     <t>Parameter</t>
   </si>
@@ -292,9 +292,6 @@
     <t>Selected lg</t>
   </si>
   <si>
-    <t>Np</t>
-  </si>
-  <si>
     <t>Bmax</t>
   </si>
   <si>
@@ -328,9 +325,6 @@
     <t>Selected Wire Diameter</t>
   </si>
   <si>
-    <t>Parallel Wires</t>
-  </si>
-  <si>
     <t>Rdc of Inductor</t>
   </si>
   <si>
@@ -442,12 +436,6 @@
     <t>Ohms (1-20)</t>
   </si>
   <si>
-    <t>kOhms (1-21)</t>
-  </si>
-  <si>
-    <t>kOhms (1-22)</t>
-  </si>
-  <si>
     <t>pF (1-23)</t>
   </si>
   <si>
@@ -535,9 +523,6 @@
     <t>Steady State Vout (avg)</t>
   </si>
   <si>
-    <t>Rv</t>
-  </si>
-  <si>
     <t>pF</t>
   </si>
   <si>
@@ -623,6 +608,42 @@
   </si>
   <si>
     <t>C = (Idelt)/(delV) = (0.05*10e-6)/0.5. &amp; Xc = 1/(2pifC)</t>
+  </si>
+  <si>
+    <t>Ohms (1-21)</t>
+  </si>
+  <si>
+    <t>Ohms (1-22)</t>
+  </si>
+  <si>
+    <t>Jmax</t>
+  </si>
+  <si>
+    <t>Parallel Wires (Np)</t>
+  </si>
+  <si>
+    <t>Inductor turns (N)</t>
+  </si>
+  <si>
+    <t>Hysteresis loss (Pv)</t>
+  </si>
+  <si>
+    <t>Total loss (Ploss)</t>
+  </si>
+  <si>
+    <t>Bac</t>
+  </si>
+  <si>
+    <t>mT</t>
+  </si>
+  <si>
+    <t>kW/m^3 (1-7)</t>
+  </si>
+  <si>
+    <t>W (1-8)</t>
+  </si>
+  <si>
+    <t>A/mm^2 (1-9)</t>
   </si>
 </sst>
 </file>
@@ -743,7 +764,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="62">
+  <borders count="65">
     <border>
       <left/>
       <right/>
@@ -1612,6 +1633,39 @@
       <bottom style="double">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -1621,7 +1675,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1698,7 +1752,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="43" xfId="2" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="45" xfId="2" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="46" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1"/>
@@ -1717,7 +1770,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="48" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="51" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="52" xfId="2" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
@@ -1757,9 +1809,17 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="61" xfId="2" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="53" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="62" xfId="2" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
@@ -2146,31 +2206,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
-  <dimension ref="A1:N120"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N119"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.44140625" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
-    <col min="4" max="7" width="12.88671875" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="4" max="7" width="12.85546875" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="11" width="12.88671875" customWidth="1"/>
-    <col min="12" max="12" width="17.44140625" customWidth="1"/>
-    <col min="13" max="13" width="18.88671875" customWidth="1"/>
+    <col min="9" max="11" width="12.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -2181,7 +2241,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="s">
         <v>36</v>
       </c>
@@ -2192,7 +2252,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
         <v>37</v>
       </c>
@@ -2203,7 +2263,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
         <v>38</v>
       </c>
@@ -2214,7 +2274,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
         <v>56</v>
       </c>
@@ -2225,7 +2285,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
         <v>57</v>
       </c>
@@ -2236,7 +2296,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -2247,16 +2307,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="16" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -2267,31 +2327,31 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="91">
+      <c r="B17" s="89">
         <f>1-(B7/B8)</f>
         <v>0.5</v>
       </c>
       <c r="C17" s="46" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="92">
+      <c r="B18" s="90">
         <f>1-(B6/B9)</f>
         <v>0.30000000000000004</v>
       </c>
       <c r="C18" s="48" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="56" t="s">
         <v>59</v>
       </c>
@@ -2300,10 +2360,10 @@
         <v>2</v>
       </c>
       <c r="C19" s="58" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="49" t="s">
         <v>60</v>
       </c>
@@ -2312,34 +2372,34 @@
         <v>0.14285714285714285</v>
       </c>
       <c r="C20" s="51" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="93">
+      <c r="B21" s="91">
         <f>1/3</f>
         <v>0.33333333333333331</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="52" t="s">
-        <v>150</v>
-      </c>
-      <c r="B22" s="94">
+        <v>146</v>
+      </c>
+      <c r="B22" s="92">
         <f>B8^2/B10</f>
         <v>50</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="52" t="s">
         <v>44</v>
       </c>
@@ -2348,12 +2408,12 @@
         <v>37.037037037037045</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="95" t="s">
-        <v>151</v>
+        <v>152</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="93" t="s">
+        <v>147</v>
       </c>
       <c r="B24" s="28">
         <f>B23*1.2</f>
@@ -2363,25 +2423,25 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="87" t="s">
-        <v>103</v>
-      </c>
-      <c r="B25" s="96">
+    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="85" t="s">
+        <v>101</v>
+      </c>
+      <c r="B25" s="94">
         <v>47</v>
       </c>
       <c r="C25" s="19" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="30" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>0</v>
       </c>
@@ -2392,7 +2452,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -2403,11 +2463,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="97" t="s">
-        <v>152</v>
-      </c>
-      <c r="B32" s="98">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="95" t="s">
+        <v>148</v>
+      </c>
+      <c r="B32" s="96">
         <f>B9/B8</f>
         <v>1</v>
       </c>
@@ -2415,7 +2475,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -2424,40 +2484,40 @@
         <v>100</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="27" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B34" s="28">
         <f>B33*1.2</f>
         <v>120</v>
       </c>
-      <c r="C34" s="99" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C34" s="97" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B35" s="96">
+      <c r="B35" s="94">
         <v>560</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="38" spans="1:11" ht="18" x14ac:dyDescent="0.35">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="40" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>0</v>
       </c>
@@ -2492,7 +2552,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -2527,7 +2587,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="44" t="s">
         <v>39</v>
       </c>
@@ -2562,7 +2622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -2598,7 +2658,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -2607,162 +2667,162 @@
         <v>50</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D44" s="24">
         <f>D41^2/D43</f>
         <v>50</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F44" s="24">
         <f>F41^2/F43</f>
         <v>5</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H44" s="24">
         <f>H41^2/H43</f>
         <v>5</v>
       </c>
       <c r="I44" s="22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J44" s="24">
         <f>J41^2/J43</f>
         <v>9.0909090909090917</v>
       </c>
       <c r="K44" s="22" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B45" s="100">
+      <c r="B45" s="98">
         <f>1-(B42/B41)</f>
         <v>0.5</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>111</v>
-      </c>
-      <c r="D45" s="100">
+        <v>109</v>
+      </c>
+      <c r="D45" s="98">
         <f>1-(D42/D41)</f>
         <v>0.30000000000000004</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>111</v>
-      </c>
-      <c r="F45" s="100">
+        <v>109</v>
+      </c>
+      <c r="F45" s="98">
         <f>1-(F42/F41)</f>
         <v>0.5</v>
       </c>
       <c r="G45" s="22" t="s">
-        <v>111</v>
-      </c>
-      <c r="H45" s="100">
+        <v>109</v>
+      </c>
+      <c r="H45" s="98">
         <f>1-(H42/H41)</f>
         <v>0.30000000000000004</v>
       </c>
       <c r="I45" s="22" t="s">
-        <v>111</v>
-      </c>
-      <c r="J45" s="100">
+        <v>109</v>
+      </c>
+      <c r="J45" s="98">
         <f>1-(J42/J41)</f>
         <v>0.4</v>
       </c>
       <c r="K45" s="22" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="B46" s="102">
+      <c r="B46" s="100">
         <f>B43/B42</f>
         <v>0.2</v>
       </c>
-      <c r="C46" s="102" t="s">
-        <v>112</v>
-      </c>
-      <c r="D46" s="102">
+      <c r="C46" s="100" t="s">
+        <v>110</v>
+      </c>
+      <c r="D46" s="100">
         <f>D43/D42</f>
         <v>0.14285714285714285</v>
       </c>
-      <c r="E46" s="102" t="s">
-        <v>112</v>
-      </c>
-      <c r="F46" s="102">
+      <c r="E46" s="100" t="s">
+        <v>110</v>
+      </c>
+      <c r="F46" s="100">
         <f>F43/F42</f>
         <v>2</v>
       </c>
-      <c r="G46" s="102" t="s">
-        <v>112</v>
-      </c>
-      <c r="H46" s="102">
+      <c r="G46" s="100" t="s">
+        <v>110</v>
+      </c>
+      <c r="H46" s="100">
         <f>H43/H42</f>
         <v>1.4285714285714286</v>
       </c>
-      <c r="I46" s="102" t="s">
-        <v>112</v>
-      </c>
-      <c r="J46" s="102">
+      <c r="I46" s="100" t="s">
+        <v>110</v>
+      </c>
+      <c r="J46" s="100">
         <f>J43/J42</f>
         <v>0.91666666666666663</v>
       </c>
       <c r="K46" s="22" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="B47" s="102">
+      <c r="B47" s="100">
         <f>B42*B45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.26595744680851069</v>
       </c>
-      <c r="C47" s="102" t="s">
-        <v>113</v>
-      </c>
-      <c r="D47" s="102">
+      <c r="C47" s="100" t="s">
+        <v>111</v>
+      </c>
+      <c r="D47" s="100">
         <f>D42*D45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.22340425531914904</v>
       </c>
-      <c r="E47" s="102" t="s">
-        <v>113</v>
-      </c>
-      <c r="F47" s="102">
+      <c r="E47" s="100" t="s">
+        <v>111</v>
+      </c>
+      <c r="F47" s="100">
         <f>F42*F45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.26595744680851069</v>
       </c>
-      <c r="G47" s="102" t="s">
-        <v>113</v>
-      </c>
-      <c r="H47" s="102">
+      <c r="G47" s="100" t="s">
+        <v>111</v>
+      </c>
+      <c r="H47" s="100">
         <f>H42*H45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.22340425531914904</v>
       </c>
-      <c r="I47" s="102" t="s">
-        <v>113</v>
-      </c>
-      <c r="J47" s="102">
+      <c r="I47" s="100" t="s">
+        <v>111</v>
+      </c>
+      <c r="J47" s="100">
         <f>J42*J45/($B$25*10^-6*$B$11*10^3)</f>
         <v>0.2553191489361703</v>
       </c>
       <c r="K47" s="22" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B48" s="101" t="str">
+      <c r="B48" s="99" t="str">
         <f>IF(B46&gt;=B47/2,"Yes","No")</f>
         <v>Yes</v>
       </c>
@@ -2788,79 +2848,79 @@
       </c>
       <c r="K48" s="23"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B49" s="102">
+      <c r="B49" s="100">
         <f>B46+(B47/2)</f>
         <v>0.33297872340425538</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="D49" s="102">
+        <v>112</v>
+      </c>
+      <c r="D49" s="100">
         <f>D46+(D47/2)</f>
         <v>0.25455927051671734</v>
       </c>
       <c r="E49" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="F49" s="102">
+        <v>112</v>
+      </c>
+      <c r="F49" s="100">
         <f>F46+(F47/2)</f>
         <v>2.1329787234042552</v>
       </c>
       <c r="G49" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="H49" s="102">
+        <v>112</v>
+      </c>
+      <c r="H49" s="100">
         <f>H46+(H47/2)</f>
         <v>1.540273556231003</v>
       </c>
       <c r="I49" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="J49" s="102">
+        <v>112</v>
+      </c>
+      <c r="J49" s="100">
         <f>J46+(J47/2)</f>
         <v>1.0443262411347518</v>
       </c>
       <c r="K49" s="22" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="B50" s="102">
+        <v>153</v>
+      </c>
+      <c r="B50" s="100">
         <f>B46-(B47/2)</f>
         <v>6.7021276595744667E-2</v>
       </c>
       <c r="C50" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="D50" s="102">
+      <c r="D50" s="100">
         <f>D46-(D47/2)</f>
         <v>3.1155015197568331E-2</v>
       </c>
       <c r="E50" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="F50" s="102">
+      <c r="F50" s="100">
         <f>F46-(F47/2)</f>
         <v>1.8670212765957446</v>
       </c>
       <c r="G50" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="H50" s="102">
+      <c r="H50" s="100">
         <f>H46-(H47/2)</f>
         <v>1.3168693009118542</v>
       </c>
       <c r="I50" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="J50" s="102">
+      <c r="J50" s="100">
         <f>J46-(J47/2)</f>
         <v>0.78900709219858145</v>
       </c>
@@ -2868,167 +2928,167 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B51" s="102">
+      <c r="B51" s="100">
         <f>SQRT(B46^2 + (B47^2/12))</f>
         <v>0.21422989277738178</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="D51" s="102">
+        <v>113</v>
+      </c>
+      <c r="D51" s="100">
         <f>SQRT(D46^2 + (D47^2/12))</f>
         <v>0.15673954523305453</v>
       </c>
       <c r="E51" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="F51" s="102">
+        <v>113</v>
+      </c>
+      <c r="F51" s="100">
         <f>SQRT(F46^2 + (F47^2/12))</f>
         <v>2.0014730692565936</v>
       </c>
       <c r="G51" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="H51" s="102">
+        <v>113</v>
+      </c>
+      <c r="H51" s="100">
         <f>SQRT(H46^2 + (H47^2/12))</f>
         <v>1.4300263802829551</v>
       </c>
       <c r="I51" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="J51" s="102">
+        <v>113</v>
+      </c>
+      <c r="J51" s="100">
         <f>SQRT(J46^2 + (J47^2/12))</f>
         <v>0.91962497796415288</v>
       </c>
       <c r="K51" s="22" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="B52" s="103">
+      <c r="B52" s="101">
         <f>B41/B44</f>
         <v>0.1</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="D52" s="103">
+        <v>114</v>
+      </c>
+      <c r="D52" s="101">
         <f>D41/D44</f>
         <v>0.1</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="F52" s="103">
+        <v>114</v>
+      </c>
+      <c r="F52" s="101">
         <f>F41/F44</f>
         <v>1</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="H52" s="103">
+        <v>114</v>
+      </c>
+      <c r="H52" s="101">
         <f>H41/H44</f>
         <v>1</v>
       </c>
       <c r="I52" s="22" t="s">
-        <v>116</v>
-      </c>
-      <c r="J52" s="103">
+        <v>114</v>
+      </c>
+      <c r="J52" s="101">
         <f>J41/J44</f>
         <v>0.54999999999999993</v>
       </c>
       <c r="K52" s="22" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="B53" s="103">
+      <c r="B53" s="101">
         <f>B51*SQRT(B45)</f>
         <v>0.15148340991575365</v>
       </c>
       <c r="C53" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="D53" s="103">
+        <v>115</v>
+      </c>
+      <c r="D53" s="101">
         <f>D51*SQRT(D45)</f>
         <v>8.5849784577245306E-2</v>
       </c>
       <c r="E53" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="F53" s="103">
+        <v>115</v>
+      </c>
+      <c r="F53" s="101">
         <f>F51*SQRT(F45)</f>
         <v>1.4152551796335899</v>
       </c>
       <c r="G53" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="H53" s="103">
+        <v>115</v>
+      </c>
+      <c r="H53" s="101">
         <f>H51*SQRT(H45)</f>
         <v>0.7832577063084355</v>
       </c>
       <c r="I53" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="J53" s="103">
+        <v>115</v>
+      </c>
+      <c r="J53" s="101">
         <f>J51*SQRT(J45)</f>
         <v>0.58162190470977582</v>
       </c>
       <c r="K53" s="22" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="B54" s="103">
+      <c r="B54" s="101">
         <f>SQRT(B46^2*B45*(1-B45) + (B47^2/12)*(1-B45))</f>
         <v>0.11378586678363989</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>118</v>
-      </c>
-      <c r="D54" s="103">
+        <v>116</v>
+      </c>
+      <c r="D54" s="101">
         <f t="shared" ref="D54:J54" si="0">SQRT(D46^2*D45*(1-D45) + (D47^2/12)*(1-D45))</f>
         <v>8.4835720825047062E-2</v>
       </c>
       <c r="E54" s="22" t="s">
-        <v>118</v>
-      </c>
-      <c r="F54" s="103">
+        <v>116</v>
+      </c>
+      <c r="F54" s="101">
         <f t="shared" si="0"/>
         <v>1.0014725275711283</v>
       </c>
       <c r="G54" s="22" t="s">
-        <v>118</v>
-      </c>
-      <c r="H54" s="103">
+        <v>116</v>
+      </c>
+      <c r="H54" s="101">
         <f t="shared" si="0"/>
         <v>0.65687351431886776</v>
       </c>
       <c r="I54" s="22" t="s">
-        <v>118</v>
-      </c>
-      <c r="J54" s="103">
+        <v>116</v>
+      </c>
+      <c r="J54" s="101">
         <f t="shared" si="0"/>
         <v>0.45268759653578</v>
       </c>
       <c r="K54" s="22" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>52</v>
       </c>
@@ -3036,162 +3096,162 @@
         <v>5</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D55" s="28">
         <v>5</v>
       </c>
       <c r="E55" s="22" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F55" s="28">
         <v>5</v>
       </c>
       <c r="G55" s="22" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H55" s="28">
         <v>5</v>
       </c>
       <c r="I55" s="22" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J55" s="28">
         <v>5</v>
       </c>
       <c r="K55" s="22" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="B56" s="106">
+      <c r="B56" s="104">
         <v>5</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="D56" s="106">
+        <v>118</v>
+      </c>
+      <c r="D56" s="104">
         <v>5</v>
       </c>
       <c r="E56" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="F56" s="106">
+        <v>118</v>
+      </c>
+      <c r="F56" s="104">
         <v>5</v>
       </c>
       <c r="G56" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="H56" s="106">
+        <v>118</v>
+      </c>
+      <c r="H56" s="104">
         <v>5</v>
       </c>
       <c r="I56" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="J56" s="106">
+        <v>118</v>
+      </c>
+      <c r="J56" s="104">
         <v>5</v>
       </c>
       <c r="K56" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="L56" s="105" t="s">
-        <v>158</v>
+        <v>118</v>
+      </c>
+      <c r="L56" s="103" t="s">
+        <v>154</v>
       </c>
       <c r="M56" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="N56" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="57" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B57" s="104">
+      <c r="B57" s="102">
         <f>10^3*B52*B45/($B$35*10^-6*$B$11*10^3)</f>
         <v>0.89285714285714302</v>
       </c>
       <c r="C57" s="30" t="s">
-        <v>121</v>
-      </c>
-      <c r="D57" s="104">
+        <v>119</v>
+      </c>
+      <c r="D57" s="102">
         <f>10^3*D52*D45/($B$35*10^-6*$B$11*10^3)</f>
         <v>0.53571428571428581</v>
       </c>
       <c r="E57" s="30" t="s">
-        <v>121</v>
-      </c>
-      <c r="F57" s="104">
+        <v>119</v>
+      </c>
+      <c r="F57" s="102">
         <f>10^3*F52*F45/($B$35*10^-6*$B$11*10^3)</f>
         <v>8.9285714285714288</v>
       </c>
       <c r="G57" s="30" t="s">
-        <v>121</v>
-      </c>
-      <c r="H57" s="104">
+        <v>119</v>
+      </c>
+      <c r="H57" s="102">
         <f>10^3*H52*H45/($B$35*10^-6*$B$11*10^3)</f>
         <v>5.3571428571428585</v>
       </c>
       <c r="I57" s="30" t="s">
-        <v>121</v>
-      </c>
-      <c r="J57" s="104">
+        <v>119</v>
+      </c>
+      <c r="J57" s="102">
         <f>10^3*J52*J45/($B$35*10^-6*$B$11*10^3)</f>
         <v>3.9285714285714284</v>
       </c>
       <c r="K57" s="30" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="58" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B58" s="32"/>
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B59" s="32"/>
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="1:14" ht="18" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="115" t="s">
+    <row r="62" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="113" t="s">
         <v>0</v>
       </c>
-      <c r="B62" s="115" t="s">
+      <c r="B62" s="113" t="s">
         <v>1</v>
       </c>
-      <c r="C62" s="115" t="s">
+      <c r="C62" s="113" t="s">
         <v>7</v>
       </c>
-      <c r="D62" s="115" t="s">
+      <c r="D62" s="113" t="s">
         <v>1</v>
       </c>
-      <c r="E62" s="115" t="s">
+      <c r="E62" s="113" t="s">
         <v>7</v>
       </c>
-      <c r="F62" s="115"/>
-      <c r="G62" s="115"/>
-      <c r="H62" s="115" t="s">
+      <c r="F62" s="113"/>
+      <c r="G62" s="113"/>
+      <c r="H62" s="113" t="s">
         <v>1</v>
       </c>
-      <c r="I62" s="115" t="s">
+      <c r="I62" s="113" t="s">
         <v>7</v>
       </c>
-      <c r="J62" s="115" t="s">
+      <c r="J62" s="113" t="s">
         <v>1</v>
       </c>
-      <c r="K62" s="115" t="s">
+      <c r="K62" s="113" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -3231,7 +3291,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -3261,134 +3321,134 @@
       </c>
       <c r="K64" s="23"/>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="38" t="s">
-        <v>162</v>
-      </c>
-      <c r="B65" s="102">
+        <v>158</v>
+      </c>
+      <c r="B65" s="100">
         <v>4.9983700000000004</v>
       </c>
       <c r="C65" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D65" s="102">
+      <c r="D65" s="100">
         <v>4.9908000000000001</v>
       </c>
       <c r="E65" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="F65" s="107">
+      <c r="F65" s="105">
         <v>4.9982800000000003</v>
       </c>
       <c r="G65" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="H65" s="102">
+      <c r="H65" s="100">
         <v>4.9980099999999998</v>
       </c>
       <c r="I65" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="J65" s="102">
+      <c r="J65" s="100">
         <v>4.9981</v>
       </c>
       <c r="K65" s="23" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="38" t="s">
-        <v>163</v>
-      </c>
-      <c r="B66" s="102">
+        <v>159</v>
+      </c>
+      <c r="B66" s="100">
         <v>0.49967400000000001</v>
       </c>
       <c r="C66" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="D66" s="102">
+      <c r="D66" s="100">
         <v>0.49961699999999998</v>
       </c>
       <c r="E66" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="F66" s="102">
+      <c r="F66" s="100">
         <v>4.9968300000000001</v>
       </c>
       <c r="G66" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="H66" s="102">
+      <c r="H66" s="100">
         <v>4.9961099999999998</v>
       </c>
       <c r="I66" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="J66" s="102">
+      <c r="J66" s="100">
         <v>2.7482099999999998</v>
       </c>
       <c r="K66" s="23" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B67" s="26" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C67" s="22"/>
-      <c r="D67" s="107" t="s">
-        <v>161</v>
+      <c r="D67" s="105" t="s">
+        <v>157</v>
       </c>
       <c r="E67" s="22"/>
-      <c r="F67" s="107" t="s">
-        <v>161</v>
+      <c r="F67" s="105" t="s">
+        <v>157</v>
       </c>
       <c r="G67" s="22"/>
-      <c r="H67" s="107" t="s">
-        <v>161</v>
+      <c r="H67" s="105" t="s">
+        <v>157</v>
       </c>
       <c r="I67" s="22"/>
-      <c r="J67" s="107" t="s">
-        <v>161</v>
+      <c r="J67" s="105" t="s">
+        <v>157</v>
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="B68" s="107">
+      <c r="B68" s="105">
         <f>0.332881-0.0669235</f>
         <v>0.26595749999999996</v>
       </c>
       <c r="C68" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D68" s="107">
+      <c r="D68" s="105">
         <f>0.254488-0.0310839</f>
         <v>0.22340409999999999</v>
       </c>
       <c r="E68" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F68" s="102">
+      <c r="F68" s="100">
         <f>2.13197-1.86601</f>
         <v>0.26595999999999997</v>
       </c>
       <c r="G68" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H68" s="107">
+      <c r="H68" s="105">
         <f>1.53955-1.31615</f>
         <v>0.22340000000000004</v>
       </c>
       <c r="I68" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="J68" s="107">
+      <c r="J68" s="105">
         <f>1.04393-0.788614</f>
         <v>0.25531599999999999</v>
       </c>
@@ -3396,301 +3456,297 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B69" s="102">
+      <c r="B69" s="100">
         <v>0.33288099999999998</v>
       </c>
       <c r="C69" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D69" s="102">
+      <c r="D69" s="100">
         <v>0.25448799999999999</v>
       </c>
       <c r="E69" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F69" s="102">
+      <c r="F69" s="100">
         <v>2.1319699999999999</v>
       </c>
       <c r="G69" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H69" s="102">
+      <c r="H69" s="100">
         <v>1.53955</v>
       </c>
       <c r="I69" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="J69" s="102">
+      <c r="J69" s="100">
         <v>1.04393</v>
       </c>
       <c r="K69" s="22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B70" s="102">
+      <c r="B70" s="100">
         <v>0.214139</v>
       </c>
       <c r="C70" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D70" s="102">
+      <c r="D70" s="100">
         <v>0.15667500000000001</v>
       </c>
       <c r="E70" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F70" s="102">
+      <c r="F70" s="100">
         <v>2.0004599999999999</v>
       </c>
       <c r="G70" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H70" s="102">
+      <c r="H70" s="100">
         <f>1.42931</f>
         <v>1.4293100000000001</v>
       </c>
       <c r="I70" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="J70" s="102">
+      <c r="J70" s="100">
         <v>0.91923299999999997</v>
       </c>
       <c r="K70" s="22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="B71" s="116">
+      <c r="B71" s="114">
         <v>9.9967399999999998E-2</v>
       </c>
       <c r="C71" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D71" s="103">
+      <c r="D71" s="101">
         <v>9.9942699999999995E-2</v>
       </c>
       <c r="E71" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F71" s="102">
+      <c r="F71" s="100">
         <v>0.99965599999999999</v>
       </c>
       <c r="G71" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H71" s="103">
+      <c r="H71" s="101">
         <v>0.99960099999999996</v>
       </c>
       <c r="I71" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="J71" s="103">
+      <c r="J71" s="101">
         <v>0.54984599999999995</v>
       </c>
       <c r="K71" s="22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="B72" s="103">
+      <c r="B72" s="101">
         <v>0.151419</v>
       </c>
       <c r="C72" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D72" s="103">
+      <c r="D72" s="101">
         <v>8.5814299999999996E-2</v>
       </c>
       <c r="E72" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F72" s="116">
+      <c r="F72" s="114">
         <v>1.4145399999999999</v>
       </c>
       <c r="G72" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H72" s="103">
+      <c r="H72" s="101">
         <v>0.78286299999999998</v>
       </c>
       <c r="I72" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="J72" s="103">
+      <c r="J72" s="101">
         <v>0.58137399999999995</v>
       </c>
       <c r="K72" s="22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="B73" s="103">
+      <c r="B73" s="101">
         <v>0.113757</v>
       </c>
       <c r="C73" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D73" s="103">
+      <c r="D73" s="101">
         <v>8.4824099999999999E-2</v>
       </c>
       <c r="E73" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F73" s="103">
+      <c r="F73" s="101">
         <v>1.0011399999999999</v>
       </c>
       <c r="G73" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H73" s="103">
+      <c r="H73" s="101">
         <v>0.65672399999999997</v>
       </c>
       <c r="I73" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="J73" s="103">
+      <c r="J73" s="101">
         <v>0.452598</v>
       </c>
       <c r="K73" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="L73" s="108"/>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L73" s="106"/>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B74" s="103">
+      <c r="B74" s="101">
         <v>5.00204</v>
       </c>
       <c r="C74" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D74" s="103">
+      <c r="D74" s="101">
         <v>5.0002899999999997</v>
       </c>
       <c r="E74" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="F74" s="103">
+      <c r="F74" s="101">
         <v>5.0350299999999999</v>
       </c>
       <c r="G74" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="H74" s="103">
+      <c r="H74" s="101">
         <v>5.02006</v>
       </c>
       <c r="I74" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="J74" s="103">
+      <c r="J74" s="101">
         <v>5.0142699999999998</v>
       </c>
       <c r="K74" s="22" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="B75" s="103">
+      <c r="B75" s="101">
         <v>5.00204</v>
       </c>
       <c r="C75" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="D75" s="103">
+      <c r="D75" s="101">
         <v>5.0002899999999997</v>
       </c>
       <c r="E75" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="F75" s="103">
+      <c r="F75" s="101">
         <v>5.0350299999999999</v>
       </c>
       <c r="G75" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="H75" s="103">
+      <c r="H75" s="101">
         <v>5.02006</v>
       </c>
       <c r="I75" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="J75" s="103">
+      <c r="J75" s="101">
         <v>5.0142699999999998</v>
       </c>
       <c r="K75" s="29" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="117" t="s">
+    <row r="76" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="115" t="s">
         <v>54</v>
       </c>
-      <c r="B76" s="118">
-        <f>(5.00204-4.99469)*10^3</f>
-        <v>7.3499999999997456</v>
-      </c>
-      <c r="C76" s="114" t="s">
-        <v>164</v>
-      </c>
-      <c r="D76" s="118">
-        <f>(5.00029 - 4.99588)*10^3</f>
-        <v>4.410000000000025</v>
-      </c>
-      <c r="E76" s="114" t="s">
-        <v>164</v>
-      </c>
-      <c r="F76" s="118">
-        <f>(5.03503-4.96153)*10^3</f>
-        <v>73.500000000000114</v>
-      </c>
-      <c r="G76" s="114" t="s">
-        <v>164</v>
-      </c>
-      <c r="H76" s="118">
-        <f>(5.02006-4.97596)*10^3</f>
-        <v>44.10000000000025</v>
-      </c>
-      <c r="I76" s="114" t="s">
-        <v>164</v>
-      </c>
-      <c r="J76" s="118">
+      <c r="B76" s="116">
+        <v>0.9</v>
+      </c>
+      <c r="C76" s="112" t="s">
+        <v>160</v>
+      </c>
+      <c r="D76" s="116">
+        <v>0.66</v>
+      </c>
+      <c r="E76" s="112" t="s">
+        <v>160</v>
+      </c>
+      <c r="F76" s="116">
+        <v>8.2100000000000009</v>
+      </c>
+      <c r="G76" s="112" t="s">
+        <v>160</v>
+      </c>
+      <c r="H76" s="116">
+        <v>5.22</v>
+      </c>
+      <c r="I76" s="112" t="s">
+        <v>160</v>
+      </c>
+      <c r="J76" s="116">
         <f>(5.01427-4.98192)*10^3</f>
         <v>32.350000000000101</v>
       </c>
-      <c r="K76" s="114" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="79" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+      <c r="K76" s="112" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="81" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="81" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
@@ -3701,9 +3757,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B82" s="5">
         <v>1</v>
@@ -3712,9 +3768,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="15" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B83" s="34">
         <v>4</v>
@@ -3723,7 +3779,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -3734,9 +3790,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="52" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B85" s="36">
         <v>22</v>
@@ -3745,9 +3801,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="52" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B86" s="34">
         <v>1</v>
@@ -3756,9 +3812,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="52" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B87" s="16">
         <v>18</v>
@@ -3767,455 +3823,444 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="52" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B88" s="16">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="C88" s="18" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="52" t="s">
-        <v>166</v>
-      </c>
-      <c r="B89" s="119">
-        <v>4.7E-2</v>
+        <v>129</v>
+      </c>
+      <c r="B89" s="16">
+        <v>39</v>
       </c>
       <c r="C89" s="18" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="B90" s="16">
+        <v>140</v>
+      </c>
+      <c r="C90" s="18" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" s="52" t="s">
         <v>131</v>
-      </c>
-      <c r="B90" s="16">
-        <v>47</v>
-      </c>
-      <c r="C90" s="18" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A91" s="52" t="s">
-        <v>132</v>
       </c>
       <c r="B91" s="16">
         <v>100</v>
       </c>
       <c r="C91" s="18" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="52" t="s">
-        <v>133</v>
+        <v>27</v>
       </c>
       <c r="B92" s="16">
-        <v>1500</v>
+        <v>100</v>
       </c>
       <c r="C92" s="18" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="52" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B93" s="16">
         <v>100</v>
       </c>
       <c r="C93" s="18" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="52" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
       <c r="B94" s="16">
-        <v>100</v>
+        <v>3300</v>
       </c>
       <c r="C94" s="18" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A95" s="52" t="s">
-        <v>126</v>
-      </c>
-      <c r="B95" s="16">
-        <v>3300</v>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="B95" s="34">
+        <v>4.7</v>
       </c>
       <c r="C95" s="18" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B96" s="34">
-        <v>4.7</v>
+        <v>10</v>
       </c>
       <c r="C96" s="18" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A97" s="15" t="s">
-        <v>123</v>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A97" s="52" t="s">
+        <v>163</v>
       </c>
       <c r="B97" s="34">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="C97" s="18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A98" s="52" t="s">
-        <v>168</v>
-      </c>
-      <c r="B98" s="34">
-        <v>150</v>
-      </c>
-      <c r="C98" s="18" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A99" s="15" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A98" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B99" s="110">
-        <v>5</v>
-      </c>
-      <c r="C99" s="18"/>
-    </row>
-    <row r="100" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A100" s="10" t="s">
+      <c r="B98" s="108">
+        <v>1</v>
+      </c>
+      <c r="C98" s="18"/>
+    </row>
+    <row r="99" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B100" s="111">
-        <v>1000</v>
-      </c>
-      <c r="C100" s="19"/>
-    </row>
-    <row r="101" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="103" spans="1:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="A103" s="2" t="s">
+      <c r="B99" s="109">
+        <v>300</v>
+      </c>
+      <c r="C99" s="19"/>
+    </row>
+    <row r="100" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A102" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="104" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="105" spans="1:11" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A105" s="3" t="s">
+    <row r="103" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="104" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B105" s="3" t="s">
+      <c r="B104" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C105" s="3" t="s">
+      <c r="C104" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D105" s="3" t="s">
+      <c r="D104" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E105" s="3" t="s">
+      <c r="E104" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F105" s="3"/>
-      <c r="G105" s="3"/>
-      <c r="H105" s="3" t="s">
+      <c r="F104" s="3"/>
+      <c r="G104" s="3"/>
+      <c r="H104" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="I105" s="3" t="s">
+      <c r="I104" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J105" s="3" t="s">
+      <c r="J104" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="K105" s="3" t="s">
+      <c r="K104" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="106" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A106" s="7" t="s">
+    <row r="105" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B106" s="8">
+      <c r="B105" s="8">
         <f>B44</f>
         <v>50</v>
       </c>
-      <c r="C106" s="22" t="s">
+      <c r="C105" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="D106" s="8">
+      <c r="D105" s="8">
         <f>D44</f>
         <v>50</v>
       </c>
-      <c r="E106" s="22" t="s">
+      <c r="E105" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="F106" s="8">
+      <c r="F105" s="8">
         <f>F44</f>
         <v>5</v>
       </c>
-      <c r="G106" s="22" t="s">
+      <c r="G105" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="H106" s="8">
+      <c r="H105" s="8">
         <f>H44</f>
         <v>5</v>
       </c>
+      <c r="I105" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J105" s="8">
+        <v>10</v>
+      </c>
+      <c r="K105" s="23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A106" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B106" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="C106" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="D106" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="E106" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F106" s="8">
+        <v>2.5</v>
+      </c>
+      <c r="G106" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="H106" s="8">
+        <v>3.5</v>
+      </c>
       <c r="I106" s="22" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="J106" s="8">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="K106" s="23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A107" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B107" s="8">
-        <v>2.5</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A107" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="B107" s="100">
+        <v>5.0006599999999999</v>
       </c>
       <c r="C107" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="D107" s="8">
-        <v>3.5</v>
+      <c r="D107" s="100">
+        <v>4.9999500000000001</v>
       </c>
       <c r="E107" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="F107" s="8">
-        <v>2.5</v>
+      <c r="F107" s="100">
+        <v>4.9983899999999997</v>
       </c>
       <c r="G107" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="H107" s="8">
-        <v>3.5</v>
+      <c r="H107" s="100">
+        <v>4.99932</v>
       </c>
       <c r="I107" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="J107" s="8">
-        <v>3</v>
+      <c r="J107" s="100">
+        <v>4.9985900000000001</v>
       </c>
       <c r="K107" s="23" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A108" s="38" t="s">
+    <row r="108" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B108" s="107">
+        <v>7.3</v>
+      </c>
+      <c r="C108" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="D108" s="107">
+        <v>5.5</v>
+      </c>
+      <c r="E108" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="F108" s="110">
+        <v>8.9</v>
+      </c>
+      <c r="G108" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="H108" s="107">
+        <v>6</v>
+      </c>
+      <c r="I108" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="J108" s="111">
+        <v>4.8</v>
+      </c>
+      <c r="K108" s="31" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A111" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="113" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="C113" s="3"/>
+      <c r="D113" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E113" s="3"/>
+      <c r="F113" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="G113" s="3"/>
+      <c r="H113" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A114" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="B108" s="102">
-        <v>4.9987000000000004</v>
-      </c>
-      <c r="C108" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="D108" s="102">
-        <v>4.9998500000000003</v>
-      </c>
-      <c r="E108" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="F108" s="102">
-        <v>4.9988000000000001</v>
-      </c>
-      <c r="G108" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="H108" s="102">
-        <v>4.9996700000000001</v>
-      </c>
-      <c r="I108" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="J108" s="102">
-        <v>4.9985900000000001</v>
-      </c>
-      <c r="K108" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="109" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A109" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B109" s="109">
-        <v>8.9</v>
-      </c>
-      <c r="C109" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="D109" s="109">
-        <v>7.7</v>
-      </c>
-      <c r="E109" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="F109" s="112">
-        <v>12.2</v>
-      </c>
-      <c r="G109" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H109" s="109">
-        <v>1.2</v>
-      </c>
-      <c r="I109" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="J109" s="113">
-        <v>4.8</v>
-      </c>
-      <c r="K109" s="31" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="110" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="112" spans="1:11" ht="18" x14ac:dyDescent="0.35">
-      <c r="A112" s="2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="113" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="114" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A114" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B114" s="3" t="s">
+      <c r="B114" s="117" t="s">
+        <v>168</v>
+      </c>
+      <c r="C114" s="22"/>
+      <c r="D114" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="E114" s="22"/>
+      <c r="F114" s="22" t="s">
+        <v>182</v>
+      </c>
+      <c r="G114" s="22"/>
+      <c r="H114" s="22" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A115" s="38" t="s">
         <v>172</v>
       </c>
-      <c r="C114" s="3"/>
-      <c r="D114" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="E114" s="3"/>
-      <c r="F114" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="G114" s="3"/>
-      <c r="H114" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="115" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="38" t="s">
-        <v>170</v>
-      </c>
-      <c r="B115" s="120" t="s">
+      <c r="B115" t="s">
         <v>173</v>
       </c>
       <c r="C115" s="22"/>
-      <c r="D115" s="22" t="s">
-        <v>185</v>
+      <c r="D115" t="s">
+        <v>181</v>
       </c>
       <c r="E115" s="22"/>
       <c r="F115" s="22" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="G115" s="22"/>
       <c r="H115" s="22" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" s="38" t="s">
-        <v>177</v>
-      </c>
-      <c r="B116" t="s">
         <v>178</v>
       </c>
+      <c r="B116" s="117" t="s">
+        <v>169</v>
+      </c>
       <c r="C116" s="22"/>
-      <c r="D116" t="s">
-        <v>186</v>
+      <c r="D116" s="118" t="s">
+        <v>179</v>
       </c>
       <c r="E116" s="22"/>
       <c r="F116" s="22" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="G116" s="22"/>
       <c r="H116" s="22" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A117" s="38" t="s">
-        <v>183</v>
-      </c>
-      <c r="B117" s="120" t="s">
-        <v>174</v>
-      </c>
-      <c r="C117" s="22"/>
-      <c r="D117" s="121" t="s">
         <v>184</v>
       </c>
-      <c r="E117" s="22"/>
-      <c r="F117" s="22" t="s">
-        <v>188</v>
-      </c>
-      <c r="G117" s="22"/>
-      <c r="H117" s="22" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="118" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A118" s="87" t="s">
+    </row>
+    <row r="117" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="85" t="s">
+        <v>170</v>
+      </c>
+      <c r="B117" s="100" t="s">
+        <v>171</v>
+      </c>
+      <c r="C117" s="30"/>
+      <c r="D117" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="B118" s="102" t="s">
+      <c r="E117" s="30"/>
+      <c r="F117" s="30" t="s">
         <v>176</v>
+      </c>
+      <c r="G117" s="30"/>
+      <c r="H117" s="30" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="85" t="s">
+        <v>186</v>
+      </c>
+      <c r="B118" s="100" t="s">
+        <v>187</v>
       </c>
       <c r="C118" s="30"/>
       <c r="D118" s="30" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="E118" s="30"/>
       <c r="F118" s="30" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="G118" s="30"/>
       <c r="H118" s="30" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="119" spans="1:8" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A119" s="87" t="s">
-        <v>191</v>
-      </c>
-      <c r="B119" s="102" t="s">
-        <v>192</v>
-      </c>
-      <c r="C119" s="30"/>
-      <c r="D119" s="30" t="s">
-        <v>193</v>
-      </c>
-      <c r="E119" s="30"/>
-      <c r="F119" s="30" t="s">
-        <v>195</v>
-      </c>
-      <c r="G119" s="30"/>
-      <c r="H119" s="30" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="120" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+        <v>189</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4226,25 +4271,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
-  <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G55"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.44140625" customWidth="1"/>
-    <col min="2" max="9" width="12.88671875" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="2" max="9" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -4255,9 +4300,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="37" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B6" s="5">
         <f>SS_Analysis!B25</f>
@@ -4267,43 +4312,43 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B7" s="8">
-        <f>SS_Analysis!H46</f>
-        <v>1.4285714285714286</v>
+        <f>SS_Analysis!F46</f>
+        <v>2</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B8" s="8">
-        <f>SS_Analysis!H49</f>
-        <v>1.540273556231003</v>
+        <f>SS_Analysis!F49</f>
+        <v>2.1329787234042552</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B9" s="8">
-        <f>SS_Analysis!H51</f>
-        <v>1.4300263802829551</v>
+        <f>SS_Analysis!F51</f>
+        <v>2.0014730692565936</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -4314,7 +4359,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -4326,18 +4371,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -4348,7 +4393,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="59" t="s">
         <v>65</v>
       </c>
@@ -4357,7 +4402,7 @@
       </c>
       <c r="C17" s="61"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
@@ -4366,93 +4411,111 @@
       </c>
       <c r="C18" s="64"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
-      <c r="B19" s="65"/>
+      <c r="B19" s="65">
+        <v>31</v>
+      </c>
       <c r="C19" s="64" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
-      <c r="B20" s="65"/>
+      <c r="B20" s="65">
+        <v>47</v>
+      </c>
       <c r="C20" s="64" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
-      <c r="B21" s="65"/>
+      <c r="B21" s="65">
+        <v>1460</v>
+      </c>
       <c r="C21" s="64" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
-      <c r="B22" s="65"/>
+      <c r="B22" s="65">
+        <v>28.1</v>
+      </c>
       <c r="C22" s="64" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
-      <c r="B23" s="65"/>
+      <c r="B23" s="65">
+        <v>40.200000000000003</v>
+      </c>
       <c r="C23" s="64" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
-      <c r="B24" s="66"/>
+      <c r="B24" s="66">
+        <f>1.724*10^-8</f>
+        <v>1.7240000000000001E-8</v>
+      </c>
       <c r="C24" s="64" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
-      <c r="B25" s="66"/>
+      <c r="B25" s="119">
+        <f>4*PI()*10^-7</f>
+        <v>1.2566370614359173E-6</v>
+      </c>
       <c r="C25" s="64" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
-      <c r="B26" s="68"/>
+      <c r="B26" s="121">
+        <v>1510</v>
+      </c>
       <c r="C26" s="64"/>
     </row>
-    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="69" t="s">
+    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="68" t="s">
         <v>82</v>
       </c>
-      <c r="B27" s="70">
+      <c r="B27" s="69">
         <v>0.65</v>
       </c>
-      <c r="C27" s="71"/>
-    </row>
-    <row r="28" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+      <c r="C27" s="70"/>
+    </row>
+    <row r="28" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="32" spans="1:3" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -4463,167 +4526,231 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A33" s="59" t="s">
         <v>84</v>
       </c>
-      <c r="B33" s="72">
+      <c r="B33" s="71">
         <v>0.1</v>
       </c>
-      <c r="C33" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="G33" s="74"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="75" t="s">
+      <c r="C33" s="72" t="s">
+        <v>138</v>
+      </c>
+      <c r="G33" s="73"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="74" t="s">
+        <v>195</v>
+      </c>
+      <c r="B34" s="123">
+        <f>ROUND(SQRT((2*B6*10^-6*B33*10^-3)/(B25*B19*10^-6)),0)</f>
+        <v>16</v>
+      </c>
+      <c r="C34" s="76" t="s">
+        <v>139</v>
+      </c>
+      <c r="G34" s="73"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="74" t="s">
         <v>85</v>
       </c>
-      <c r="B34" s="76"/>
-      <c r="C34" s="77" t="s">
-        <v>143</v>
-      </c>
-      <c r="G34" s="74"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="75" t="s">
+      <c r="B35" s="77">
+        <f>B34*B8*B25/(2*B33*10^-3)</f>
+        <v>0.2144304092067246</v>
+      </c>
+      <c r="C35" s="76" t="s">
+        <v>140</v>
+      </c>
+      <c r="F35" s="78"/>
+      <c r="G35" s="73"/>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="74" t="s">
         <v>86</v>
       </c>
-      <c r="B35" s="78"/>
-      <c r="C35" s="77" t="s">
-        <v>144</v>
-      </c>
-      <c r="F35" s="79"/>
-      <c r="G35" s="74"/>
-    </row>
-    <row r="36" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="75" t="s">
-        <v>87</v>
-      </c>
-      <c r="B36" s="80" t="str">
+      <c r="B36" s="79" t="str">
         <f>IF(B35&lt;=B10,"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="C36" s="77"/>
+      <c r="C36" s="76"/>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="75" t="s">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="74" t="s">
+        <v>87</v>
+      </c>
+      <c r="B37" s="122">
+        <f>10^3*SQRT(B24/(PI()*B25*B11*10^3))</f>
+        <v>0.20897231909955821</v>
+      </c>
+      <c r="C37" s="76" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="81" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" s="80">
+        <v>0.5</v>
+      </c>
+      <c r="C38" s="76" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="81" t="s">
+        <v>94</v>
+      </c>
+      <c r="B39" s="120">
+        <f>PI()*B38^2/4</f>
+        <v>0.19634954084936207</v>
+      </c>
+      <c r="C39" s="76" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="81" t="s">
+        <v>194</v>
+      </c>
+      <c r="B40" s="80">
+        <v>5</v>
+      </c>
+      <c r="C40" s="76"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="81" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41" s="122">
+        <f>10^3*B24*B34*B23*10^-3/(B40*B39*10^-6)</f>
+        <v>11.294926335995074</v>
+      </c>
+      <c r="C41" s="76" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="83" t="s">
         <v>88</v>
       </c>
-      <c r="B37" s="76"/>
-      <c r="C37" s="77" t="s">
+      <c r="B42" s="124">
+        <f>B9^2*B41*10^-3</f>
+        <v>4.5246282688178256E-2</v>
+      </c>
+      <c r="C42" s="84" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="125" t="s">
+        <v>198</v>
+      </c>
+      <c r="B43" s="126">
+        <f>B35*10^3*SS_Analysis!F47/(2*B8)</f>
+        <v>13.368479376977847</v>
+      </c>
+      <c r="C43" s="127" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="125" t="s">
+        <v>196</v>
+      </c>
+      <c r="B44" s="126">
+        <f>1.71*10^-5*B11^1.12*B43^2.29</f>
+        <v>1.1264811121722047</v>
+      </c>
+      <c r="C44" s="127" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="125" t="s">
+        <v>197</v>
+      </c>
+      <c r="B45" s="126">
+        <f>(B44*10^3*B21*10^-9) + B42</f>
+        <v>4.6890945111949675E-2</v>
+      </c>
+      <c r="C45" s="127" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="74" t="s">
+        <v>193</v>
+      </c>
+      <c r="B46" s="77">
+        <f>B9/(B40*B39)</f>
+        <v>2.0386837275999632</v>
+      </c>
+      <c r="C46" s="76" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="50" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="81" t="s">
+        <v>98</v>
+      </c>
+      <c r="B51" s="75"/>
+      <c r="C51" s="76" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="74" t="s">
+        <v>85</v>
+      </c>
+      <c r="B52" s="88"/>
+      <c r="C52" s="64" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="81" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="82" t="s">
-        <v>96</v>
-      </c>
-      <c r="B38" s="81">
-        <v>0.5</v>
-      </c>
-      <c r="C38" s="77" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="82" t="s">
-        <v>95</v>
-      </c>
-      <c r="B39" s="76"/>
-      <c r="C39" s="77" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="82" t="s">
-        <v>97</v>
-      </c>
-      <c r="B40" s="81">
-        <v>5</v>
-      </c>
-      <c r="C40" s="77"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="82" t="s">
-        <v>98</v>
-      </c>
-      <c r="B41" s="76"/>
-      <c r="C41" s="77" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="84" t="s">
-        <v>89</v>
-      </c>
-      <c r="B42" s="85"/>
-      <c r="C42" s="86" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="74"/>
-    </row>
-    <row r="45" spans="1:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="A45" s="2" t="s">
+      <c r="B53" s="88"/>
+      <c r="C53" s="64" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="82" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="47" spans="1:7" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="82" t="s">
+      <c r="B54" s="86"/>
+      <c r="C54" s="87" t="s">
         <v>100</v>
       </c>
-      <c r="B48" s="76"/>
-      <c r="C48" s="77" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="75" t="s">
-        <v>86</v>
-      </c>
-      <c r="B49" s="90"/>
-      <c r="C49" s="64" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="82" t="s">
-        <v>149</v>
-      </c>
-      <c r="B50" s="90"/>
-      <c r="C50" s="64" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="83" t="s">
-        <v>101</v>
-      </c>
-      <c r="B51" s="88"/>
-      <c r="C51" s="89" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    </row>
+    <row r="55" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Calculated additional values on PCB and justifications.
</commit_message>
<xml_diff>
--- a/Excel/Boost Converter Design Params.xlsx
+++ b/Excel/Boost Converter Design Params.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wwei275\Documents\GitHub\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weiwi\OneDrive\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CFF7BB6-10F2-4CF5-BF41-862A5BB5013A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A21EF389-5E2F-4FE6-B20B-22B3D5565A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{0EA872C3-4804-43CB-9F0B-5F94DB7B4351}"/>
   </bookViews>
   <sheets>
     <sheet name="SS_Analysis" sheetId="1" r:id="rId1"/>
@@ -30,12 +30,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="220">
   <si>
     <t>Parameter</t>
   </si>
@@ -644,6 +647,57 @@
   </si>
   <si>
     <t>A/mm^2 (1-9)</t>
+  </si>
+  <si>
+    <t>Total conductor area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R15 and R13 is voltage divider which determines the voltage which the boost converter output must exceed for Vo to be pulled high and </t>
+  </si>
+  <si>
+    <t>10*R13/R16 sets the hysteresis which is set to 0.01V</t>
+  </si>
+  <si>
+    <t>R13 = 1kOhm</t>
+  </si>
+  <si>
+    <t>R15 = 3.3kOhm</t>
+  </si>
+  <si>
+    <t>R16 = 1MOhm</t>
+  </si>
+  <si>
+    <t>R7 limits current through IB/IC.</t>
+  </si>
+  <si>
+    <t>R7 = 200kOhms</t>
+  </si>
+  <si>
+    <t>C13 = 10nF</t>
+  </si>
+  <si>
+    <t>R10 = 15kOhm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C13 and R10 forms a high-pass filter which basically filters out the DC shift of RT/CT. </t>
+  </si>
+  <si>
+    <t>OVP</t>
+  </si>
+  <si>
+    <t>Slope Compensation</t>
+  </si>
+  <si>
+    <t>R11 = 1.5kOhm</t>
+  </si>
+  <si>
+    <t>R10/R11 is a factor that modifies the RT/CT(ac) component to be 20% of the current sense voltage ripple for slope compensation.</t>
+  </si>
+  <si>
+    <t>R23 = 500Ohm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limits current through IC. </t>
   </si>
 </sst>
 </file>
@@ -658,7 +712,7 @@
     <numFmt numFmtId="168" formatCode="0.0000000"/>
     <numFmt numFmtId="169" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -726,6 +780,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1675,7 +1736,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1820,12 +1881,17 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="62" xfId="2" applyBorder="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="2" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
     <cellStyle name="Check Cell" xfId="1" builtinId="23"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Per cent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1851,7 +1917,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>184785</xdr:colOff>
+      <xdr:colOff>189547</xdr:colOff>
       <xdr:row>97</xdr:row>
       <xdr:rowOff>116205</xdr:rowOff>
     </xdr:to>
@@ -2206,31 +2272,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C28CAE-7D6E-414C-9BF7-B54583CFEE9E}">
-  <dimension ref="A1:N119"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:N129"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" customWidth="1"/>
-    <col min="4" max="7" width="12.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.4375" customWidth="1"/>
+    <col min="2" max="2" width="13.5625" customWidth="1"/>
+    <col min="3" max="3" width="13.3125" customWidth="1"/>
+    <col min="4" max="7" width="12.875" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="11" width="12.85546875" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" customWidth="1"/>
-    <col min="13" max="13" width="18.85546875" customWidth="1"/>
+    <col min="9" max="11" width="12.875" customWidth="1"/>
+    <col min="12" max="12" width="17.4375" customWidth="1"/>
+    <col min="13" max="13" width="18.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="20.65">
       <c r="A1" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="17.649999999999999">
       <c r="A3" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -2241,7 +2307,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="13.9" thickTop="1">
       <c r="A6" s="37" t="s">
         <v>36</v>
       </c>
@@ -2252,7 +2318,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" s="38" t="s">
         <v>37</v>
       </c>
@@ -2263,7 +2329,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" s="38" t="s">
         <v>38</v>
       </c>
@@ -2274,7 +2340,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" s="38" t="s">
         <v>56</v>
       </c>
@@ -2285,7 +2351,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" s="38" t="s">
         <v>57</v>
       </c>
@@ -2296,7 +2362,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.9" thickBot="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -2307,16 +2373,16 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="15.4" thickTop="1">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="17.649999999999999">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -2327,7 +2393,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="13.9" thickTop="1">
       <c r="A17" s="45" t="s">
         <v>41</v>
       </c>
@@ -2339,7 +2405,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18" s="47" t="s">
         <v>40</v>
       </c>
@@ -2351,7 +2417,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19" s="56" t="s">
         <v>59</v>
       </c>
@@ -2363,7 +2429,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3">
       <c r="A20" s="49" t="s">
         <v>60</v>
       </c>
@@ -2375,7 +2441,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3">
       <c r="A21" s="52" t="s">
         <v>43</v>
       </c>
@@ -2387,7 +2453,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3">
       <c r="A22" s="52" t="s">
         <v>146</v>
       </c>
@@ -2399,7 +2465,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3">
       <c r="A23" s="52" t="s">
         <v>44</v>
       </c>
@@ -2411,7 +2477,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3">
       <c r="A24" s="93" t="s">
         <v>147</v>
       </c>
@@ -2423,7 +2489,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="13.9" thickBot="1">
       <c r="A25" s="85" t="s">
         <v>101</v>
       </c>
@@ -2434,14 +2500,14 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="13.9" thickTop="1"/>
+    <row r="28" spans="1:3" ht="17.649999999999999">
       <c r="A28" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="30" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A30" s="3" t="s">
         <v>0</v>
       </c>
@@ -2452,7 +2518,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="13.9" thickTop="1">
       <c r="A31" s="4" t="s">
         <v>10</v>
       </c>
@@ -2463,7 +2529,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3">
       <c r="A32" s="95" t="s">
         <v>148</v>
       </c>
@@ -2475,7 +2541,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11">
       <c r="A33" s="15" t="s">
         <v>11</v>
       </c>
@@ -2487,7 +2553,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11">
       <c r="A34" s="27" t="s">
         <v>149</v>
       </c>
@@ -2499,7 +2565,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="13.9" thickBot="1">
       <c r="A35" s="10" t="s">
         <v>12</v>
       </c>
@@ -2510,14 +2576,14 @@
         <v>107</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="13.9" thickTop="1"/>
+    <row r="38" spans="1:11" ht="17.649999999999999">
       <c r="A38" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="40" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="13.9" thickBot="1"/>
+    <row r="40" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
       <c r="A40" s="3" t="s">
         <v>0</v>
       </c>
@@ -2552,7 +2618,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" ht="13.9" thickTop="1">
       <c r="A41" s="4" t="s">
         <v>14</v>
       </c>
@@ -2587,7 +2653,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11">
       <c r="A42" s="44" t="s">
         <v>39</v>
       </c>
@@ -2622,7 +2688,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
@@ -2658,7 +2724,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11">
       <c r="A44" s="7" t="s">
         <v>16</v>
       </c>
@@ -2698,7 +2764,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11">
       <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
@@ -2738,7 +2804,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11">
       <c r="A46" s="38" t="s">
         <v>46</v>
       </c>
@@ -2778,7 +2844,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11">
       <c r="A47" s="38" t="s">
         <v>45</v>
       </c>
@@ -2818,7 +2884,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
@@ -2848,7 +2914,7 @@
       </c>
       <c r="K48" s="23"/>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14">
       <c r="A49" s="7" t="s">
         <v>48</v>
       </c>
@@ -2888,7 +2954,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14">
       <c r="A50" s="7" t="s">
         <v>153</v>
       </c>
@@ -2928,7 +2994,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14">
       <c r="A51" s="7" t="s">
         <v>47</v>
       </c>
@@ -2968,7 +3034,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14">
       <c r="A52" s="27" t="s">
         <v>49</v>
       </c>
@@ -3008,7 +3074,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14">
       <c r="A53" s="27" t="s">
         <v>51</v>
       </c>
@@ -3048,7 +3114,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14">
       <c r="A54" s="27" t="s">
         <v>50</v>
       </c>
@@ -3088,7 +3154,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14">
       <c r="A55" s="7" t="s">
         <v>52</v>
       </c>
@@ -3123,7 +3189,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14">
       <c r="A56" s="27" t="s">
         <v>53</v>
       </c>
@@ -3167,7 +3233,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" ht="13.9" thickBot="1">
       <c r="A57" s="10" t="s">
         <v>54</v>
       </c>
@@ -3207,20 +3273,20 @@
         <v>119</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" ht="13.9" thickTop="1">
       <c r="B58" s="32"/>
       <c r="C58" s="33"/>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14">
       <c r="B59" s="32"/>
       <c r="C59" s="33"/>
     </row>
-    <row r="60" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:14" ht="17.649999999999999">
       <c r="A60" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:14" ht="14.25" thickBot="1">
       <c r="A62" s="113" t="s">
         <v>0</v>
       </c>
@@ -3236,7 +3302,9 @@
       <c r="E62" s="113" t="s">
         <v>7</v>
       </c>
-      <c r="F62" s="113"/>
+      <c r="F62" s="113" t="s">
+        <v>1</v>
+      </c>
       <c r="G62" s="113"/>
       <c r="H62" s="113" t="s">
         <v>1</v>
@@ -3251,7 +3319,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" ht="13.9" thickTop="1">
       <c r="A63" s="7" t="s">
         <v>16</v>
       </c>
@@ -3291,7 +3359,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14">
       <c r="A64" s="7" t="s">
         <v>17</v>
       </c>
@@ -3321,7 +3389,7 @@
       </c>
       <c r="K64" s="23"/>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:12">
       <c r="A65" s="38" t="s">
         <v>158</v>
       </c>
@@ -3356,7 +3424,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:12">
       <c r="A66" s="38" t="s">
         <v>159</v>
       </c>
@@ -3391,7 +3459,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:12">
       <c r="A67" s="7" t="s">
         <v>18</v>
       </c>
@@ -3416,7 +3484,7 @@
       </c>
       <c r="K67" s="23"/>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:12">
       <c r="A68" s="38" t="s">
         <v>45</v>
       </c>
@@ -3456,7 +3524,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:12">
       <c r="A69" s="7" t="s">
         <v>48</v>
       </c>
@@ -3491,7 +3559,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:12">
       <c r="A70" s="7" t="s">
         <v>47</v>
       </c>
@@ -3527,7 +3595,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:12">
       <c r="A71" s="27" t="s">
         <v>49</v>
       </c>
@@ -3562,7 +3630,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:12">
       <c r="A72" s="27" t="s">
         <v>51</v>
       </c>
@@ -3597,7 +3665,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:12">
       <c r="A73" s="27" t="s">
         <v>50</v>
       </c>
@@ -3633,7 +3701,7 @@
       </c>
       <c r="L73" s="106"/>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:12">
       <c r="A74" s="7" t="s">
         <v>52</v>
       </c>
@@ -3668,7 +3736,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:12">
       <c r="A75" s="27" t="s">
         <v>53</v>
       </c>
@@ -3703,7 +3771,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" ht="13.9" thickBot="1">
       <c r="A76" s="115" t="s">
         <v>54</v>
       </c>
@@ -3739,14 +3807,14 @@
         <v>160</v>
       </c>
     </row>
-    <row r="77" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:12" ht="13.9" thickTop="1"/>
+    <row r="79" spans="1:12" ht="17.649999999999999">
       <c r="A79" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="81" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:12" ht="13.9" thickBot="1"/>
+    <row r="81" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A81" s="3" t="s">
         <v>0</v>
       </c>
@@ -3757,7 +3825,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" ht="13.9" thickTop="1">
       <c r="A82" s="4" t="s">
         <v>122</v>
       </c>
@@ -3768,7 +3836,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3">
       <c r="A83" s="15" t="s">
         <v>123</v>
       </c>
@@ -3779,7 +3847,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3">
       <c r="A84" s="15" t="s">
         <v>23</v>
       </c>
@@ -3790,7 +3858,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" ht="15">
       <c r="A85" s="52" t="s">
         <v>128</v>
       </c>
@@ -3801,7 +3869,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3">
       <c r="A86" s="52" t="s">
         <v>127</v>
       </c>
@@ -3812,7 +3880,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3">
       <c r="A87" s="52" t="s">
         <v>126</v>
       </c>
@@ -3823,7 +3891,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3">
       <c r="A88" s="52" t="s">
         <v>125</v>
       </c>
@@ -3834,7 +3902,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3">
       <c r="A89" s="52" t="s">
         <v>129</v>
       </c>
@@ -3845,7 +3913,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3">
       <c r="A90" s="52" t="s">
         <v>130</v>
       </c>
@@ -3856,7 +3924,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3">
       <c r="A91" s="52" t="s">
         <v>131</v>
       </c>
@@ -3867,7 +3935,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3">
       <c r="A92" s="52" t="s">
         <v>27</v>
       </c>
@@ -3878,7 +3946,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3">
       <c r="A93" s="52" t="s">
         <v>28</v>
       </c>
@@ -3889,7 +3957,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3">
       <c r="A94" s="52" t="s">
         <v>124</v>
       </c>
@@ -3900,7 +3968,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3">
       <c r="A95" s="15" t="s">
         <v>120</v>
       </c>
@@ -3911,7 +3979,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3">
       <c r="A96" s="15" t="s">
         <v>121</v>
       </c>
@@ -3922,7 +3990,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11">
       <c r="A97" s="52" t="s">
         <v>163</v>
       </c>
@@ -3933,7 +4001,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11">
       <c r="A98" s="15" t="s">
         <v>30</v>
       </c>
@@ -3942,7 +4010,7 @@
       </c>
       <c r="C98" s="18"/>
     </row>
-    <row r="99" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" ht="13.9" thickBot="1">
       <c r="A99" s="10" t="s">
         <v>31</v>
       </c>
@@ -3951,14 +4019,14 @@
       </c>
       <c r="C99" s="19"/>
     </row>
-    <row r="100" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" ht="13.9" thickTop="1"/>
+    <row r="102" spans="1:11" ht="17.649999999999999">
       <c r="A102" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="103" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="104" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" ht="13.9" thickBot="1"/>
+    <row r="104" spans="1:11" ht="14.65" thickTop="1" thickBot="1">
       <c r="A104" s="3" t="s">
         <v>0</v>
       </c>
@@ -3989,7 +4057,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="105" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" ht="13.9" thickTop="1">
       <c r="A105" s="7" t="s">
         <v>16</v>
       </c>
@@ -4028,7 +4096,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11">
       <c r="A106" s="7" t="s">
         <v>33</v>
       </c>
@@ -4063,7 +4131,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11">
       <c r="A107" s="38" t="s">
         <v>161</v>
       </c>
@@ -4098,7 +4166,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" ht="13.9" thickBot="1">
       <c r="A108" s="10" t="s">
         <v>34</v>
       </c>
@@ -4133,14 +4201,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" ht="13.9" thickTop="1"/>
+    <row r="111" spans="1:11" ht="17.649999999999999">
       <c r="A111" s="2" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="112" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="113" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" ht="13.9" thickBot="1"/>
+    <row r="113" spans="1:8" ht="14.65" thickTop="1" thickBot="1">
       <c r="A113" s="3" t="s">
         <v>0</v>
       </c>
@@ -4160,7 +4228,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:8" ht="13.9" thickTop="1">
       <c r="A114" s="38" t="s">
         <v>165</v>
       </c>
@@ -4180,7 +4248,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:8">
       <c r="A115" s="38" t="s">
         <v>172</v>
       </c>
@@ -4200,7 +4268,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:8">
       <c r="A116" s="38" t="s">
         <v>178</v>
       </c>
@@ -4220,7 +4288,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:8" ht="13.9" thickBot="1">
       <c r="A117" s="85" t="s">
         <v>170</v>
       </c>
@@ -4240,7 +4308,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" ht="14.25" thickTop="1" thickBot="1">
       <c r="A118" s="85" t="s">
         <v>186</v>
       </c>
@@ -4260,7 +4328,75 @@
         <v>189</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="1:8" ht="13.9" thickTop="1"/>
+    <row r="120" spans="1:8" ht="13.9">
+      <c r="A120" s="131" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8">
+      <c r="A121" s="132" t="s">
+        <v>207</v>
+      </c>
+      <c r="B121" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8">
+      <c r="A122" s="132" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8">
+      <c r="A123" s="132" t="s">
+        <v>208</v>
+      </c>
+      <c r="B123" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8">
+      <c r="A124" s="132" t="s">
+        <v>210</v>
+      </c>
+      <c r="B124" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8" ht="13.9">
+      <c r="A125" s="131" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8">
+      <c r="A126" s="132" t="s">
+        <v>211</v>
+      </c>
+      <c r="B126" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8">
+      <c r="A127" s="132" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="128" spans="1:8">
+      <c r="A128" s="132" t="s">
+        <v>216</v>
+      </c>
+      <c r="B128" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" s="132" t="s">
+        <v>218</v>
+      </c>
+      <c r="B129" t="s">
+        <v>219</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4271,25 +4407,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F74A05D-7210-44AC-859D-2846F0884F7B}">
-  <dimension ref="A1:G55"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G56"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
-    <col min="2" max="9" width="12.85546875" customWidth="1"/>
+    <col min="1" max="1" width="24.4375" customWidth="1"/>
+    <col min="2" max="9" width="12.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="20.65">
       <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="17.649999999999999">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="5" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
@@ -4300,7 +4436,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="13.9" thickTop="1">
       <c r="A6" s="37" t="s">
         <v>101</v>
       </c>
@@ -4312,7 +4448,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" s="38" t="s">
         <v>92</v>
       </c>
@@ -4324,7 +4460,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" s="38" t="s">
         <v>93</v>
       </c>
@@ -4336,7 +4472,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" s="38" t="s">
         <v>91</v>
       </c>
@@ -4348,7 +4484,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -4359,7 +4495,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="13.9" thickBot="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -4371,18 +4507,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="15.4" thickTop="1">
       <c r="A12" s="13"/>
     </row>
-    <row r="14" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="17.649999999999999">
       <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="18" thickBot="1">
       <c r="A15" s="2"/>
     </row>
-    <row r="16" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
@@ -4393,7 +4529,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="13.9" thickTop="1">
       <c r="A17" s="59" t="s">
         <v>65</v>
       </c>
@@ -4402,7 +4538,7 @@
       </c>
       <c r="C17" s="61"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3">
       <c r="A18" s="62" t="s">
         <v>67</v>
       </c>
@@ -4411,7 +4547,7 @@
       </c>
       <c r="C18" s="64"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3">
       <c r="A19" s="62" t="s">
         <v>69</v>
       </c>
@@ -4422,7 +4558,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3">
       <c r="A20" s="62" t="s">
         <v>71</v>
       </c>
@@ -4433,7 +4569,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3">
       <c r="A21" s="62" t="s">
         <v>73</v>
       </c>
@@ -4444,7 +4580,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3">
       <c r="A22" s="62" t="s">
         <v>75</v>
       </c>
@@ -4455,7 +4591,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3">
       <c r="A23" s="62" t="s">
         <v>76</v>
       </c>
@@ -4466,7 +4602,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3">
       <c r="A24" s="62" t="s">
         <v>77</v>
       </c>
@@ -4478,7 +4614,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3">
       <c r="A25" s="62" t="s">
         <v>79</v>
       </c>
@@ -4490,16 +4626,15 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3">
       <c r="A26" s="67" t="s">
         <v>81</v>
       </c>
       <c r="B26" s="121">
         <v>1510</v>
       </c>
-      <c r="C26" s="64"/>
-    </row>
-    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:3" ht="13.9" thickBot="1">
       <c r="A27" s="68" t="s">
         <v>82</v>
       </c>
@@ -4508,14 +4643,14 @@
       </c>
       <c r="C27" s="70"/>
     </row>
-    <row r="28" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" ht="13.9" thickTop="1"/>
+    <row r="30" spans="1:3" ht="17.649999999999999">
       <c r="A30" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="32" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
       <c r="A32" s="3" t="s">
         <v>0</v>
       </c>
@@ -4526,7 +4661,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="13.9" thickTop="1">
       <c r="A33" s="59" t="s">
         <v>84</v>
       </c>
@@ -4538,7 +4673,7 @@
       </c>
       <c r="G33" s="73"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7">
       <c r="A34" s="74" t="s">
         <v>195</v>
       </c>
@@ -4551,7 +4686,7 @@
       </c>
       <c r="G34" s="73"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7">
       <c r="A35" s="74" t="s">
         <v>85</v>
       </c>
@@ -4565,7 +4700,7 @@
       <c r="F35" s="78"/>
       <c r="G35" s="73"/>
     </row>
-    <row r="36" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" ht="15">
       <c r="A36" s="74" t="s">
         <v>86</v>
       </c>
@@ -4578,7 +4713,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7">
       <c r="A37" s="74" t="s">
         <v>87</v>
       </c>
@@ -4590,7 +4725,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7">
       <c r="A38" s="81" t="s">
         <v>95</v>
       </c>
@@ -4601,7 +4736,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7">
       <c r="A39" s="81" t="s">
         <v>94</v>
       </c>
@@ -4613,7 +4748,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7">
       <c r="A40" s="81" t="s">
         <v>194</v>
       </c>
@@ -4622,7 +4757,7 @@
       </c>
       <c r="C40" s="76"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7">
       <c r="A41" s="81" t="s">
         <v>96</v>
       </c>
@@ -4634,7 +4769,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" ht="13.9" thickBot="1">
       <c r="A42" s="83" t="s">
         <v>88</v>
       </c>
@@ -4646,7 +4781,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" ht="13.9" thickTop="1">
       <c r="A43" s="125" t="s">
         <v>198</v>
       </c>
@@ -4658,7 +4793,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7">
       <c r="A44" s="125" t="s">
         <v>196</v>
       </c>
@@ -4670,7 +4805,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7">
       <c r="A45" s="125" t="s">
         <v>197</v>
       </c>
@@ -4682,7 +4817,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7">
       <c r="A46" s="74" t="s">
         <v>193</v>
       </c>
@@ -4694,60 +4829,72 @@
         <v>202</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
+    <row r="47" spans="1:7">
+      <c r="A47" s="128" t="s">
+        <v>203</v>
+      </c>
+      <c r="B47" s="129">
+        <f>B34*B40*B39/B27</f>
+        <v>24.166097335306102</v>
+      </c>
+      <c r="C47" s="130" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="17.649999999999999">
+      <c r="A49" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="50" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="3" t="s">
+    <row r="50" spans="1:3" ht="13.9" thickBot="1"/>
+    <row r="51" spans="1:3" ht="14.65" thickTop="1" thickBot="1">
+      <c r="A51" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B50" s="3" t="s">
+      <c r="B51" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C50" s="3" t="s">
+      <c r="C51" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="81" t="s">
+    <row r="52" spans="1:3" ht="13.9" thickTop="1">
+      <c r="A52" s="81" t="s">
         <v>98</v>
       </c>
-      <c r="B51" s="75"/>
-      <c r="C51" s="76" t="s">
+      <c r="B52" s="75"/>
+      <c r="C52" s="76" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="74" t="s">
+    <row r="53" spans="1:3">
+      <c r="A53" s="74" t="s">
         <v>85</v>
-      </c>
-      <c r="B52" s="88"/>
-      <c r="C52" s="64" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="81" t="s">
-        <v>145</v>
       </c>
       <c r="B53" s="88"/>
       <c r="C53" s="64" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="82" t="s">
+    <row r="54" spans="1:3">
+      <c r="A54" s="81" t="s">
+        <v>145</v>
+      </c>
+      <c r="B54" s="88"/>
+      <c r="C54" s="64" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="13.9" thickBot="1">
+      <c r="A55" s="82" t="s">
         <v>99</v>
       </c>
-      <c r="B54" s="86"/>
-      <c r="C54" s="87" t="s">
+      <c r="B55" s="86"/>
+      <c r="C55" s="87" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="1:3" ht="13.9" thickTop="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>